<commit_message>
Adiciona classe LCI / LCA à planilha de acompanhamento
https://claude.ai/code/session_012B6pvzwHHmCv3nAgYhFWdt
</commit_message>
<xml_diff>
--- a/acompanhamento_mensal.xlsx
+++ b/acompanhamento_mensal.xlsx
@@ -100,7 +100,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -169,6 +169,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="002E8B57"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00C0392B"/>
       </patternFill>
     </fill>
@@ -199,7 +204,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -271,6 +276,9 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -423,7 +431,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Acompanhamento Mensal'!B49</f>
+              <f>'Acompanhamento Mensal'!B56</f>
             </strRef>
           </tx>
           <spPr>
@@ -441,12 +449,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Acompanhamento Mensal'!$A$50:$A$61</f>
+              <f>'Acompanhamento Mensal'!$A$57:$A$68</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Acompanhamento Mensal'!$B$50:$B$61</f>
+              <f>'Acompanhamento Mensal'!$B$57:$B$68</f>
             </numRef>
           </val>
         </ser>
@@ -455,7 +463,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Acompanhamento Mensal'!C49</f>
+              <f>'Acompanhamento Mensal'!C56</f>
             </strRef>
           </tx>
           <spPr>
@@ -473,12 +481,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Acompanhamento Mensal'!$A$50:$A$61</f>
+              <f>'Acompanhamento Mensal'!$A$57:$A$68</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Acompanhamento Mensal'!$C$50:$C$61</f>
+              <f>'Acompanhamento Mensal'!$C$57:$C$68</f>
             </numRef>
           </val>
         </ser>
@@ -561,7 +569,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Acompanhamento Mensal'!E49</f>
+              <f>'Acompanhamento Mensal'!E56</f>
             </strRef>
           </tx>
           <spPr>
@@ -571,12 +579,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Acompanhamento Mensal'!$A$50:$A$61</f>
+              <f>'Acompanhamento Mensal'!$A$57:$A$68</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Acompanhamento Mensal'!$E$50:$E$61</f>
+              <f>'Acompanhamento Mensal'!$E$57:$E$68</f>
             </numRef>
           </val>
         </ser>
@@ -620,7 +628,7 @@
     <from>
       <col>7</col>
       <colOff>0</colOff>
-      <row>47</row>
+      <row>54</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="3600000"/>
@@ -642,7 +650,7 @@
     <from>
       <col>7</col>
       <colOff>0</colOff>
-      <row>68</row>
+      <row>75</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="3600000"/>
@@ -952,7 +960,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BJ61"/>
+  <dimension ref="A1:BJ68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1468,23 +1476,23 @@
         </is>
       </c>
       <c r="B8" s="9">
-        <f>IF(SUM(B9,B16,B23,B30,B35,B42)=0,"",SUM(B9,B16,B23,B30,B35,B42))</f>
+        <f>IF(SUM(B9,B16,B23,B30,B35,B42,B49)=0,"",SUM(B9,B16,B23,B30,B35,B42,B49))</f>
         <v/>
       </c>
       <c r="C8" s="9">
-        <f>IF(SUM(C9,C16,C23,C30,C35,C42)=0,"",SUM(C9,C16,C23,C30,C35,C42))</f>
+        <f>IF(SUM(C9,C16,C23,C30,C35,C42,C49)=0,"",SUM(C9,C16,C23,C30,C35,C42,C49))</f>
         <v/>
       </c>
       <c r="D8" s="9">
-        <f>IF(SUM(D9,D16,D23,D30,D35,D42)=0,"",SUM(D9,D16,D23,D30,D35,D42))</f>
+        <f>IF(SUM(D9,D16,D23,D30,D35,D42,D49)=0,"",SUM(D9,D16,D23,D30,D35,D42,D49))</f>
         <v/>
       </c>
       <c r="E8" s="9">
-        <f>IF(SUM(E9,E16,E23,E30,E35,E42)=0,"",SUM(E9,E16,E23,E30,E35,E42))</f>
+        <f>IF(SUM(E9,E16,E23,E30,E35,E42,E49)=0,"",SUM(E9,E16,E23,E30,E35,E42,E49))</f>
         <v/>
       </c>
       <c r="F8" s="9">
-        <f>IF(SUM(F9,F16,F23,F30,F35,F42)=0,"",SUM(F9,F16,F23,F30,F35,F42))</f>
+        <f>IF(SUM(F9,F16,F23,F30,F35,F42,F49)=0,"",SUM(F9,F16,F23,F30,F35,F42,F49))</f>
         <v/>
       </c>
       <c r="G8" s="10">
@@ -1492,19 +1500,19 @@
         <v/>
       </c>
       <c r="H8" s="9">
-        <f>IF(SUM(H9,H16,H23,H30,H35,H42)=0,"",SUM(H9,H16,H23,H30,H35,H42))</f>
+        <f>IF(SUM(H9,H16,H23,H30,H35,H42,H49)=0,"",SUM(H9,H16,H23,H30,H35,H42,H49))</f>
         <v/>
       </c>
       <c r="I8" s="9">
-        <f>IF(SUM(I9,I16,I23,I30,I35,I42)=0,"",SUM(I9,I16,I23,I30,I35,I42))</f>
+        <f>IF(SUM(I9,I16,I23,I30,I35,I42,I49)=0,"",SUM(I9,I16,I23,I30,I35,I42,I49))</f>
         <v/>
       </c>
       <c r="J8" s="9">
-        <f>IF(SUM(J9,J16,J23,J30,J35,J42)=0,"",SUM(J9,J16,J23,J30,J35,J42))</f>
+        <f>IF(SUM(J9,J16,J23,J30,J35,J42,J49)=0,"",SUM(J9,J16,J23,J30,J35,J42,J49))</f>
         <v/>
       </c>
       <c r="K8" s="9">
-        <f>IF(SUM(K9,K16,K23,K30,K35,K42)=0,"",SUM(K9,K16,K23,K30,K35,K42))</f>
+        <f>IF(SUM(K9,K16,K23,K30,K35,K42,K49)=0,"",SUM(K9,K16,K23,K30,K35,K42,K49))</f>
         <v/>
       </c>
       <c r="L8" s="10">
@@ -1512,19 +1520,19 @@
         <v/>
       </c>
       <c r="M8" s="9">
-        <f>IF(SUM(M9,M16,M23,M30,M35,M42)=0,"",SUM(M9,M16,M23,M30,M35,M42))</f>
+        <f>IF(SUM(M9,M16,M23,M30,M35,M42,M49)=0,"",SUM(M9,M16,M23,M30,M35,M42,M49))</f>
         <v/>
       </c>
       <c r="N8" s="9">
-        <f>IF(SUM(N9,N16,N23,N30,N35,N42)=0,"",SUM(N9,N16,N23,N30,N35,N42))</f>
+        <f>IF(SUM(N9,N16,N23,N30,N35,N42,N49)=0,"",SUM(N9,N16,N23,N30,N35,N42,N49))</f>
         <v/>
       </c>
       <c r="O8" s="9">
-        <f>IF(SUM(O9,O16,O23,O30,O35,O42)=0,"",SUM(O9,O16,O23,O30,O35,O42))</f>
+        <f>IF(SUM(O9,O16,O23,O30,O35,O42,O49)=0,"",SUM(O9,O16,O23,O30,O35,O42,O49))</f>
         <v/>
       </c>
       <c r="P8" s="9">
-        <f>IF(SUM(P9,P16,P23,P30,P35,P42)=0,"",SUM(P9,P16,P23,P30,P35,P42))</f>
+        <f>IF(SUM(P9,P16,P23,P30,P35,P42,P49)=0,"",SUM(P9,P16,P23,P30,P35,P42,P49))</f>
         <v/>
       </c>
       <c r="Q8" s="10">
@@ -1532,19 +1540,19 @@
         <v/>
       </c>
       <c r="R8" s="9">
-        <f>IF(SUM(R9,R16,R23,R30,R35,R42)=0,"",SUM(R9,R16,R23,R30,R35,R42))</f>
+        <f>IF(SUM(R9,R16,R23,R30,R35,R42,R49)=0,"",SUM(R9,R16,R23,R30,R35,R42,R49))</f>
         <v/>
       </c>
       <c r="S8" s="9">
-        <f>IF(SUM(S9,S16,S23,S30,S35,S42)=0,"",SUM(S9,S16,S23,S30,S35,S42))</f>
+        <f>IF(SUM(S9,S16,S23,S30,S35,S42,S49)=0,"",SUM(S9,S16,S23,S30,S35,S42,S49))</f>
         <v/>
       </c>
       <c r="T8" s="9">
-        <f>IF(SUM(T9,T16,T23,T30,T35,T42)=0,"",SUM(T9,T16,T23,T30,T35,T42))</f>
+        <f>IF(SUM(T9,T16,T23,T30,T35,T42,T49)=0,"",SUM(T9,T16,T23,T30,T35,T42,T49))</f>
         <v/>
       </c>
       <c r="U8" s="9">
-        <f>IF(SUM(U9,U16,U23,U30,U35,U42)=0,"",SUM(U9,U16,U23,U30,U35,U42))</f>
+        <f>IF(SUM(U9,U16,U23,U30,U35,U42,U49)=0,"",SUM(U9,U16,U23,U30,U35,U42,U49))</f>
         <v/>
       </c>
       <c r="V8" s="10">
@@ -1552,19 +1560,19 @@
         <v/>
       </c>
       <c r="W8" s="9">
-        <f>IF(SUM(W9,W16,W23,W30,W35,W42)=0,"",SUM(W9,W16,W23,W30,W35,W42))</f>
+        <f>IF(SUM(W9,W16,W23,W30,W35,W42,W49)=0,"",SUM(W9,W16,W23,W30,W35,W42,W49))</f>
         <v/>
       </c>
       <c r="X8" s="9">
-        <f>IF(SUM(X9,X16,X23,X30,X35,X42)=0,"",SUM(X9,X16,X23,X30,X35,X42))</f>
+        <f>IF(SUM(X9,X16,X23,X30,X35,X42,X49)=0,"",SUM(X9,X16,X23,X30,X35,X42,X49))</f>
         <v/>
       </c>
       <c r="Y8" s="9">
-        <f>IF(SUM(Y9,Y16,Y23,Y30,Y35,Y42)=0,"",SUM(Y9,Y16,Y23,Y30,Y35,Y42))</f>
+        <f>IF(SUM(Y9,Y16,Y23,Y30,Y35,Y42,Y49)=0,"",SUM(Y9,Y16,Y23,Y30,Y35,Y42,Y49))</f>
         <v/>
       </c>
       <c r="Z8" s="9">
-        <f>IF(SUM(Z9,Z16,Z23,Z30,Z35,Z42)=0,"",SUM(Z9,Z16,Z23,Z30,Z35,Z42))</f>
+        <f>IF(SUM(Z9,Z16,Z23,Z30,Z35,Z42,Z49)=0,"",SUM(Z9,Z16,Z23,Z30,Z35,Z42,Z49))</f>
         <v/>
       </c>
       <c r="AA8" s="10">
@@ -1572,19 +1580,19 @@
         <v/>
       </c>
       <c r="AB8" s="9">
-        <f>IF(SUM(AB9,AB16,AB23,AB30,AB35,AB42)=0,"",SUM(AB9,AB16,AB23,AB30,AB35,AB42))</f>
+        <f>IF(SUM(AB9,AB16,AB23,AB30,AB35,AB42,AB49)=0,"",SUM(AB9,AB16,AB23,AB30,AB35,AB42,AB49))</f>
         <v/>
       </c>
       <c r="AC8" s="9">
-        <f>IF(SUM(AC9,AC16,AC23,AC30,AC35,AC42)=0,"",SUM(AC9,AC16,AC23,AC30,AC35,AC42))</f>
+        <f>IF(SUM(AC9,AC16,AC23,AC30,AC35,AC42,AC49)=0,"",SUM(AC9,AC16,AC23,AC30,AC35,AC42,AC49))</f>
         <v/>
       </c>
       <c r="AD8" s="9">
-        <f>IF(SUM(AD9,AD16,AD23,AD30,AD35,AD42)=0,"",SUM(AD9,AD16,AD23,AD30,AD35,AD42))</f>
+        <f>IF(SUM(AD9,AD16,AD23,AD30,AD35,AD42,AD49)=0,"",SUM(AD9,AD16,AD23,AD30,AD35,AD42,AD49))</f>
         <v/>
       </c>
       <c r="AE8" s="9">
-        <f>IF(SUM(AE9,AE16,AE23,AE30,AE35,AE42)=0,"",SUM(AE9,AE16,AE23,AE30,AE35,AE42))</f>
+        <f>IF(SUM(AE9,AE16,AE23,AE30,AE35,AE42,AE49)=0,"",SUM(AE9,AE16,AE23,AE30,AE35,AE42,AE49))</f>
         <v/>
       </c>
       <c r="AF8" s="10">
@@ -1592,19 +1600,19 @@
         <v/>
       </c>
       <c r="AG8" s="9">
-        <f>IF(SUM(AG9,AG16,AG23,AG30,AG35,AG42)=0,"",SUM(AG9,AG16,AG23,AG30,AG35,AG42))</f>
+        <f>IF(SUM(AG9,AG16,AG23,AG30,AG35,AG42,AG49)=0,"",SUM(AG9,AG16,AG23,AG30,AG35,AG42,AG49))</f>
         <v/>
       </c>
       <c r="AH8" s="9">
-        <f>IF(SUM(AH9,AH16,AH23,AH30,AH35,AH42)=0,"",SUM(AH9,AH16,AH23,AH30,AH35,AH42))</f>
+        <f>IF(SUM(AH9,AH16,AH23,AH30,AH35,AH42,AH49)=0,"",SUM(AH9,AH16,AH23,AH30,AH35,AH42,AH49))</f>
         <v/>
       </c>
       <c r="AI8" s="9">
-        <f>IF(SUM(AI9,AI16,AI23,AI30,AI35,AI42)=0,"",SUM(AI9,AI16,AI23,AI30,AI35,AI42))</f>
+        <f>IF(SUM(AI9,AI16,AI23,AI30,AI35,AI42,AI49)=0,"",SUM(AI9,AI16,AI23,AI30,AI35,AI42,AI49))</f>
         <v/>
       </c>
       <c r="AJ8" s="9">
-        <f>IF(SUM(AJ9,AJ16,AJ23,AJ30,AJ35,AJ42)=0,"",SUM(AJ9,AJ16,AJ23,AJ30,AJ35,AJ42))</f>
+        <f>IF(SUM(AJ9,AJ16,AJ23,AJ30,AJ35,AJ42,AJ49)=0,"",SUM(AJ9,AJ16,AJ23,AJ30,AJ35,AJ42,AJ49))</f>
         <v/>
       </c>
       <c r="AK8" s="10">
@@ -1612,19 +1620,19 @@
         <v/>
       </c>
       <c r="AL8" s="9">
-        <f>IF(SUM(AL9,AL16,AL23,AL30,AL35,AL42)=0,"",SUM(AL9,AL16,AL23,AL30,AL35,AL42))</f>
+        <f>IF(SUM(AL9,AL16,AL23,AL30,AL35,AL42,AL49)=0,"",SUM(AL9,AL16,AL23,AL30,AL35,AL42,AL49))</f>
         <v/>
       </c>
       <c r="AM8" s="9">
-        <f>IF(SUM(AM9,AM16,AM23,AM30,AM35,AM42)=0,"",SUM(AM9,AM16,AM23,AM30,AM35,AM42))</f>
+        <f>IF(SUM(AM9,AM16,AM23,AM30,AM35,AM42,AM49)=0,"",SUM(AM9,AM16,AM23,AM30,AM35,AM42,AM49))</f>
         <v/>
       </c>
       <c r="AN8" s="9">
-        <f>IF(SUM(AN9,AN16,AN23,AN30,AN35,AN42)=0,"",SUM(AN9,AN16,AN23,AN30,AN35,AN42))</f>
+        <f>IF(SUM(AN9,AN16,AN23,AN30,AN35,AN42,AN49)=0,"",SUM(AN9,AN16,AN23,AN30,AN35,AN42,AN49))</f>
         <v/>
       </c>
       <c r="AO8" s="9">
-        <f>IF(SUM(AO9,AO16,AO23,AO30,AO35,AO42)=0,"",SUM(AO9,AO16,AO23,AO30,AO35,AO42))</f>
+        <f>IF(SUM(AO9,AO16,AO23,AO30,AO35,AO42,AO49)=0,"",SUM(AO9,AO16,AO23,AO30,AO35,AO42,AO49))</f>
         <v/>
       </c>
       <c r="AP8" s="10">
@@ -1632,19 +1640,19 @@
         <v/>
       </c>
       <c r="AQ8" s="9">
-        <f>IF(SUM(AQ9,AQ16,AQ23,AQ30,AQ35,AQ42)=0,"",SUM(AQ9,AQ16,AQ23,AQ30,AQ35,AQ42))</f>
+        <f>IF(SUM(AQ9,AQ16,AQ23,AQ30,AQ35,AQ42,AQ49)=0,"",SUM(AQ9,AQ16,AQ23,AQ30,AQ35,AQ42,AQ49))</f>
         <v/>
       </c>
       <c r="AR8" s="9">
-        <f>IF(SUM(AR9,AR16,AR23,AR30,AR35,AR42)=0,"",SUM(AR9,AR16,AR23,AR30,AR35,AR42))</f>
+        <f>IF(SUM(AR9,AR16,AR23,AR30,AR35,AR42,AR49)=0,"",SUM(AR9,AR16,AR23,AR30,AR35,AR42,AR49))</f>
         <v/>
       </c>
       <c r="AS8" s="9">
-        <f>IF(SUM(AS9,AS16,AS23,AS30,AS35,AS42)=0,"",SUM(AS9,AS16,AS23,AS30,AS35,AS42))</f>
+        <f>IF(SUM(AS9,AS16,AS23,AS30,AS35,AS42,AS49)=0,"",SUM(AS9,AS16,AS23,AS30,AS35,AS42,AS49))</f>
         <v/>
       </c>
       <c r="AT8" s="9">
-        <f>IF(SUM(AT9,AT16,AT23,AT30,AT35,AT42)=0,"",SUM(AT9,AT16,AT23,AT30,AT35,AT42))</f>
+        <f>IF(SUM(AT9,AT16,AT23,AT30,AT35,AT42,AT49)=0,"",SUM(AT9,AT16,AT23,AT30,AT35,AT42,AT49))</f>
         <v/>
       </c>
       <c r="AU8" s="10">
@@ -1652,19 +1660,19 @@
         <v/>
       </c>
       <c r="AV8" s="9">
-        <f>IF(SUM(AV9,AV16,AV23,AV30,AV35,AV42)=0,"",SUM(AV9,AV16,AV23,AV30,AV35,AV42))</f>
+        <f>IF(SUM(AV9,AV16,AV23,AV30,AV35,AV42,AV49)=0,"",SUM(AV9,AV16,AV23,AV30,AV35,AV42,AV49))</f>
         <v/>
       </c>
       <c r="AW8" s="9">
-        <f>IF(SUM(AW9,AW16,AW23,AW30,AW35,AW42)=0,"",SUM(AW9,AW16,AW23,AW30,AW35,AW42))</f>
+        <f>IF(SUM(AW9,AW16,AW23,AW30,AW35,AW42,AW49)=0,"",SUM(AW9,AW16,AW23,AW30,AW35,AW42,AW49))</f>
         <v/>
       </c>
       <c r="AX8" s="9">
-        <f>IF(SUM(AX9,AX16,AX23,AX30,AX35,AX42)=0,"",SUM(AX9,AX16,AX23,AX30,AX35,AX42))</f>
+        <f>IF(SUM(AX9,AX16,AX23,AX30,AX35,AX42,AX49)=0,"",SUM(AX9,AX16,AX23,AX30,AX35,AX42,AX49))</f>
         <v/>
       </c>
       <c r="AY8" s="9">
-        <f>IF(SUM(AY9,AY16,AY23,AY30,AY35,AY42)=0,"",SUM(AY9,AY16,AY23,AY30,AY35,AY42))</f>
+        <f>IF(SUM(AY9,AY16,AY23,AY30,AY35,AY42,AY49)=0,"",SUM(AY9,AY16,AY23,AY30,AY35,AY42,AY49))</f>
         <v/>
       </c>
       <c r="AZ8" s="10">
@@ -1672,19 +1680,19 @@
         <v/>
       </c>
       <c r="BA8" s="9">
-        <f>IF(SUM(BA9,BA16,BA23,BA30,BA35,BA42)=0,"",SUM(BA9,BA16,BA23,BA30,BA35,BA42))</f>
+        <f>IF(SUM(BA9,BA16,BA23,BA30,BA35,BA42,BA49)=0,"",SUM(BA9,BA16,BA23,BA30,BA35,BA42,BA49))</f>
         <v/>
       </c>
       <c r="BB8" s="9">
-        <f>IF(SUM(BB9,BB16,BB23,BB30,BB35,BB42)=0,"",SUM(BB9,BB16,BB23,BB30,BB35,BB42))</f>
+        <f>IF(SUM(BB9,BB16,BB23,BB30,BB35,BB42,BB49)=0,"",SUM(BB9,BB16,BB23,BB30,BB35,BB42,BB49))</f>
         <v/>
       </c>
       <c r="BC8" s="9">
-        <f>IF(SUM(BC9,BC16,BC23,BC30,BC35,BC42)=0,"",SUM(BC9,BC16,BC23,BC30,BC35,BC42))</f>
+        <f>IF(SUM(BC9,BC16,BC23,BC30,BC35,BC42,BC49)=0,"",SUM(BC9,BC16,BC23,BC30,BC35,BC42,BC49))</f>
         <v/>
       </c>
       <c r="BD8" s="9">
-        <f>IF(SUM(BD9,BD16,BD23,BD30,BD35,BD42)=0,"",SUM(BD9,BD16,BD23,BD30,BD35,BD42))</f>
+        <f>IF(SUM(BD9,BD16,BD23,BD30,BD35,BD42,BD49)=0,"",SUM(BD9,BD16,BD23,BD30,BD35,BD42,BD49))</f>
         <v/>
       </c>
       <c r="BE8" s="10">
@@ -1692,19 +1700,19 @@
         <v/>
       </c>
       <c r="BF8" s="9">
-        <f>IF(SUM(BF9,BF16,BF23,BF30,BF35,BF42)=0,"",SUM(BF9,BF16,BF23,BF30,BF35,BF42))</f>
+        <f>IF(SUM(BF9,BF16,BF23,BF30,BF35,BF42,BF49)=0,"",SUM(BF9,BF16,BF23,BF30,BF35,BF42,BF49))</f>
         <v/>
       </c>
       <c r="BG8" s="9">
-        <f>IF(SUM(BG9,BG16,BG23,BG30,BG35,BG42)=0,"",SUM(BG9,BG16,BG23,BG30,BG35,BG42))</f>
+        <f>IF(SUM(BG9,BG16,BG23,BG30,BG35,BG42,BG49)=0,"",SUM(BG9,BG16,BG23,BG30,BG35,BG42,BG49))</f>
         <v/>
       </c>
       <c r="BH8" s="9">
-        <f>IF(SUM(BH9,BH16,BH23,BH30,BH35,BH42)=0,"",SUM(BH9,BH16,BH23,BH30,BH35,BH42))</f>
+        <f>IF(SUM(BH9,BH16,BH23,BH30,BH35,BH42,BH49)=0,"",SUM(BH9,BH16,BH23,BH30,BH35,BH42,BH49))</f>
         <v/>
       </c>
       <c r="BI8" s="9">
-        <f>IF(SUM(BI9,BI16,BI23,BI30,BI35,BI42)=0,"",SUM(BI9,BI16,BI23,BI30,BI35,BI42))</f>
+        <f>IF(SUM(BI9,BI16,BI23,BI30,BI35,BI42,BI49)=0,"",SUM(BI9,BI16,BI23,BI30,BI35,BI42,BI49))</f>
         <v/>
       </c>
       <c r="BJ8" s="10">
@@ -6778,27 +6786,27 @@
     <row r="42" ht="21" customHeight="1">
       <c r="A42" s="24" t="inlineStr">
         <is>
-          <t>POUPANÇA</t>
+          <t>LCI / LCA</t>
         </is>
       </c>
       <c r="B42" s="12">
-        <f>IF(SUM(B43,B44,B45)=0,"",SUM(B43,B44,B45))</f>
+        <f>IF(SUM(B43,B44,B45,B46,B47,B48)=0,"",SUM(B43,B44,B45,B46,B47,B48))</f>
         <v/>
       </c>
       <c r="C42" s="12">
-        <f>IF(SUM(C43:C45)=0,"",SUM(C43:C45))</f>
+        <f>IF(SUM(C43:C48)=0,"",SUM(C43:C48))</f>
         <v/>
       </c>
       <c r="D42" s="12">
-        <f>IF(SUM(D43:D45)=0,"",SUM(D43:D45))</f>
+        <f>IF(SUM(D43:D48)=0,"",SUM(D43:D48))</f>
         <v/>
       </c>
       <c r="E42" s="12">
-        <f>SUM(E43:E45)</f>
+        <f>SUM(E43:E48)</f>
         <v/>
       </c>
       <c r="F42" s="12">
-        <f>IF(SUM(F43:F45)=0,"",SUM(F43:F45))</f>
+        <f>IF(SUM(F43:F48)=0,"",SUM(F43:F48))</f>
         <v/>
       </c>
       <c r="G42" s="13">
@@ -6806,19 +6814,19 @@
         <v/>
       </c>
       <c r="H42" s="12">
-        <f>IF(SUM(H43:H45)=0,"",SUM(H43:H45))</f>
+        <f>IF(SUM(H43:H48)=0,"",SUM(H43:H48))</f>
         <v/>
       </c>
       <c r="I42" s="12">
-        <f>IF(SUM(I43:I45)=0,"",SUM(I43:I45))</f>
+        <f>IF(SUM(I43:I48)=0,"",SUM(I43:I48))</f>
         <v/>
       </c>
       <c r="J42" s="12">
-        <f>SUM(J43:J45)</f>
+        <f>SUM(J43:J48)</f>
         <v/>
       </c>
       <c r="K42" s="12">
-        <f>IF(SUM(K43:K45)=0,"",SUM(K43:K45))</f>
+        <f>IF(SUM(K43:K48)=0,"",SUM(K43:K48))</f>
         <v/>
       </c>
       <c r="L42" s="13">
@@ -6826,19 +6834,19 @@
         <v/>
       </c>
       <c r="M42" s="12">
-        <f>IF(SUM(M43:M45)=0,"",SUM(M43:M45))</f>
+        <f>IF(SUM(M43:M48)=0,"",SUM(M43:M48))</f>
         <v/>
       </c>
       <c r="N42" s="12">
-        <f>IF(SUM(N43:N45)=0,"",SUM(N43:N45))</f>
+        <f>IF(SUM(N43:N48)=0,"",SUM(N43:N48))</f>
         <v/>
       </c>
       <c r="O42" s="12">
-        <f>SUM(O43:O45)</f>
+        <f>SUM(O43:O48)</f>
         <v/>
       </c>
       <c r="P42" s="12">
-        <f>IF(SUM(P43:P45)=0,"",SUM(P43:P45))</f>
+        <f>IF(SUM(P43:P48)=0,"",SUM(P43:P48))</f>
         <v/>
       </c>
       <c r="Q42" s="13">
@@ -6846,19 +6854,19 @@
         <v/>
       </c>
       <c r="R42" s="12">
-        <f>IF(SUM(R43:R45)=0,"",SUM(R43:R45))</f>
+        <f>IF(SUM(R43:R48)=0,"",SUM(R43:R48))</f>
         <v/>
       </c>
       <c r="S42" s="12">
-        <f>IF(SUM(S43:S45)=0,"",SUM(S43:S45))</f>
+        <f>IF(SUM(S43:S48)=0,"",SUM(S43:S48))</f>
         <v/>
       </c>
       <c r="T42" s="12">
-        <f>SUM(T43:T45)</f>
+        <f>SUM(T43:T48)</f>
         <v/>
       </c>
       <c r="U42" s="12">
-        <f>IF(SUM(U43:U45)=0,"",SUM(U43:U45))</f>
+        <f>IF(SUM(U43:U48)=0,"",SUM(U43:U48))</f>
         <v/>
       </c>
       <c r="V42" s="13">
@@ -6866,19 +6874,19 @@
         <v/>
       </c>
       <c r="W42" s="12">
-        <f>IF(SUM(W43:W45)=0,"",SUM(W43:W45))</f>
+        <f>IF(SUM(W43:W48)=0,"",SUM(W43:W48))</f>
         <v/>
       </c>
       <c r="X42" s="12">
-        <f>IF(SUM(X43:X45)=0,"",SUM(X43:X45))</f>
+        <f>IF(SUM(X43:X48)=0,"",SUM(X43:X48))</f>
         <v/>
       </c>
       <c r="Y42" s="12">
-        <f>SUM(Y43:Y45)</f>
+        <f>SUM(Y43:Y48)</f>
         <v/>
       </c>
       <c r="Z42" s="12">
-        <f>IF(SUM(Z43:Z45)=0,"",SUM(Z43:Z45))</f>
+        <f>IF(SUM(Z43:Z48)=0,"",SUM(Z43:Z48))</f>
         <v/>
       </c>
       <c r="AA42" s="13">
@@ -6886,19 +6894,19 @@
         <v/>
       </c>
       <c r="AB42" s="12">
-        <f>IF(SUM(AB43:AB45)=0,"",SUM(AB43:AB45))</f>
+        <f>IF(SUM(AB43:AB48)=0,"",SUM(AB43:AB48))</f>
         <v/>
       </c>
       <c r="AC42" s="12">
-        <f>IF(SUM(AC43:AC45)=0,"",SUM(AC43:AC45))</f>
+        <f>IF(SUM(AC43:AC48)=0,"",SUM(AC43:AC48))</f>
         <v/>
       </c>
       <c r="AD42" s="12">
-        <f>SUM(AD43:AD45)</f>
+        <f>SUM(AD43:AD48)</f>
         <v/>
       </c>
       <c r="AE42" s="12">
-        <f>IF(SUM(AE43:AE45)=0,"",SUM(AE43:AE45))</f>
+        <f>IF(SUM(AE43:AE48)=0,"",SUM(AE43:AE48))</f>
         <v/>
       </c>
       <c r="AF42" s="13">
@@ -6906,19 +6914,19 @@
         <v/>
       </c>
       <c r="AG42" s="12">
-        <f>IF(SUM(AG43:AG45)=0,"",SUM(AG43:AG45))</f>
+        <f>IF(SUM(AG43:AG48)=0,"",SUM(AG43:AG48))</f>
         <v/>
       </c>
       <c r="AH42" s="12">
-        <f>IF(SUM(AH43:AH45)=0,"",SUM(AH43:AH45))</f>
+        <f>IF(SUM(AH43:AH48)=0,"",SUM(AH43:AH48))</f>
         <v/>
       </c>
       <c r="AI42" s="12">
-        <f>SUM(AI43:AI45)</f>
+        <f>SUM(AI43:AI48)</f>
         <v/>
       </c>
       <c r="AJ42" s="12">
-        <f>IF(SUM(AJ43:AJ45)=0,"",SUM(AJ43:AJ45))</f>
+        <f>IF(SUM(AJ43:AJ48)=0,"",SUM(AJ43:AJ48))</f>
         <v/>
       </c>
       <c r="AK42" s="13">
@@ -6926,19 +6934,19 @@
         <v/>
       </c>
       <c r="AL42" s="12">
-        <f>IF(SUM(AL43:AL45)=0,"",SUM(AL43:AL45))</f>
+        <f>IF(SUM(AL43:AL48)=0,"",SUM(AL43:AL48))</f>
         <v/>
       </c>
       <c r="AM42" s="12">
-        <f>IF(SUM(AM43:AM45)=0,"",SUM(AM43:AM45))</f>
+        <f>IF(SUM(AM43:AM48)=0,"",SUM(AM43:AM48))</f>
         <v/>
       </c>
       <c r="AN42" s="12">
-        <f>SUM(AN43:AN45)</f>
+        <f>SUM(AN43:AN48)</f>
         <v/>
       </c>
       <c r="AO42" s="12">
-        <f>IF(SUM(AO43:AO45)=0,"",SUM(AO43:AO45))</f>
+        <f>IF(SUM(AO43:AO48)=0,"",SUM(AO43:AO48))</f>
         <v/>
       </c>
       <c r="AP42" s="13">
@@ -6946,19 +6954,19 @@
         <v/>
       </c>
       <c r="AQ42" s="12">
-        <f>IF(SUM(AQ43:AQ45)=0,"",SUM(AQ43:AQ45))</f>
+        <f>IF(SUM(AQ43:AQ48)=0,"",SUM(AQ43:AQ48))</f>
         <v/>
       </c>
       <c r="AR42" s="12">
-        <f>IF(SUM(AR43:AR45)=0,"",SUM(AR43:AR45))</f>
+        <f>IF(SUM(AR43:AR48)=0,"",SUM(AR43:AR48))</f>
         <v/>
       </c>
       <c r="AS42" s="12">
-        <f>SUM(AS43:AS45)</f>
+        <f>SUM(AS43:AS48)</f>
         <v/>
       </c>
       <c r="AT42" s="12">
-        <f>IF(SUM(AT43:AT45)=0,"",SUM(AT43:AT45))</f>
+        <f>IF(SUM(AT43:AT48)=0,"",SUM(AT43:AT48))</f>
         <v/>
       </c>
       <c r="AU42" s="13">
@@ -6966,19 +6974,19 @@
         <v/>
       </c>
       <c r="AV42" s="12">
-        <f>IF(SUM(AV43:AV45)=0,"",SUM(AV43:AV45))</f>
+        <f>IF(SUM(AV43:AV48)=0,"",SUM(AV43:AV48))</f>
         <v/>
       </c>
       <c r="AW42" s="12">
-        <f>IF(SUM(AW43:AW45)=0,"",SUM(AW43:AW45))</f>
+        <f>IF(SUM(AW43:AW48)=0,"",SUM(AW43:AW48))</f>
         <v/>
       </c>
       <c r="AX42" s="12">
-        <f>SUM(AX43:AX45)</f>
+        <f>SUM(AX43:AX48)</f>
         <v/>
       </c>
       <c r="AY42" s="12">
-        <f>IF(SUM(AY43:AY45)=0,"",SUM(AY43:AY45))</f>
+        <f>IF(SUM(AY43:AY48)=0,"",SUM(AY43:AY48))</f>
         <v/>
       </c>
       <c r="AZ42" s="13">
@@ -6986,19 +6994,19 @@
         <v/>
       </c>
       <c r="BA42" s="12">
-        <f>IF(SUM(BA43:BA45)=0,"",SUM(BA43:BA45))</f>
+        <f>IF(SUM(BA43:BA48)=0,"",SUM(BA43:BA48))</f>
         <v/>
       </c>
       <c r="BB42" s="12">
-        <f>IF(SUM(BB43:BB45)=0,"",SUM(BB43:BB45))</f>
+        <f>IF(SUM(BB43:BB48)=0,"",SUM(BB43:BB48))</f>
         <v/>
       </c>
       <c r="BC42" s="12">
-        <f>SUM(BC43:BC45)</f>
+        <f>SUM(BC43:BC48)</f>
         <v/>
       </c>
       <c r="BD42" s="12">
-        <f>IF(SUM(BD43:BD45)=0,"",SUM(BD43:BD45))</f>
+        <f>IF(SUM(BD43:BD48)=0,"",SUM(BD43:BD48))</f>
         <v/>
       </c>
       <c r="BE42" s="13">
@@ -7006,19 +7014,19 @@
         <v/>
       </c>
       <c r="BF42" s="12">
-        <f>IF(SUM(BF43:BF45)=0,"",SUM(BF43:BF45))</f>
+        <f>IF(SUM(BF43:BF48)=0,"",SUM(BF43:BF48))</f>
         <v/>
       </c>
       <c r="BG42" s="12">
-        <f>IF(SUM(BG43:BG45)=0,"",SUM(BG43:BG45))</f>
+        <f>IF(SUM(BG43:BG48)=0,"",SUM(BG43:BG48))</f>
         <v/>
       </c>
       <c r="BH42" s="12">
-        <f>SUM(BH43:BH45)</f>
+        <f>SUM(BH43:BH48)</f>
         <v/>
       </c>
       <c r="BI42" s="12">
-        <f>IF(SUM(BI43:BI45)=0,"",SUM(BI43:BI45))</f>
+        <f>IF(SUM(BI43:BI48)=0,"",SUM(BI43:BI48))</f>
         <v/>
       </c>
       <c r="BJ42" s="13">
@@ -7434,366 +7442,1433 @@
         <v/>
       </c>
     </row>
-    <row r="48" ht="24" customHeight="1">
-      <c r="A48" s="25" t="inlineStr">
+    <row r="46" outlineLevel="1" ht="18" customHeight="1">
+      <c r="A46" s="17" t="n"/>
+      <c r="B46" s="18" t="n"/>
+      <c r="C46" s="18" t="n"/>
+      <c r="D46" s="18" t="n"/>
+      <c r="E46" s="18" t="n"/>
+      <c r="F46" s="18">
+        <f>IF(C46="","",C46-B46-E46)</f>
+        <v/>
+      </c>
+      <c r="G46" s="19">
+        <f>IF(OR(C46="",B46="",(B46+E46)=0),"",(C46-B46-E46)/(B46+E46))</f>
+        <v/>
+      </c>
+      <c r="H46" s="18" t="n"/>
+      <c r="I46" s="18" t="n"/>
+      <c r="J46" s="18" t="n"/>
+      <c r="K46" s="18">
+        <f>IF(H46="","",H46-C46-J46)</f>
+        <v/>
+      </c>
+      <c r="L46" s="19">
+        <f>IF(OR(H46="",C46="",(C46+J46)=0),"",(H46-C46-J46)/(C46+J46))</f>
+        <v/>
+      </c>
+      <c r="M46" s="18" t="n"/>
+      <c r="N46" s="18" t="n"/>
+      <c r="O46" s="18" t="n"/>
+      <c r="P46" s="18">
+        <f>IF(M46="","",M46-H46-O46)</f>
+        <v/>
+      </c>
+      <c r="Q46" s="19">
+        <f>IF(OR(M46="",H46="",(H46+O46)=0),"",(M46-H46-O46)/(H46+O46))</f>
+        <v/>
+      </c>
+      <c r="R46" s="18" t="n"/>
+      <c r="S46" s="18" t="n"/>
+      <c r="T46" s="18" t="n"/>
+      <c r="U46" s="18">
+        <f>IF(R46="","",R46-M46-T46)</f>
+        <v/>
+      </c>
+      <c r="V46" s="19">
+        <f>IF(OR(R46="",M46="",(M46+T46)=0),"",(R46-M46-T46)/(M46+T46))</f>
+        <v/>
+      </c>
+      <c r="W46" s="18" t="n"/>
+      <c r="X46" s="18" t="n"/>
+      <c r="Y46" s="18" t="n"/>
+      <c r="Z46" s="18">
+        <f>IF(W46="","",W46-R46-Y46)</f>
+        <v/>
+      </c>
+      <c r="AA46" s="19">
+        <f>IF(OR(W46="",R46="",(R46+Y46)=0),"",(W46-R46-Y46)/(R46+Y46))</f>
+        <v/>
+      </c>
+      <c r="AB46" s="18" t="n"/>
+      <c r="AC46" s="18" t="n"/>
+      <c r="AD46" s="18" t="n"/>
+      <c r="AE46" s="18">
+        <f>IF(AB46="","",AB46-W46-AD46)</f>
+        <v/>
+      </c>
+      <c r="AF46" s="19">
+        <f>IF(OR(AB46="",W46="",(W46+AD46)=0),"",(AB46-W46-AD46)/(W46+AD46))</f>
+        <v/>
+      </c>
+      <c r="AG46" s="18" t="n"/>
+      <c r="AH46" s="18" t="n"/>
+      <c r="AI46" s="18" t="n"/>
+      <c r="AJ46" s="18">
+        <f>IF(AG46="","",AG46-AB46-AI46)</f>
+        <v/>
+      </c>
+      <c r="AK46" s="19">
+        <f>IF(OR(AG46="",AB46="",(AB46+AI46)=0),"",(AG46-AB46-AI46)/(AB46+AI46))</f>
+        <v/>
+      </c>
+      <c r="AL46" s="18" t="n"/>
+      <c r="AM46" s="18" t="n"/>
+      <c r="AN46" s="18" t="n"/>
+      <c r="AO46" s="18">
+        <f>IF(AL46="","",AL46-AG46-AN46)</f>
+        <v/>
+      </c>
+      <c r="AP46" s="19">
+        <f>IF(OR(AL46="",AG46="",(AG46+AN46)=0),"",(AL46-AG46-AN46)/(AG46+AN46))</f>
+        <v/>
+      </c>
+      <c r="AQ46" s="18" t="n"/>
+      <c r="AR46" s="18" t="n"/>
+      <c r="AS46" s="18" t="n"/>
+      <c r="AT46" s="18">
+        <f>IF(AQ46="","",AQ46-AL46-AS46)</f>
+        <v/>
+      </c>
+      <c r="AU46" s="19">
+        <f>IF(OR(AQ46="",AL46="",(AL46+AS46)=0),"",(AQ46-AL46-AS46)/(AL46+AS46))</f>
+        <v/>
+      </c>
+      <c r="AV46" s="18" t="n"/>
+      <c r="AW46" s="18" t="n"/>
+      <c r="AX46" s="18" t="n"/>
+      <c r="AY46" s="18">
+        <f>IF(AV46="","",AV46-AQ46-AX46)</f>
+        <v/>
+      </c>
+      <c r="AZ46" s="19">
+        <f>IF(OR(AV46="",AQ46="",(AQ46+AX46)=0),"",(AV46-AQ46-AX46)/(AQ46+AX46))</f>
+        <v/>
+      </c>
+      <c r="BA46" s="18" t="n"/>
+      <c r="BB46" s="18" t="n"/>
+      <c r="BC46" s="18" t="n"/>
+      <c r="BD46" s="18">
+        <f>IF(BA46="","",BA46-AV46-BC46)</f>
+        <v/>
+      </c>
+      <c r="BE46" s="19">
+        <f>IF(OR(BA46="",AV46="",(AV46+BC46)=0),"",(BA46-AV46-BC46)/(AV46+BC46))</f>
+        <v/>
+      </c>
+      <c r="BF46" s="18" t="n"/>
+      <c r="BG46" s="18" t="n"/>
+      <c r="BH46" s="18" t="n"/>
+      <c r="BI46" s="18">
+        <f>IF(BF46="","",BF46-BA46-BH46)</f>
+        <v/>
+      </c>
+      <c r="BJ46" s="19">
+        <f>IF(OR(BF46="",BA46="",(BA46+BH46)=0),"",(BF46-BA46-BH46)/(BA46+BH46))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" outlineLevel="1" ht="18" customHeight="1">
+      <c r="A47" s="14" t="n"/>
+      <c r="B47" s="15" t="n"/>
+      <c r="C47" s="15" t="n"/>
+      <c r="D47" s="15" t="n"/>
+      <c r="E47" s="15" t="n"/>
+      <c r="F47" s="15">
+        <f>IF(C47="","",C47-B47-E47)</f>
+        <v/>
+      </c>
+      <c r="G47" s="16">
+        <f>IF(OR(C47="",B47="",(B47+E47)=0),"",(C47-B47-E47)/(B47+E47))</f>
+        <v/>
+      </c>
+      <c r="H47" s="15" t="n"/>
+      <c r="I47" s="15" t="n"/>
+      <c r="J47" s="15" t="n"/>
+      <c r="K47" s="15">
+        <f>IF(H47="","",H47-C47-J47)</f>
+        <v/>
+      </c>
+      <c r="L47" s="16">
+        <f>IF(OR(H47="",C47="",(C47+J47)=0),"",(H47-C47-J47)/(C47+J47))</f>
+        <v/>
+      </c>
+      <c r="M47" s="15" t="n"/>
+      <c r="N47" s="15" t="n"/>
+      <c r="O47" s="15" t="n"/>
+      <c r="P47" s="15">
+        <f>IF(M47="","",M47-H47-O47)</f>
+        <v/>
+      </c>
+      <c r="Q47" s="16">
+        <f>IF(OR(M47="",H47="",(H47+O47)=0),"",(M47-H47-O47)/(H47+O47))</f>
+        <v/>
+      </c>
+      <c r="R47" s="15" t="n"/>
+      <c r="S47" s="15" t="n"/>
+      <c r="T47" s="15" t="n"/>
+      <c r="U47" s="15">
+        <f>IF(R47="","",R47-M47-T47)</f>
+        <v/>
+      </c>
+      <c r="V47" s="16">
+        <f>IF(OR(R47="",M47="",(M47+T47)=0),"",(R47-M47-T47)/(M47+T47))</f>
+        <v/>
+      </c>
+      <c r="W47" s="15" t="n"/>
+      <c r="X47" s="15" t="n"/>
+      <c r="Y47" s="15" t="n"/>
+      <c r="Z47" s="15">
+        <f>IF(W47="","",W47-R47-Y47)</f>
+        <v/>
+      </c>
+      <c r="AA47" s="16">
+        <f>IF(OR(W47="",R47="",(R47+Y47)=0),"",(W47-R47-Y47)/(R47+Y47))</f>
+        <v/>
+      </c>
+      <c r="AB47" s="15" t="n"/>
+      <c r="AC47" s="15" t="n"/>
+      <c r="AD47" s="15" t="n"/>
+      <c r="AE47" s="15">
+        <f>IF(AB47="","",AB47-W47-AD47)</f>
+        <v/>
+      </c>
+      <c r="AF47" s="16">
+        <f>IF(OR(AB47="",W47="",(W47+AD47)=0),"",(AB47-W47-AD47)/(W47+AD47))</f>
+        <v/>
+      </c>
+      <c r="AG47" s="15" t="n"/>
+      <c r="AH47" s="15" t="n"/>
+      <c r="AI47" s="15" t="n"/>
+      <c r="AJ47" s="15">
+        <f>IF(AG47="","",AG47-AB47-AI47)</f>
+        <v/>
+      </c>
+      <c r="AK47" s="16">
+        <f>IF(OR(AG47="",AB47="",(AB47+AI47)=0),"",(AG47-AB47-AI47)/(AB47+AI47))</f>
+        <v/>
+      </c>
+      <c r="AL47" s="15" t="n"/>
+      <c r="AM47" s="15" t="n"/>
+      <c r="AN47" s="15" t="n"/>
+      <c r="AO47" s="15">
+        <f>IF(AL47="","",AL47-AG47-AN47)</f>
+        <v/>
+      </c>
+      <c r="AP47" s="16">
+        <f>IF(OR(AL47="",AG47="",(AG47+AN47)=0),"",(AL47-AG47-AN47)/(AG47+AN47))</f>
+        <v/>
+      </c>
+      <c r="AQ47" s="15" t="n"/>
+      <c r="AR47" s="15" t="n"/>
+      <c r="AS47" s="15" t="n"/>
+      <c r="AT47" s="15">
+        <f>IF(AQ47="","",AQ47-AL47-AS47)</f>
+        <v/>
+      </c>
+      <c r="AU47" s="16">
+        <f>IF(OR(AQ47="",AL47="",(AL47+AS47)=0),"",(AQ47-AL47-AS47)/(AL47+AS47))</f>
+        <v/>
+      </c>
+      <c r="AV47" s="15" t="n"/>
+      <c r="AW47" s="15" t="n"/>
+      <c r="AX47" s="15" t="n"/>
+      <c r="AY47" s="15">
+        <f>IF(AV47="","",AV47-AQ47-AX47)</f>
+        <v/>
+      </c>
+      <c r="AZ47" s="16">
+        <f>IF(OR(AV47="",AQ47="",(AQ47+AX47)=0),"",(AV47-AQ47-AX47)/(AQ47+AX47))</f>
+        <v/>
+      </c>
+      <c r="BA47" s="15" t="n"/>
+      <c r="BB47" s="15" t="n"/>
+      <c r="BC47" s="15" t="n"/>
+      <c r="BD47" s="15">
+        <f>IF(BA47="","",BA47-AV47-BC47)</f>
+        <v/>
+      </c>
+      <c r="BE47" s="16">
+        <f>IF(OR(BA47="",AV47="",(AV47+BC47)=0),"",(BA47-AV47-BC47)/(AV47+BC47))</f>
+        <v/>
+      </c>
+      <c r="BF47" s="15" t="n"/>
+      <c r="BG47" s="15" t="n"/>
+      <c r="BH47" s="15" t="n"/>
+      <c r="BI47" s="15">
+        <f>IF(BF47="","",BF47-BA47-BH47)</f>
+        <v/>
+      </c>
+      <c r="BJ47" s="16">
+        <f>IF(OR(BF47="",BA47="",(BA47+BH47)=0),"",(BF47-BA47-BH47)/(BA47+BH47))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" outlineLevel="1" ht="18" customHeight="1">
+      <c r="A48" s="17" t="n"/>
+      <c r="B48" s="18" t="n"/>
+      <c r="C48" s="18" t="n"/>
+      <c r="D48" s="18" t="n"/>
+      <c r="E48" s="18" t="n"/>
+      <c r="F48" s="18">
+        <f>IF(C48="","",C48-B48-E48)</f>
+        <v/>
+      </c>
+      <c r="G48" s="19">
+        <f>IF(OR(C48="",B48="",(B48+E48)=0),"",(C48-B48-E48)/(B48+E48))</f>
+        <v/>
+      </c>
+      <c r="H48" s="18" t="n"/>
+      <c r="I48" s="18" t="n"/>
+      <c r="J48" s="18" t="n"/>
+      <c r="K48" s="18">
+        <f>IF(H48="","",H48-C48-J48)</f>
+        <v/>
+      </c>
+      <c r="L48" s="19">
+        <f>IF(OR(H48="",C48="",(C48+J48)=0),"",(H48-C48-J48)/(C48+J48))</f>
+        <v/>
+      </c>
+      <c r="M48" s="18" t="n"/>
+      <c r="N48" s="18" t="n"/>
+      <c r="O48" s="18" t="n"/>
+      <c r="P48" s="18">
+        <f>IF(M48="","",M48-H48-O48)</f>
+        <v/>
+      </c>
+      <c r="Q48" s="19">
+        <f>IF(OR(M48="",H48="",(H48+O48)=0),"",(M48-H48-O48)/(H48+O48))</f>
+        <v/>
+      </c>
+      <c r="R48" s="18" t="n"/>
+      <c r="S48" s="18" t="n"/>
+      <c r="T48" s="18" t="n"/>
+      <c r="U48" s="18">
+        <f>IF(R48="","",R48-M48-T48)</f>
+        <v/>
+      </c>
+      <c r="V48" s="19">
+        <f>IF(OR(R48="",M48="",(M48+T48)=0),"",(R48-M48-T48)/(M48+T48))</f>
+        <v/>
+      </c>
+      <c r="W48" s="18" t="n"/>
+      <c r="X48" s="18" t="n"/>
+      <c r="Y48" s="18" t="n"/>
+      <c r="Z48" s="18">
+        <f>IF(W48="","",W48-R48-Y48)</f>
+        <v/>
+      </c>
+      <c r="AA48" s="19">
+        <f>IF(OR(W48="",R48="",(R48+Y48)=0),"",(W48-R48-Y48)/(R48+Y48))</f>
+        <v/>
+      </c>
+      <c r="AB48" s="18" t="n"/>
+      <c r="AC48" s="18" t="n"/>
+      <c r="AD48" s="18" t="n"/>
+      <c r="AE48" s="18">
+        <f>IF(AB48="","",AB48-W48-AD48)</f>
+        <v/>
+      </c>
+      <c r="AF48" s="19">
+        <f>IF(OR(AB48="",W48="",(W48+AD48)=0),"",(AB48-W48-AD48)/(W48+AD48))</f>
+        <v/>
+      </c>
+      <c r="AG48" s="18" t="n"/>
+      <c r="AH48" s="18" t="n"/>
+      <c r="AI48" s="18" t="n"/>
+      <c r="AJ48" s="18">
+        <f>IF(AG48="","",AG48-AB48-AI48)</f>
+        <v/>
+      </c>
+      <c r="AK48" s="19">
+        <f>IF(OR(AG48="",AB48="",(AB48+AI48)=0),"",(AG48-AB48-AI48)/(AB48+AI48))</f>
+        <v/>
+      </c>
+      <c r="AL48" s="18" t="n"/>
+      <c r="AM48" s="18" t="n"/>
+      <c r="AN48" s="18" t="n"/>
+      <c r="AO48" s="18">
+        <f>IF(AL48="","",AL48-AG48-AN48)</f>
+        <v/>
+      </c>
+      <c r="AP48" s="19">
+        <f>IF(OR(AL48="",AG48="",(AG48+AN48)=0),"",(AL48-AG48-AN48)/(AG48+AN48))</f>
+        <v/>
+      </c>
+      <c r="AQ48" s="18" t="n"/>
+      <c r="AR48" s="18" t="n"/>
+      <c r="AS48" s="18" t="n"/>
+      <c r="AT48" s="18">
+        <f>IF(AQ48="","",AQ48-AL48-AS48)</f>
+        <v/>
+      </c>
+      <c r="AU48" s="19">
+        <f>IF(OR(AQ48="",AL48="",(AL48+AS48)=0),"",(AQ48-AL48-AS48)/(AL48+AS48))</f>
+        <v/>
+      </c>
+      <c r="AV48" s="18" t="n"/>
+      <c r="AW48" s="18" t="n"/>
+      <c r="AX48" s="18" t="n"/>
+      <c r="AY48" s="18">
+        <f>IF(AV48="","",AV48-AQ48-AX48)</f>
+        <v/>
+      </c>
+      <c r="AZ48" s="19">
+        <f>IF(OR(AV48="",AQ48="",(AQ48+AX48)=0),"",(AV48-AQ48-AX48)/(AQ48+AX48))</f>
+        <v/>
+      </c>
+      <c r="BA48" s="18" t="n"/>
+      <c r="BB48" s="18" t="n"/>
+      <c r="BC48" s="18" t="n"/>
+      <c r="BD48" s="18">
+        <f>IF(BA48="","",BA48-AV48-BC48)</f>
+        <v/>
+      </c>
+      <c r="BE48" s="19">
+        <f>IF(OR(BA48="",AV48="",(AV48+BC48)=0),"",(BA48-AV48-BC48)/(AV48+BC48))</f>
+        <v/>
+      </c>
+      <c r="BF48" s="18" t="n"/>
+      <c r="BG48" s="18" t="n"/>
+      <c r="BH48" s="18" t="n"/>
+      <c r="BI48" s="18">
+        <f>IF(BF48="","",BF48-BA48-BH48)</f>
+        <v/>
+      </c>
+      <c r="BJ48" s="19">
+        <f>IF(OR(BF48="",BA48="",(BA48+BH48)=0),"",(BF48-BA48-BH48)/(BA48+BH48))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="21" customHeight="1">
+      <c r="A49" s="25" t="inlineStr">
+        <is>
+          <t>POUPANÇA</t>
+        </is>
+      </c>
+      <c r="B49" s="12">
+        <f>IF(SUM(B50,B51,B52)=0,"",SUM(B50,B51,B52))</f>
+        <v/>
+      </c>
+      <c r="C49" s="12">
+        <f>IF(SUM(C50:C52)=0,"",SUM(C50:C52))</f>
+        <v/>
+      </c>
+      <c r="D49" s="12">
+        <f>IF(SUM(D50:D52)=0,"",SUM(D50:D52))</f>
+        <v/>
+      </c>
+      <c r="E49" s="12">
+        <f>SUM(E50:E52)</f>
+        <v/>
+      </c>
+      <c r="F49" s="12">
+        <f>IF(SUM(F50:F52)=0,"",SUM(F50:F52))</f>
+        <v/>
+      </c>
+      <c r="G49" s="13">
+        <f>IF(OR(C49="",B49="",(B49+E49)=0),"",(C49-B49-E49)/(B49+E49))</f>
+        <v/>
+      </c>
+      <c r="H49" s="12">
+        <f>IF(SUM(H50:H52)=0,"",SUM(H50:H52))</f>
+        <v/>
+      </c>
+      <c r="I49" s="12">
+        <f>IF(SUM(I50:I52)=0,"",SUM(I50:I52))</f>
+        <v/>
+      </c>
+      <c r="J49" s="12">
+        <f>SUM(J50:J52)</f>
+        <v/>
+      </c>
+      <c r="K49" s="12">
+        <f>IF(SUM(K50:K52)=0,"",SUM(K50:K52))</f>
+        <v/>
+      </c>
+      <c r="L49" s="13">
+        <f>IF(OR(H49="",C49="",(C49+J49)=0),"",(H49-C49-J49)/(C49+J49))</f>
+        <v/>
+      </c>
+      <c r="M49" s="12">
+        <f>IF(SUM(M50:M52)=0,"",SUM(M50:M52))</f>
+        <v/>
+      </c>
+      <c r="N49" s="12">
+        <f>IF(SUM(N50:N52)=0,"",SUM(N50:N52))</f>
+        <v/>
+      </c>
+      <c r="O49" s="12">
+        <f>SUM(O50:O52)</f>
+        <v/>
+      </c>
+      <c r="P49" s="12">
+        <f>IF(SUM(P50:P52)=0,"",SUM(P50:P52))</f>
+        <v/>
+      </c>
+      <c r="Q49" s="13">
+        <f>IF(OR(M49="",H49="",(H49+O49)=0),"",(M49-H49-O49)/(H49+O49))</f>
+        <v/>
+      </c>
+      <c r="R49" s="12">
+        <f>IF(SUM(R50:R52)=0,"",SUM(R50:R52))</f>
+        <v/>
+      </c>
+      <c r="S49" s="12">
+        <f>IF(SUM(S50:S52)=0,"",SUM(S50:S52))</f>
+        <v/>
+      </c>
+      <c r="T49" s="12">
+        <f>SUM(T50:T52)</f>
+        <v/>
+      </c>
+      <c r="U49" s="12">
+        <f>IF(SUM(U50:U52)=0,"",SUM(U50:U52))</f>
+        <v/>
+      </c>
+      <c r="V49" s="13">
+        <f>IF(OR(R49="",M49="",(M49+T49)=0),"",(R49-M49-T49)/(M49+T49))</f>
+        <v/>
+      </c>
+      <c r="W49" s="12">
+        <f>IF(SUM(W50:W52)=0,"",SUM(W50:W52))</f>
+        <v/>
+      </c>
+      <c r="X49" s="12">
+        <f>IF(SUM(X50:X52)=0,"",SUM(X50:X52))</f>
+        <v/>
+      </c>
+      <c r="Y49" s="12">
+        <f>SUM(Y50:Y52)</f>
+        <v/>
+      </c>
+      <c r="Z49" s="12">
+        <f>IF(SUM(Z50:Z52)=0,"",SUM(Z50:Z52))</f>
+        <v/>
+      </c>
+      <c r="AA49" s="13">
+        <f>IF(OR(W49="",R49="",(R49+Y49)=0),"",(W49-R49-Y49)/(R49+Y49))</f>
+        <v/>
+      </c>
+      <c r="AB49" s="12">
+        <f>IF(SUM(AB50:AB52)=0,"",SUM(AB50:AB52))</f>
+        <v/>
+      </c>
+      <c r="AC49" s="12">
+        <f>IF(SUM(AC50:AC52)=0,"",SUM(AC50:AC52))</f>
+        <v/>
+      </c>
+      <c r="AD49" s="12">
+        <f>SUM(AD50:AD52)</f>
+        <v/>
+      </c>
+      <c r="AE49" s="12">
+        <f>IF(SUM(AE50:AE52)=0,"",SUM(AE50:AE52))</f>
+        <v/>
+      </c>
+      <c r="AF49" s="13">
+        <f>IF(OR(AB49="",W49="",(W49+AD49)=0),"",(AB49-W49-AD49)/(W49+AD49))</f>
+        <v/>
+      </c>
+      <c r="AG49" s="12">
+        <f>IF(SUM(AG50:AG52)=0,"",SUM(AG50:AG52))</f>
+        <v/>
+      </c>
+      <c r="AH49" s="12">
+        <f>IF(SUM(AH50:AH52)=0,"",SUM(AH50:AH52))</f>
+        <v/>
+      </c>
+      <c r="AI49" s="12">
+        <f>SUM(AI50:AI52)</f>
+        <v/>
+      </c>
+      <c r="AJ49" s="12">
+        <f>IF(SUM(AJ50:AJ52)=0,"",SUM(AJ50:AJ52))</f>
+        <v/>
+      </c>
+      <c r="AK49" s="13">
+        <f>IF(OR(AG49="",AB49="",(AB49+AI49)=0),"",(AG49-AB49-AI49)/(AB49+AI49))</f>
+        <v/>
+      </c>
+      <c r="AL49" s="12">
+        <f>IF(SUM(AL50:AL52)=0,"",SUM(AL50:AL52))</f>
+        <v/>
+      </c>
+      <c r="AM49" s="12">
+        <f>IF(SUM(AM50:AM52)=0,"",SUM(AM50:AM52))</f>
+        <v/>
+      </c>
+      <c r="AN49" s="12">
+        <f>SUM(AN50:AN52)</f>
+        <v/>
+      </c>
+      <c r="AO49" s="12">
+        <f>IF(SUM(AO50:AO52)=0,"",SUM(AO50:AO52))</f>
+        <v/>
+      </c>
+      <c r="AP49" s="13">
+        <f>IF(OR(AL49="",AG49="",(AG49+AN49)=0),"",(AL49-AG49-AN49)/(AG49+AN49))</f>
+        <v/>
+      </c>
+      <c r="AQ49" s="12">
+        <f>IF(SUM(AQ50:AQ52)=0,"",SUM(AQ50:AQ52))</f>
+        <v/>
+      </c>
+      <c r="AR49" s="12">
+        <f>IF(SUM(AR50:AR52)=0,"",SUM(AR50:AR52))</f>
+        <v/>
+      </c>
+      <c r="AS49" s="12">
+        <f>SUM(AS50:AS52)</f>
+        <v/>
+      </c>
+      <c r="AT49" s="12">
+        <f>IF(SUM(AT50:AT52)=0,"",SUM(AT50:AT52))</f>
+        <v/>
+      </c>
+      <c r="AU49" s="13">
+        <f>IF(OR(AQ49="",AL49="",(AL49+AS49)=0),"",(AQ49-AL49-AS49)/(AL49+AS49))</f>
+        <v/>
+      </c>
+      <c r="AV49" s="12">
+        <f>IF(SUM(AV50:AV52)=0,"",SUM(AV50:AV52))</f>
+        <v/>
+      </c>
+      <c r="AW49" s="12">
+        <f>IF(SUM(AW50:AW52)=0,"",SUM(AW50:AW52))</f>
+        <v/>
+      </c>
+      <c r="AX49" s="12">
+        <f>SUM(AX50:AX52)</f>
+        <v/>
+      </c>
+      <c r="AY49" s="12">
+        <f>IF(SUM(AY50:AY52)=0,"",SUM(AY50:AY52))</f>
+        <v/>
+      </c>
+      <c r="AZ49" s="13">
+        <f>IF(OR(AV49="",AQ49="",(AQ49+AX49)=0),"",(AV49-AQ49-AX49)/(AQ49+AX49))</f>
+        <v/>
+      </c>
+      <c r="BA49" s="12">
+        <f>IF(SUM(BA50:BA52)=0,"",SUM(BA50:BA52))</f>
+        <v/>
+      </c>
+      <c r="BB49" s="12">
+        <f>IF(SUM(BB50:BB52)=0,"",SUM(BB50:BB52))</f>
+        <v/>
+      </c>
+      <c r="BC49" s="12">
+        <f>SUM(BC50:BC52)</f>
+        <v/>
+      </c>
+      <c r="BD49" s="12">
+        <f>IF(SUM(BD50:BD52)=0,"",SUM(BD50:BD52))</f>
+        <v/>
+      </c>
+      <c r="BE49" s="13">
+        <f>IF(OR(BA49="",AV49="",(AV49+BC49)=0),"",(BA49-AV49-BC49)/(AV49+BC49))</f>
+        <v/>
+      </c>
+      <c r="BF49" s="12">
+        <f>IF(SUM(BF50:BF52)=0,"",SUM(BF50:BF52))</f>
+        <v/>
+      </c>
+      <c r="BG49" s="12">
+        <f>IF(SUM(BG50:BG52)=0,"",SUM(BG50:BG52))</f>
+        <v/>
+      </c>
+      <c r="BH49" s="12">
+        <f>SUM(BH50:BH52)</f>
+        <v/>
+      </c>
+      <c r="BI49" s="12">
+        <f>IF(SUM(BI50:BI52)=0,"",SUM(BI50:BI52))</f>
+        <v/>
+      </c>
+      <c r="BJ49" s="13">
+        <f>IF(OR(BF49="",BA49="",(BA49+BH49)=0),"",(BF49-BA49-BH49)/(BA49+BH49))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" outlineLevel="1" ht="18" customHeight="1">
+      <c r="A50" s="14" t="n"/>
+      <c r="B50" s="15" t="n"/>
+      <c r="C50" s="15" t="n"/>
+      <c r="D50" s="15" t="n"/>
+      <c r="E50" s="15" t="n"/>
+      <c r="F50" s="15">
+        <f>IF(C50="","",C50-B50-E50)</f>
+        <v/>
+      </c>
+      <c r="G50" s="16">
+        <f>IF(OR(C50="",B50="",(B50+E50)=0),"",(C50-B50-E50)/(B50+E50))</f>
+        <v/>
+      </c>
+      <c r="H50" s="15" t="n"/>
+      <c r="I50" s="15" t="n"/>
+      <c r="J50" s="15" t="n"/>
+      <c r="K50" s="15">
+        <f>IF(H50="","",H50-C50-J50)</f>
+        <v/>
+      </c>
+      <c r="L50" s="16">
+        <f>IF(OR(H50="",C50="",(C50+J50)=0),"",(H50-C50-J50)/(C50+J50))</f>
+        <v/>
+      </c>
+      <c r="M50" s="15" t="n"/>
+      <c r="N50" s="15" t="n"/>
+      <c r="O50" s="15" t="n"/>
+      <c r="P50" s="15">
+        <f>IF(M50="","",M50-H50-O50)</f>
+        <v/>
+      </c>
+      <c r="Q50" s="16">
+        <f>IF(OR(M50="",H50="",(H50+O50)=0),"",(M50-H50-O50)/(H50+O50))</f>
+        <v/>
+      </c>
+      <c r="R50" s="15" t="n"/>
+      <c r="S50" s="15" t="n"/>
+      <c r="T50" s="15" t="n"/>
+      <c r="U50" s="15">
+        <f>IF(R50="","",R50-M50-T50)</f>
+        <v/>
+      </c>
+      <c r="V50" s="16">
+        <f>IF(OR(R50="",M50="",(M50+T50)=0),"",(R50-M50-T50)/(M50+T50))</f>
+        <v/>
+      </c>
+      <c r="W50" s="15" t="n"/>
+      <c r="X50" s="15" t="n"/>
+      <c r="Y50" s="15" t="n"/>
+      <c r="Z50" s="15">
+        <f>IF(W50="","",W50-R50-Y50)</f>
+        <v/>
+      </c>
+      <c r="AA50" s="16">
+        <f>IF(OR(W50="",R50="",(R50+Y50)=0),"",(W50-R50-Y50)/(R50+Y50))</f>
+        <v/>
+      </c>
+      <c r="AB50" s="15" t="n"/>
+      <c r="AC50" s="15" t="n"/>
+      <c r="AD50" s="15" t="n"/>
+      <c r="AE50" s="15">
+        <f>IF(AB50="","",AB50-W50-AD50)</f>
+        <v/>
+      </c>
+      <c r="AF50" s="16">
+        <f>IF(OR(AB50="",W50="",(W50+AD50)=0),"",(AB50-W50-AD50)/(W50+AD50))</f>
+        <v/>
+      </c>
+      <c r="AG50" s="15" t="n"/>
+      <c r="AH50" s="15" t="n"/>
+      <c r="AI50" s="15" t="n"/>
+      <c r="AJ50" s="15">
+        <f>IF(AG50="","",AG50-AB50-AI50)</f>
+        <v/>
+      </c>
+      <c r="AK50" s="16">
+        <f>IF(OR(AG50="",AB50="",(AB50+AI50)=0),"",(AG50-AB50-AI50)/(AB50+AI50))</f>
+        <v/>
+      </c>
+      <c r="AL50" s="15" t="n"/>
+      <c r="AM50" s="15" t="n"/>
+      <c r="AN50" s="15" t="n"/>
+      <c r="AO50" s="15">
+        <f>IF(AL50="","",AL50-AG50-AN50)</f>
+        <v/>
+      </c>
+      <c r="AP50" s="16">
+        <f>IF(OR(AL50="",AG50="",(AG50+AN50)=0),"",(AL50-AG50-AN50)/(AG50+AN50))</f>
+        <v/>
+      </c>
+      <c r="AQ50" s="15" t="n"/>
+      <c r="AR50" s="15" t="n"/>
+      <c r="AS50" s="15" t="n"/>
+      <c r="AT50" s="15">
+        <f>IF(AQ50="","",AQ50-AL50-AS50)</f>
+        <v/>
+      </c>
+      <c r="AU50" s="16">
+        <f>IF(OR(AQ50="",AL50="",(AL50+AS50)=0),"",(AQ50-AL50-AS50)/(AL50+AS50))</f>
+        <v/>
+      </c>
+      <c r="AV50" s="15" t="n"/>
+      <c r="AW50" s="15" t="n"/>
+      <c r="AX50" s="15" t="n"/>
+      <c r="AY50" s="15">
+        <f>IF(AV50="","",AV50-AQ50-AX50)</f>
+        <v/>
+      </c>
+      <c r="AZ50" s="16">
+        <f>IF(OR(AV50="",AQ50="",(AQ50+AX50)=0),"",(AV50-AQ50-AX50)/(AQ50+AX50))</f>
+        <v/>
+      </c>
+      <c r="BA50" s="15" t="n"/>
+      <c r="BB50" s="15" t="n"/>
+      <c r="BC50" s="15" t="n"/>
+      <c r="BD50" s="15">
+        <f>IF(BA50="","",BA50-AV50-BC50)</f>
+        <v/>
+      </c>
+      <c r="BE50" s="16">
+        <f>IF(OR(BA50="",AV50="",(AV50+BC50)=0),"",(BA50-AV50-BC50)/(AV50+BC50))</f>
+        <v/>
+      </c>
+      <c r="BF50" s="15" t="n"/>
+      <c r="BG50" s="15" t="n"/>
+      <c r="BH50" s="15" t="n"/>
+      <c r="BI50" s="15">
+        <f>IF(BF50="","",BF50-BA50-BH50)</f>
+        <v/>
+      </c>
+      <c r="BJ50" s="16">
+        <f>IF(OR(BF50="",BA50="",(BA50+BH50)=0),"",(BF50-BA50-BH50)/(BA50+BH50))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" outlineLevel="1" ht="18" customHeight="1">
+      <c r="A51" s="17" t="n"/>
+      <c r="B51" s="18" t="n"/>
+      <c r="C51" s="18" t="n"/>
+      <c r="D51" s="18" t="n"/>
+      <c r="E51" s="18" t="n"/>
+      <c r="F51" s="18">
+        <f>IF(C51="","",C51-B51-E51)</f>
+        <v/>
+      </c>
+      <c r="G51" s="19">
+        <f>IF(OR(C51="",B51="",(B51+E51)=0),"",(C51-B51-E51)/(B51+E51))</f>
+        <v/>
+      </c>
+      <c r="H51" s="18" t="n"/>
+      <c r="I51" s="18" t="n"/>
+      <c r="J51" s="18" t="n"/>
+      <c r="K51" s="18">
+        <f>IF(H51="","",H51-C51-J51)</f>
+        <v/>
+      </c>
+      <c r="L51" s="19">
+        <f>IF(OR(H51="",C51="",(C51+J51)=0),"",(H51-C51-J51)/(C51+J51))</f>
+        <v/>
+      </c>
+      <c r="M51" s="18" t="n"/>
+      <c r="N51" s="18" t="n"/>
+      <c r="O51" s="18" t="n"/>
+      <c r="P51" s="18">
+        <f>IF(M51="","",M51-H51-O51)</f>
+        <v/>
+      </c>
+      <c r="Q51" s="19">
+        <f>IF(OR(M51="",H51="",(H51+O51)=0),"",(M51-H51-O51)/(H51+O51))</f>
+        <v/>
+      </c>
+      <c r="R51" s="18" t="n"/>
+      <c r="S51" s="18" t="n"/>
+      <c r="T51" s="18" t="n"/>
+      <c r="U51" s="18">
+        <f>IF(R51="","",R51-M51-T51)</f>
+        <v/>
+      </c>
+      <c r="V51" s="19">
+        <f>IF(OR(R51="",M51="",(M51+T51)=0),"",(R51-M51-T51)/(M51+T51))</f>
+        <v/>
+      </c>
+      <c r="W51" s="18" t="n"/>
+      <c r="X51" s="18" t="n"/>
+      <c r="Y51" s="18" t="n"/>
+      <c r="Z51" s="18">
+        <f>IF(W51="","",W51-R51-Y51)</f>
+        <v/>
+      </c>
+      <c r="AA51" s="19">
+        <f>IF(OR(W51="",R51="",(R51+Y51)=0),"",(W51-R51-Y51)/(R51+Y51))</f>
+        <v/>
+      </c>
+      <c r="AB51" s="18" t="n"/>
+      <c r="AC51" s="18" t="n"/>
+      <c r="AD51" s="18" t="n"/>
+      <c r="AE51" s="18">
+        <f>IF(AB51="","",AB51-W51-AD51)</f>
+        <v/>
+      </c>
+      <c r="AF51" s="19">
+        <f>IF(OR(AB51="",W51="",(W51+AD51)=0),"",(AB51-W51-AD51)/(W51+AD51))</f>
+        <v/>
+      </c>
+      <c r="AG51" s="18" t="n"/>
+      <c r="AH51" s="18" t="n"/>
+      <c r="AI51" s="18" t="n"/>
+      <c r="AJ51" s="18">
+        <f>IF(AG51="","",AG51-AB51-AI51)</f>
+        <v/>
+      </c>
+      <c r="AK51" s="19">
+        <f>IF(OR(AG51="",AB51="",(AB51+AI51)=0),"",(AG51-AB51-AI51)/(AB51+AI51))</f>
+        <v/>
+      </c>
+      <c r="AL51" s="18" t="n"/>
+      <c r="AM51" s="18" t="n"/>
+      <c r="AN51" s="18" t="n"/>
+      <c r="AO51" s="18">
+        <f>IF(AL51="","",AL51-AG51-AN51)</f>
+        <v/>
+      </c>
+      <c r="AP51" s="19">
+        <f>IF(OR(AL51="",AG51="",(AG51+AN51)=0),"",(AL51-AG51-AN51)/(AG51+AN51))</f>
+        <v/>
+      </c>
+      <c r="AQ51" s="18" t="n"/>
+      <c r="AR51" s="18" t="n"/>
+      <c r="AS51" s="18" t="n"/>
+      <c r="AT51" s="18">
+        <f>IF(AQ51="","",AQ51-AL51-AS51)</f>
+        <v/>
+      </c>
+      <c r="AU51" s="19">
+        <f>IF(OR(AQ51="",AL51="",(AL51+AS51)=0),"",(AQ51-AL51-AS51)/(AL51+AS51))</f>
+        <v/>
+      </c>
+      <c r="AV51" s="18" t="n"/>
+      <c r="AW51" s="18" t="n"/>
+      <c r="AX51" s="18" t="n"/>
+      <c r="AY51" s="18">
+        <f>IF(AV51="","",AV51-AQ51-AX51)</f>
+        <v/>
+      </c>
+      <c r="AZ51" s="19">
+        <f>IF(OR(AV51="",AQ51="",(AQ51+AX51)=0),"",(AV51-AQ51-AX51)/(AQ51+AX51))</f>
+        <v/>
+      </c>
+      <c r="BA51" s="18" t="n"/>
+      <c r="BB51" s="18" t="n"/>
+      <c r="BC51" s="18" t="n"/>
+      <c r="BD51" s="18">
+        <f>IF(BA51="","",BA51-AV51-BC51)</f>
+        <v/>
+      </c>
+      <c r="BE51" s="19">
+        <f>IF(OR(BA51="",AV51="",(AV51+BC51)=0),"",(BA51-AV51-BC51)/(AV51+BC51))</f>
+        <v/>
+      </c>
+      <c r="BF51" s="18" t="n"/>
+      <c r="BG51" s="18" t="n"/>
+      <c r="BH51" s="18" t="n"/>
+      <c r="BI51" s="18">
+        <f>IF(BF51="","",BF51-BA51-BH51)</f>
+        <v/>
+      </c>
+      <c r="BJ51" s="19">
+        <f>IF(OR(BF51="",BA51="",(BA51+BH51)=0),"",(BF51-BA51-BH51)/(BA51+BH51))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" outlineLevel="1" ht="18" customHeight="1">
+      <c r="A52" s="14" t="n"/>
+      <c r="B52" s="15" t="n"/>
+      <c r="C52" s="15" t="n"/>
+      <c r="D52" s="15" t="n"/>
+      <c r="E52" s="15" t="n"/>
+      <c r="F52" s="15">
+        <f>IF(C52="","",C52-B52-E52)</f>
+        <v/>
+      </c>
+      <c r="G52" s="16">
+        <f>IF(OR(C52="",B52="",(B52+E52)=0),"",(C52-B52-E52)/(B52+E52))</f>
+        <v/>
+      </c>
+      <c r="H52" s="15" t="n"/>
+      <c r="I52" s="15" t="n"/>
+      <c r="J52" s="15" t="n"/>
+      <c r="K52" s="15">
+        <f>IF(H52="","",H52-C52-J52)</f>
+        <v/>
+      </c>
+      <c r="L52" s="16">
+        <f>IF(OR(H52="",C52="",(C52+J52)=0),"",(H52-C52-J52)/(C52+J52))</f>
+        <v/>
+      </c>
+      <c r="M52" s="15" t="n"/>
+      <c r="N52" s="15" t="n"/>
+      <c r="O52" s="15" t="n"/>
+      <c r="P52" s="15">
+        <f>IF(M52="","",M52-H52-O52)</f>
+        <v/>
+      </c>
+      <c r="Q52" s="16">
+        <f>IF(OR(M52="",H52="",(H52+O52)=0),"",(M52-H52-O52)/(H52+O52))</f>
+        <v/>
+      </c>
+      <c r="R52" s="15" t="n"/>
+      <c r="S52" s="15" t="n"/>
+      <c r="T52" s="15" t="n"/>
+      <c r="U52" s="15">
+        <f>IF(R52="","",R52-M52-T52)</f>
+        <v/>
+      </c>
+      <c r="V52" s="16">
+        <f>IF(OR(R52="",M52="",(M52+T52)=0),"",(R52-M52-T52)/(M52+T52))</f>
+        <v/>
+      </c>
+      <c r="W52" s="15" t="n"/>
+      <c r="X52" s="15" t="n"/>
+      <c r="Y52" s="15" t="n"/>
+      <c r="Z52" s="15">
+        <f>IF(W52="","",W52-R52-Y52)</f>
+        <v/>
+      </c>
+      <c r="AA52" s="16">
+        <f>IF(OR(W52="",R52="",(R52+Y52)=0),"",(W52-R52-Y52)/(R52+Y52))</f>
+        <v/>
+      </c>
+      <c r="AB52" s="15" t="n"/>
+      <c r="AC52" s="15" t="n"/>
+      <c r="AD52" s="15" t="n"/>
+      <c r="AE52" s="15">
+        <f>IF(AB52="","",AB52-W52-AD52)</f>
+        <v/>
+      </c>
+      <c r="AF52" s="16">
+        <f>IF(OR(AB52="",W52="",(W52+AD52)=0),"",(AB52-W52-AD52)/(W52+AD52))</f>
+        <v/>
+      </c>
+      <c r="AG52" s="15" t="n"/>
+      <c r="AH52" s="15" t="n"/>
+      <c r="AI52" s="15" t="n"/>
+      <c r="AJ52" s="15">
+        <f>IF(AG52="","",AG52-AB52-AI52)</f>
+        <v/>
+      </c>
+      <c r="AK52" s="16">
+        <f>IF(OR(AG52="",AB52="",(AB52+AI52)=0),"",(AG52-AB52-AI52)/(AB52+AI52))</f>
+        <v/>
+      </c>
+      <c r="AL52" s="15" t="n"/>
+      <c r="AM52" s="15" t="n"/>
+      <c r="AN52" s="15" t="n"/>
+      <c r="AO52" s="15">
+        <f>IF(AL52="","",AL52-AG52-AN52)</f>
+        <v/>
+      </c>
+      <c r="AP52" s="16">
+        <f>IF(OR(AL52="",AG52="",(AG52+AN52)=0),"",(AL52-AG52-AN52)/(AG52+AN52))</f>
+        <v/>
+      </c>
+      <c r="AQ52" s="15" t="n"/>
+      <c r="AR52" s="15" t="n"/>
+      <c r="AS52" s="15" t="n"/>
+      <c r="AT52" s="15">
+        <f>IF(AQ52="","",AQ52-AL52-AS52)</f>
+        <v/>
+      </c>
+      <c r="AU52" s="16">
+        <f>IF(OR(AQ52="",AL52="",(AL52+AS52)=0),"",(AQ52-AL52-AS52)/(AL52+AS52))</f>
+        <v/>
+      </c>
+      <c r="AV52" s="15" t="n"/>
+      <c r="AW52" s="15" t="n"/>
+      <c r="AX52" s="15" t="n"/>
+      <c r="AY52" s="15">
+        <f>IF(AV52="","",AV52-AQ52-AX52)</f>
+        <v/>
+      </c>
+      <c r="AZ52" s="16">
+        <f>IF(OR(AV52="",AQ52="",(AQ52+AX52)=0),"",(AV52-AQ52-AX52)/(AQ52+AX52))</f>
+        <v/>
+      </c>
+      <c r="BA52" s="15" t="n"/>
+      <c r="BB52" s="15" t="n"/>
+      <c r="BC52" s="15" t="n"/>
+      <c r="BD52" s="15">
+        <f>IF(BA52="","",BA52-AV52-BC52)</f>
+        <v/>
+      </c>
+      <c r="BE52" s="16">
+        <f>IF(OR(BA52="",AV52="",(AV52+BC52)=0),"",(BA52-AV52-BC52)/(AV52+BC52))</f>
+        <v/>
+      </c>
+      <c r="BF52" s="15" t="n"/>
+      <c r="BG52" s="15" t="n"/>
+      <c r="BH52" s="15" t="n"/>
+      <c r="BI52" s="15">
+        <f>IF(BF52="","",BF52-BA52-BH52)</f>
+        <v/>
+      </c>
+      <c r="BJ52" s="16">
+        <f>IF(OR(BF52="",BA52="",(BA52+BH52)=0),"",(BF52-BA52-BH52)/(BA52+BH52))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="24" customHeight="1">
+      <c r="A55" s="26" t="inlineStr">
         <is>
           <t>RESUMO – EVOLUÇÃO DO PATRIMÔNIO</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="30" customHeight="1">
-      <c r="A49" s="26" t="inlineStr">
+    <row r="56" ht="30" customHeight="1">
+      <c r="A56" s="27" t="inlineStr">
         <is>
           <t>Mês</t>
         </is>
       </c>
-      <c r="B49" s="26" t="inlineStr">
+      <c r="B56" s="27" t="inlineStr">
         <is>
           <t>Patrimônio Bruto</t>
         </is>
       </c>
-      <c r="C49" s="26" t="inlineStr">
+      <c r="C56" s="27" t="inlineStr">
         <is>
           <t>Patrimônio Líquido</t>
         </is>
       </c>
-      <c r="D49" s="26" t="inlineStr">
+      <c r="D56" s="27" t="inlineStr">
         <is>
           <t>Rentab. Mensal (R$)</t>
         </is>
       </c>
-      <c r="E49" s="26" t="inlineStr">
+      <c r="E56" s="27" t="inlineStr">
         <is>
           <t>Rentab. Mensal (%)</t>
         </is>
       </c>
-      <c r="F49" s="26" t="inlineStr">
+      <c r="F56" s="27" t="inlineStr">
         <is>
           <t>Rentab. Acum. (%)</t>
         </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="27" t="inlineStr">
-        <is>
-          <t>jan/26</t>
-        </is>
-      </c>
-      <c r="B50" s="28">
-        <f>IF(C8="","",C8)</f>
-        <v/>
-      </c>
-      <c r="C50" s="28">
-        <f>IF(D8="","",D8)</f>
-        <v/>
-      </c>
-      <c r="D50" s="28">
-        <f>IF(F8="","",F8)</f>
-        <v/>
-      </c>
-      <c r="E50" s="29">
-        <f>IF(G8="","",G8)</f>
-        <v/>
-      </c>
-      <c r="F50" s="30">
-        <f>IF(E50="","",E50)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="31" t="inlineStr">
-        <is>
-          <t>fev/26</t>
-        </is>
-      </c>
-      <c r="B51" s="32">
-        <f>IF(H8="","",H8)</f>
-        <v/>
-      </c>
-      <c r="C51" s="32">
-        <f>IF(I8="","",I8)</f>
-        <v/>
-      </c>
-      <c r="D51" s="32">
-        <f>IF(K8="","",K8)</f>
-        <v/>
-      </c>
-      <c r="E51" s="33">
-        <f>IF(L8="","",L8)</f>
-        <v/>
-      </c>
-      <c r="F51" s="34">
-        <f>IF(E51="",F50,IF(F50="",E51,(1+F50)*(1+E51)-1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="27" t="inlineStr">
-        <is>
-          <t>mar/26</t>
-        </is>
-      </c>
-      <c r="B52" s="28">
-        <f>IF(M8="","",M8)</f>
-        <v/>
-      </c>
-      <c r="C52" s="28">
-        <f>IF(N8="","",N8)</f>
-        <v/>
-      </c>
-      <c r="D52" s="28">
-        <f>IF(P8="","",P8)</f>
-        <v/>
-      </c>
-      <c r="E52" s="29">
-        <f>IF(Q8="","",Q8)</f>
-        <v/>
-      </c>
-      <c r="F52" s="30">
-        <f>IF(E52="",F51,IF(F51="",E52,(1+F51)*(1+E52)-1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="31" t="inlineStr">
-        <is>
-          <t>abr/26</t>
-        </is>
-      </c>
-      <c r="B53" s="32">
-        <f>IF(R8="","",R8)</f>
-        <v/>
-      </c>
-      <c r="C53" s="32">
-        <f>IF(S8="","",S8)</f>
-        <v/>
-      </c>
-      <c r="D53" s="32">
-        <f>IF(U8="","",U8)</f>
-        <v/>
-      </c>
-      <c r="E53" s="33">
-        <f>IF(V8="","",V8)</f>
-        <v/>
-      </c>
-      <c r="F53" s="34">
-        <f>IF(E53="",F52,IF(F52="",E53,(1+F52)*(1+E53)-1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="27" t="inlineStr">
-        <is>
-          <t>mai/26</t>
-        </is>
-      </c>
-      <c r="B54" s="28">
-        <f>IF(W8="","",W8)</f>
-        <v/>
-      </c>
-      <c r="C54" s="28">
-        <f>IF(X8="","",X8)</f>
-        <v/>
-      </c>
-      <c r="D54" s="28">
-        <f>IF(Z8="","",Z8)</f>
-        <v/>
-      </c>
-      <c r="E54" s="29">
-        <f>IF(AA8="","",AA8)</f>
-        <v/>
-      </c>
-      <c r="F54" s="30">
-        <f>IF(E54="",F53,IF(F53="",E54,(1+F53)*(1+E54)-1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="31" t="inlineStr">
-        <is>
-          <t>jun/26</t>
-        </is>
-      </c>
-      <c r="B55" s="32">
-        <f>IF(AB8="","",AB8)</f>
-        <v/>
-      </c>
-      <c r="C55" s="32">
-        <f>IF(AC8="","",AC8)</f>
-        <v/>
-      </c>
-      <c r="D55" s="32">
-        <f>IF(AE8="","",AE8)</f>
-        <v/>
-      </c>
-      <c r="E55" s="33">
-        <f>IF(AF8="","",AF8)</f>
-        <v/>
-      </c>
-      <c r="F55" s="34">
-        <f>IF(E55="",F54,IF(F54="",E55,(1+F54)*(1+E55)-1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="27" t="inlineStr">
-        <is>
-          <t>jul/26</t>
-        </is>
-      </c>
-      <c r="B56" s="28">
-        <f>IF(AG8="","",AG8)</f>
-        <v/>
-      </c>
-      <c r="C56" s="28">
-        <f>IF(AH8="","",AH8)</f>
-        <v/>
-      </c>
-      <c r="D56" s="28">
-        <f>IF(AJ8="","",AJ8)</f>
-        <v/>
-      </c>
-      <c r="E56" s="29">
-        <f>IF(AK8="","",AK8)</f>
-        <v/>
-      </c>
-      <c r="F56" s="30">
-        <f>IF(E56="",F55,IF(F55="",E56,(1+F55)*(1+E56)-1))</f>
-        <v/>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="31" t="inlineStr">
-        <is>
-          <t>ago/26</t>
-        </is>
-      </c>
-      <c r="B57" s="32">
-        <f>IF(AL8="","",AL8)</f>
-        <v/>
-      </c>
-      <c r="C57" s="32">
-        <f>IF(AM8="","",AM8)</f>
-        <v/>
-      </c>
-      <c r="D57" s="32">
-        <f>IF(AO8="","",AO8)</f>
-        <v/>
-      </c>
-      <c r="E57" s="33">
-        <f>IF(AP8="","",AP8)</f>
-        <v/>
-      </c>
-      <c r="F57" s="34">
-        <f>IF(E57="",F56,IF(F56="",E57,(1+F56)*(1+E57)-1))</f>
+      <c r="A57" s="28" t="inlineStr">
+        <is>
+          <t>jan/26</t>
+        </is>
+      </c>
+      <c r="B57" s="29">
+        <f>IF(C8="","",C8)</f>
+        <v/>
+      </c>
+      <c r="C57" s="29">
+        <f>IF(D8="","",D8)</f>
+        <v/>
+      </c>
+      <c r="D57" s="29">
+        <f>IF(F8="","",F8)</f>
+        <v/>
+      </c>
+      <c r="E57" s="30">
+        <f>IF(G8="","",G8)</f>
+        <v/>
+      </c>
+      <c r="F57" s="31">
+        <f>IF(E57="","",E57)</f>
         <v/>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="27" t="inlineStr">
-        <is>
-          <t>set/26</t>
-        </is>
-      </c>
-      <c r="B58" s="28">
-        <f>IF(AQ8="","",AQ8)</f>
-        <v/>
-      </c>
-      <c r="C58" s="28">
-        <f>IF(AR8="","",AR8)</f>
-        <v/>
-      </c>
-      <c r="D58" s="28">
-        <f>IF(AT8="","",AT8)</f>
-        <v/>
-      </c>
-      <c r="E58" s="29">
-        <f>IF(AU8="","",AU8)</f>
-        <v/>
-      </c>
-      <c r="F58" s="30">
+      <c r="A58" s="32" t="inlineStr">
+        <is>
+          <t>fev/26</t>
+        </is>
+      </c>
+      <c r="B58" s="33">
+        <f>IF(H8="","",H8)</f>
+        <v/>
+      </c>
+      <c r="C58" s="33">
+        <f>IF(I8="","",I8)</f>
+        <v/>
+      </c>
+      <c r="D58" s="33">
+        <f>IF(K8="","",K8)</f>
+        <v/>
+      </c>
+      <c r="E58" s="34">
+        <f>IF(L8="","",L8)</f>
+        <v/>
+      </c>
+      <c r="F58" s="35">
         <f>IF(E58="",F57,IF(F57="",E58,(1+F57)*(1+E58)-1))</f>
         <v/>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="31" t="inlineStr">
-        <is>
-          <t>out/26</t>
-        </is>
-      </c>
-      <c r="B59" s="32">
-        <f>IF(AV8="","",AV8)</f>
-        <v/>
-      </c>
-      <c r="C59" s="32">
-        <f>IF(AW8="","",AW8)</f>
-        <v/>
-      </c>
-      <c r="D59" s="32">
-        <f>IF(AY8="","",AY8)</f>
-        <v/>
-      </c>
-      <c r="E59" s="33">
-        <f>IF(AZ8="","",AZ8)</f>
-        <v/>
-      </c>
-      <c r="F59" s="34">
+      <c r="A59" s="28" t="inlineStr">
+        <is>
+          <t>mar/26</t>
+        </is>
+      </c>
+      <c r="B59" s="29">
+        <f>IF(M8="","",M8)</f>
+        <v/>
+      </c>
+      <c r="C59" s="29">
+        <f>IF(N8="","",N8)</f>
+        <v/>
+      </c>
+      <c r="D59" s="29">
+        <f>IF(P8="","",P8)</f>
+        <v/>
+      </c>
+      <c r="E59" s="30">
+        <f>IF(Q8="","",Q8)</f>
+        <v/>
+      </c>
+      <c r="F59" s="31">
         <f>IF(E59="",F58,IF(F58="",E59,(1+F58)*(1+E59)-1))</f>
         <v/>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="27" t="inlineStr">
-        <is>
-          <t>nov/26</t>
-        </is>
-      </c>
-      <c r="B60" s="28">
-        <f>IF(BA8="","",BA8)</f>
-        <v/>
-      </c>
-      <c r="C60" s="28">
-        <f>IF(BB8="","",BB8)</f>
-        <v/>
-      </c>
-      <c r="D60" s="28">
-        <f>IF(BD8="","",BD8)</f>
-        <v/>
-      </c>
-      <c r="E60" s="29">
-        <f>IF(BE8="","",BE8)</f>
-        <v/>
-      </c>
-      <c r="F60" s="30">
+      <c r="A60" s="32" t="inlineStr">
+        <is>
+          <t>abr/26</t>
+        </is>
+      </c>
+      <c r="B60" s="33">
+        <f>IF(R8="","",R8)</f>
+        <v/>
+      </c>
+      <c r="C60" s="33">
+        <f>IF(S8="","",S8)</f>
+        <v/>
+      </c>
+      <c r="D60" s="33">
+        <f>IF(U8="","",U8)</f>
+        <v/>
+      </c>
+      <c r="E60" s="34">
+        <f>IF(V8="","",V8)</f>
+        <v/>
+      </c>
+      <c r="F60" s="35">
         <f>IF(E60="",F59,IF(F59="",E60,(1+F59)*(1+E60)-1))</f>
         <v/>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="31" t="inlineStr">
+      <c r="A61" s="28" t="inlineStr">
+        <is>
+          <t>mai/26</t>
+        </is>
+      </c>
+      <c r="B61" s="29">
+        <f>IF(W8="","",W8)</f>
+        <v/>
+      </c>
+      <c r="C61" s="29">
+        <f>IF(X8="","",X8)</f>
+        <v/>
+      </c>
+      <c r="D61" s="29">
+        <f>IF(Z8="","",Z8)</f>
+        <v/>
+      </c>
+      <c r="E61" s="30">
+        <f>IF(AA8="","",AA8)</f>
+        <v/>
+      </c>
+      <c r="F61" s="31">
+        <f>IF(E61="",F60,IF(F60="",E61,(1+F60)*(1+E61)-1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="32" t="inlineStr">
+        <is>
+          <t>jun/26</t>
+        </is>
+      </c>
+      <c r="B62" s="33">
+        <f>IF(AB8="","",AB8)</f>
+        <v/>
+      </c>
+      <c r="C62" s="33">
+        <f>IF(AC8="","",AC8)</f>
+        <v/>
+      </c>
+      <c r="D62" s="33">
+        <f>IF(AE8="","",AE8)</f>
+        <v/>
+      </c>
+      <c r="E62" s="34">
+        <f>IF(AF8="","",AF8)</f>
+        <v/>
+      </c>
+      <c r="F62" s="35">
+        <f>IF(E62="",F61,IF(F61="",E62,(1+F61)*(1+E62)-1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="28" t="inlineStr">
+        <is>
+          <t>jul/26</t>
+        </is>
+      </c>
+      <c r="B63" s="29">
+        <f>IF(AG8="","",AG8)</f>
+        <v/>
+      </c>
+      <c r="C63" s="29">
+        <f>IF(AH8="","",AH8)</f>
+        <v/>
+      </c>
+      <c r="D63" s="29">
+        <f>IF(AJ8="","",AJ8)</f>
+        <v/>
+      </c>
+      <c r="E63" s="30">
+        <f>IF(AK8="","",AK8)</f>
+        <v/>
+      </c>
+      <c r="F63" s="31">
+        <f>IF(E63="",F62,IF(F62="",E63,(1+F62)*(1+E63)-1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="32" t="inlineStr">
+        <is>
+          <t>ago/26</t>
+        </is>
+      </c>
+      <c r="B64" s="33">
+        <f>IF(AL8="","",AL8)</f>
+        <v/>
+      </c>
+      <c r="C64" s="33">
+        <f>IF(AM8="","",AM8)</f>
+        <v/>
+      </c>
+      <c r="D64" s="33">
+        <f>IF(AO8="","",AO8)</f>
+        <v/>
+      </c>
+      <c r="E64" s="34">
+        <f>IF(AP8="","",AP8)</f>
+        <v/>
+      </c>
+      <c r="F64" s="35">
+        <f>IF(E64="",F63,IF(F63="",E64,(1+F63)*(1+E64)-1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="28" t="inlineStr">
+        <is>
+          <t>set/26</t>
+        </is>
+      </c>
+      <c r="B65" s="29">
+        <f>IF(AQ8="","",AQ8)</f>
+        <v/>
+      </c>
+      <c r="C65" s="29">
+        <f>IF(AR8="","",AR8)</f>
+        <v/>
+      </c>
+      <c r="D65" s="29">
+        <f>IF(AT8="","",AT8)</f>
+        <v/>
+      </c>
+      <c r="E65" s="30">
+        <f>IF(AU8="","",AU8)</f>
+        <v/>
+      </c>
+      <c r="F65" s="31">
+        <f>IF(E65="",F64,IF(F64="",E65,(1+F64)*(1+E65)-1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="32" t="inlineStr">
+        <is>
+          <t>out/26</t>
+        </is>
+      </c>
+      <c r="B66" s="33">
+        <f>IF(AV8="","",AV8)</f>
+        <v/>
+      </c>
+      <c r="C66" s="33">
+        <f>IF(AW8="","",AW8)</f>
+        <v/>
+      </c>
+      <c r="D66" s="33">
+        <f>IF(AY8="","",AY8)</f>
+        <v/>
+      </c>
+      <c r="E66" s="34">
+        <f>IF(AZ8="","",AZ8)</f>
+        <v/>
+      </c>
+      <c r="F66" s="35">
+        <f>IF(E66="",F65,IF(F65="",E66,(1+F65)*(1+E66)-1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="28" t="inlineStr">
+        <is>
+          <t>nov/26</t>
+        </is>
+      </c>
+      <c r="B67" s="29">
+        <f>IF(BA8="","",BA8)</f>
+        <v/>
+      </c>
+      <c r="C67" s="29">
+        <f>IF(BB8="","",BB8)</f>
+        <v/>
+      </c>
+      <c r="D67" s="29">
+        <f>IF(BD8="","",BD8)</f>
+        <v/>
+      </c>
+      <c r="E67" s="30">
+        <f>IF(BE8="","",BE8)</f>
+        <v/>
+      </c>
+      <c r="F67" s="31">
+        <f>IF(E67="",F66,IF(F66="",E67,(1+F66)*(1+E67)-1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="32" t="inlineStr">
         <is>
           <t>dez/26</t>
         </is>
       </c>
-      <c r="B61" s="32">
+      <c r="B68" s="33">
         <f>IF(BF8="","",BF8)</f>
         <v/>
       </c>
-      <c r="C61" s="32">
+      <c r="C68" s="33">
         <f>IF(BG8="","",BG8)</f>
         <v/>
       </c>
-      <c r="D61" s="32">
+      <c r="D68" s="33">
         <f>IF(BI8="","",BI8)</f>
         <v/>
       </c>
-      <c r="E61" s="33">
+      <c r="E68" s="34">
         <f>IF(BJ8="","",BJ8)</f>
         <v/>
       </c>
-      <c r="F61" s="34">
-        <f>IF(E61="",F60,IF(F60="",E61,(1+F60)*(1+E61)-1))</f>
+      <c r="F68" s="35">
+        <f>IF(E68="",F67,IF(F67="",E68,(1+F67)*(1+E68)-1))</f>
         <v/>
       </c>
     </row>
@@ -7807,6 +8882,7 @@
     <mergeCell ref="W6:AA6"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="BF6:BJ6"/>
+    <mergeCell ref="A55:F55"/>
     <mergeCell ref="AG6:AK6"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="H6:L6"/>
@@ -7815,141 +8891,140 @@
     <mergeCell ref="A1:BJ1"/>
     <mergeCell ref="M6:Q6"/>
     <mergeCell ref="BA6:BE6"/>
-    <mergeCell ref="A48:F48"/>
     <mergeCell ref="AV6:AZ6"/>
     <mergeCell ref="AQ6:AU6"/>
   </mergeCells>
-  <conditionalFormatting sqref="F8:F45">
+  <conditionalFormatting sqref="F8:F52">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G8:G45">
+  <conditionalFormatting sqref="G8:G52">
     <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K8:K45">
+  <conditionalFormatting sqref="K8:K52">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L8:L45">
+  <conditionalFormatting sqref="L8:L52">
     <cfRule type="cellIs" priority="4" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P8:P45">
+  <conditionalFormatting sqref="P8:P52">
     <cfRule type="cellIs" priority="5" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q8:Q45">
+  <conditionalFormatting sqref="Q8:Q52">
     <cfRule type="cellIs" priority="6" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U8:U45">
+  <conditionalFormatting sqref="U8:U52">
     <cfRule type="cellIs" priority="7" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V8:V45">
+  <conditionalFormatting sqref="V8:V52">
     <cfRule type="cellIs" priority="8" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Z8:Z45">
+  <conditionalFormatting sqref="Z8:Z52">
     <cfRule type="cellIs" priority="9" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AA8:AA45">
+  <conditionalFormatting sqref="AA8:AA52">
     <cfRule type="cellIs" priority="10" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AE8:AE45">
+  <conditionalFormatting sqref="AE8:AE52">
     <cfRule type="cellIs" priority="11" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AF8:AF45">
+  <conditionalFormatting sqref="AF8:AF52">
     <cfRule type="cellIs" priority="12" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AJ8:AJ45">
+  <conditionalFormatting sqref="AJ8:AJ52">
     <cfRule type="cellIs" priority="13" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AK8:AK45">
+  <conditionalFormatting sqref="AK8:AK52">
     <cfRule type="cellIs" priority="14" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AO8:AO45">
+  <conditionalFormatting sqref="AO8:AO52">
     <cfRule type="cellIs" priority="15" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AP8:AP45">
+  <conditionalFormatting sqref="AP8:AP52">
     <cfRule type="cellIs" priority="16" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AT8:AT45">
+  <conditionalFormatting sqref="AT8:AT52">
     <cfRule type="cellIs" priority="17" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AU8:AU45">
+  <conditionalFormatting sqref="AU8:AU52">
     <cfRule type="cellIs" priority="18" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AY8:AY45">
+  <conditionalFormatting sqref="AY8:AY52">
     <cfRule type="cellIs" priority="19" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AZ8:AZ45">
+  <conditionalFormatting sqref="AZ8:AZ52">
     <cfRule type="cellIs" priority="20" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="BD8:BD45">
+  <conditionalFormatting sqref="BD8:BD52">
     <cfRule type="cellIs" priority="21" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="BE8:BE45">
+  <conditionalFormatting sqref="BE8:BE52">
     <cfRule type="cellIs" priority="22" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="BI8:BI45">
+  <conditionalFormatting sqref="BI8:BI52">
     <cfRule type="cellIs" priority="23" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="BJ8:BJ45">
+  <conditionalFormatting sqref="BJ8:BJ52">
     <cfRule type="cellIs" priority="24" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D50:D61">
+  <conditionalFormatting sqref="D57:D68">
     <cfRule type="cellIs" priority="25" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E50:E61">
+  <conditionalFormatting sqref="E57:E68">
     <cfRule type="cellIs" priority="26" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F50:F61">
+  <conditionalFormatting sqref="F57:F68">
     <cfRule type="cellIs" priority="27" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -7972,139 +9047,139 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="35" t="inlineStr">
+      <c r="A1" s="36" t="inlineStr">
         <is>
           <t>COMO USAR ESTA PLANILHA</t>
         </is>
       </c>
     </row>
     <row r="2" ht="19" customHeight="1">
-      <c r="A2" s="36" t="inlineStr"/>
+      <c r="A2" s="37" t="inlineStr"/>
     </row>
     <row r="3" ht="19" customHeight="1">
-      <c r="A3" s="37" t="inlineStr">
+      <c r="A3" s="38" t="inlineStr">
         <is>
           <t>1. Preencha o nome do cliente, o assessor e o período no topo da aba 'Acompanhamento Mensal'.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="19" customHeight="1">
-      <c r="A4" s="36" t="inlineStr"/>
+      <c r="A4" s="37" t="inlineStr"/>
     </row>
     <row r="5" ht="19" customHeight="1">
-      <c r="A5" s="37" t="inlineStr">
+      <c r="A5" s="38" t="inlineStr">
         <is>
           <t>2. Para cada classe, digite o nome dos ativos nas linhas em branco (coluna CLASSE / ATIVO).</t>
         </is>
       </c>
     </row>
     <row r="6" ht="19" customHeight="1">
-      <c r="A6" s="36" t="inlineStr"/>
+      <c r="A6" s="37" t="inlineStr"/>
     </row>
     <row r="7" ht="19" customHeight="1">
-      <c r="A7" s="37" t="inlineStr">
+      <c r="A7" s="38" t="inlineStr">
         <is>
           <t>3. Em cada mês preencha apenas 3 colunas por ativo:</t>
         </is>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1">
-      <c r="A8" s="36" t="inlineStr">
+      <c r="A8" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">     • Valor Bruto      – valor de mercado antes de impostos.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1">
-      <c r="A9" s="36" t="inlineStr">
+      <c r="A9" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">     • Valor Líquido    – valor já descontado o IR no resgate.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1">
-      <c r="A10" s="36" t="inlineStr">
+      <c r="A10" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">                          (em investimentos ISENTOS, repita o valor bruto)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1">
-      <c r="A11" s="36" t="inlineStr">
+      <c r="A11" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">     • Movimentação     – aportes com sinal +  e  resgates com sinal −  (deixe vazio se não houve).</t>
         </is>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1">
-      <c r="A12" s="36" t="inlineStr"/>
+      <c r="A12" s="37" t="inlineStr"/>
     </row>
     <row r="13" ht="19" customHeight="1">
-      <c r="A13" s="37" t="inlineStr">
+      <c r="A13" s="38" t="inlineStr">
         <is>
           <t>4. As colunas Rentabilidade (R$) e Rentabilidade (%) são calculadas automaticamente:</t>
         </is>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1">
-      <c r="A14" s="36" t="inlineStr">
+      <c r="A14" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">     Rentab. R$ = Valor Bruto do mês − Valor Bruto do mês anterior − Movimentação.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1">
-      <c r="A15" s="36" t="inlineStr">
+      <c r="A15" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">     Assim, aportes e resgates NÃO são contados como rendimento.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1">
-      <c r="A16" s="36" t="inlineStr"/>
+      <c r="A16" s="37" t="inlineStr"/>
     </row>
     <row r="17" ht="19" customHeight="1">
-      <c r="A17" s="37" t="inlineStr">
+      <c r="A17" s="38" t="inlineStr">
         <is>
           <t>5. A coluna 'Saldo Inicial (Bruto)' é a base do 1º mês. Preencha-a com o valor antes do período acompanhado.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1">
-      <c r="A18" s="36" t="inlineStr"/>
+      <c r="A18" s="37" t="inlineStr"/>
     </row>
     <row r="19" ht="19" customHeight="1">
-      <c r="A19" s="37" t="inlineStr">
+      <c r="A19" s="38" t="inlineStr">
         <is>
           <t>6. As linhas de classe e a linha PATRIMÔNIO TOTAL somam tudo sozinhas — não digite nada nelas.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1">
-      <c r="A20" s="36" t="inlineStr"/>
+      <c r="A20" s="37" t="inlineStr"/>
     </row>
     <row r="21" ht="19" customHeight="1">
-      <c r="A21" s="37" t="inlineStr">
+      <c r="A21" s="38" t="inlineStr">
         <is>
           <t>7. Use os botões [-] / [+] à esquerda das linhas para recolher ou expandir os ativos de cada classe.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="19" customHeight="1">
-      <c r="A22" s="36" t="inlineStr"/>
+      <c r="A22" s="37" t="inlineStr"/>
     </row>
     <row r="23" ht="19" customHeight="1">
-      <c r="A23" s="37" t="inlineStr">
+      <c r="A23" s="38" t="inlineStr">
         <is>
           <t>8. O bloco RESUMO e os gráficos no fim da aba se atualizam sozinhos e podem ser usados no envio ao cliente.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="19" customHeight="1">
-      <c r="A24" s="36" t="inlineStr"/>
+      <c r="A24" s="37" t="inlineStr"/>
     </row>
     <row r="25" ht="19" customHeight="1">
-      <c r="A25" s="36" t="inlineStr">
+      <c r="A25" s="37" t="inlineStr">
         <is>
           <t>Observação: a diferença entre Valor Bruto e Valor Líquido mostra ao cliente quanto o IR impacta o resgate. Em produtos isentos (LCI, LCA, CRI, CRA, debêntures incentivadas, poupança) os dois valores são iguais.</t>
         </is>

</xml_diff>

<commit_message>
Corrige erro #VALOR! na coluna Rentabilidade (%)
A fórmula somava o saldo anterior e a movimentação dentro do OR(),
gerando #VALOR! quando uma dessas células retornava texto vazio "".
Agora a movimentação é tratada com N() e o cálculo só ocorre após a
verificação de células preenchidas.

https://claude.ai/code/session_012B6pvzwHHmCv3nAgYhFWdt
</commit_message>
<xml_diff>
--- a/acompanhamento_mensal.xlsx
+++ b/acompanhamento_mensal.xlsx
@@ -1496,7 +1496,7 @@
         <v/>
       </c>
       <c r="G8" s="10">
-        <f>IF(OR(C8="",B8="",(B8+E8)=0),"",(C8-B8-E8)/(B8+E8))</f>
+        <f>IF(OR(C8="",B8=""),"",IF((B8+N(E8))=0,"",(C8-B8-N(E8))/(B8+N(E8))))</f>
         <v/>
       </c>
       <c r="H8" s="9">
@@ -1516,7 +1516,7 @@
         <v/>
       </c>
       <c r="L8" s="10">
-        <f>IF(OR(H8="",C8="",(C8+J8)=0),"",(H8-C8-J8)/(C8+J8))</f>
+        <f>IF(OR(H8="",C8=""),"",IF((C8+N(J8))=0,"",(H8-C8-N(J8))/(C8+N(J8))))</f>
         <v/>
       </c>
       <c r="M8" s="9">
@@ -1536,7 +1536,7 @@
         <v/>
       </c>
       <c r="Q8" s="10">
-        <f>IF(OR(M8="",H8="",(H8+O8)=0),"",(M8-H8-O8)/(H8+O8))</f>
+        <f>IF(OR(M8="",H8=""),"",IF((H8+N(O8))=0,"",(M8-H8-N(O8))/(H8+N(O8))))</f>
         <v/>
       </c>
       <c r="R8" s="9">
@@ -1556,7 +1556,7 @@
         <v/>
       </c>
       <c r="V8" s="10">
-        <f>IF(OR(R8="",M8="",(M8+T8)=0),"",(R8-M8-T8)/(M8+T8))</f>
+        <f>IF(OR(R8="",M8=""),"",IF((M8+N(T8))=0,"",(R8-M8-N(T8))/(M8+N(T8))))</f>
         <v/>
       </c>
       <c r="W8" s="9">
@@ -1576,7 +1576,7 @@
         <v/>
       </c>
       <c r="AA8" s="10">
-        <f>IF(OR(W8="",R8="",(R8+Y8)=0),"",(W8-R8-Y8)/(R8+Y8))</f>
+        <f>IF(OR(W8="",R8=""),"",IF((R8+N(Y8))=0,"",(W8-R8-N(Y8))/(R8+N(Y8))))</f>
         <v/>
       </c>
       <c r="AB8" s="9">
@@ -1596,7 +1596,7 @@
         <v/>
       </c>
       <c r="AF8" s="10">
-        <f>IF(OR(AB8="",W8="",(W8+AD8)=0),"",(AB8-W8-AD8)/(W8+AD8))</f>
+        <f>IF(OR(AB8="",W8=""),"",IF((W8+N(AD8))=0,"",(AB8-W8-N(AD8))/(W8+N(AD8))))</f>
         <v/>
       </c>
       <c r="AG8" s="9">
@@ -1616,7 +1616,7 @@
         <v/>
       </c>
       <c r="AK8" s="10">
-        <f>IF(OR(AG8="",AB8="",(AB8+AI8)=0),"",(AG8-AB8-AI8)/(AB8+AI8))</f>
+        <f>IF(OR(AG8="",AB8=""),"",IF((AB8+N(AI8))=0,"",(AG8-AB8-N(AI8))/(AB8+N(AI8))))</f>
         <v/>
       </c>
       <c r="AL8" s="9">
@@ -1636,7 +1636,7 @@
         <v/>
       </c>
       <c r="AP8" s="10">
-        <f>IF(OR(AL8="",AG8="",(AG8+AN8)=0),"",(AL8-AG8-AN8)/(AG8+AN8))</f>
+        <f>IF(OR(AL8="",AG8=""),"",IF((AG8+N(AN8))=0,"",(AL8-AG8-N(AN8))/(AG8+N(AN8))))</f>
         <v/>
       </c>
       <c r="AQ8" s="9">
@@ -1656,7 +1656,7 @@
         <v/>
       </c>
       <c r="AU8" s="10">
-        <f>IF(OR(AQ8="",AL8="",(AL8+AS8)=0),"",(AQ8-AL8-AS8)/(AL8+AS8))</f>
+        <f>IF(OR(AQ8="",AL8=""),"",IF((AL8+N(AS8))=0,"",(AQ8-AL8-N(AS8))/(AL8+N(AS8))))</f>
         <v/>
       </c>
       <c r="AV8" s="9">
@@ -1676,7 +1676,7 @@
         <v/>
       </c>
       <c r="AZ8" s="10">
-        <f>IF(OR(AV8="",AQ8="",(AQ8+AX8)=0),"",(AV8-AQ8-AX8)/(AQ8+AX8))</f>
+        <f>IF(OR(AV8="",AQ8=""),"",IF((AQ8+N(AX8))=0,"",(AV8-AQ8-N(AX8))/(AQ8+N(AX8))))</f>
         <v/>
       </c>
       <c r="BA8" s="9">
@@ -1696,7 +1696,7 @@
         <v/>
       </c>
       <c r="BE8" s="10">
-        <f>IF(OR(BA8="",AV8="",(AV8+BC8)=0),"",(BA8-AV8-BC8)/(AV8+BC8))</f>
+        <f>IF(OR(BA8="",AV8=""),"",IF((AV8+N(BC8))=0,"",(BA8-AV8-N(BC8))/(AV8+N(BC8))))</f>
         <v/>
       </c>
       <c r="BF8" s="9">
@@ -1716,7 +1716,7 @@
         <v/>
       </c>
       <c r="BJ8" s="10">
-        <f>IF(OR(BF8="",BA8="",(BA8+BH8)=0),"",(BF8-BA8-BH8)/(BA8+BH8))</f>
+        <f>IF(OR(BF8="",BA8=""),"",IF((BA8+N(BH8))=0,"",(BF8-BA8-N(BH8))/(BA8+N(BH8))))</f>
         <v/>
       </c>
     </row>
@@ -1747,7 +1747,7 @@
         <v/>
       </c>
       <c r="G9" s="13">
-        <f>IF(OR(C9="",B9="",(B9+E9)=0),"",(C9-B9-E9)/(B9+E9))</f>
+        <f>IF(OR(C9="",B9=""),"",IF((B9+N(E9))=0,"",(C9-B9-N(E9))/(B9+N(E9))))</f>
         <v/>
       </c>
       <c r="H9" s="12">
@@ -1767,7 +1767,7 @@
         <v/>
       </c>
       <c r="L9" s="13">
-        <f>IF(OR(H9="",C9="",(C9+J9)=0),"",(H9-C9-J9)/(C9+J9))</f>
+        <f>IF(OR(H9="",C9=""),"",IF((C9+N(J9))=0,"",(H9-C9-N(J9))/(C9+N(J9))))</f>
         <v/>
       </c>
       <c r="M9" s="12">
@@ -1787,7 +1787,7 @@
         <v/>
       </c>
       <c r="Q9" s="13">
-        <f>IF(OR(M9="",H9="",(H9+O9)=0),"",(M9-H9-O9)/(H9+O9))</f>
+        <f>IF(OR(M9="",H9=""),"",IF((H9+N(O9))=0,"",(M9-H9-N(O9))/(H9+N(O9))))</f>
         <v/>
       </c>
       <c r="R9" s="12">
@@ -1807,7 +1807,7 @@
         <v/>
       </c>
       <c r="V9" s="13">
-        <f>IF(OR(R9="",M9="",(M9+T9)=0),"",(R9-M9-T9)/(M9+T9))</f>
+        <f>IF(OR(R9="",M9=""),"",IF((M9+N(T9))=0,"",(R9-M9-N(T9))/(M9+N(T9))))</f>
         <v/>
       </c>
       <c r="W9" s="12">
@@ -1827,7 +1827,7 @@
         <v/>
       </c>
       <c r="AA9" s="13">
-        <f>IF(OR(W9="",R9="",(R9+Y9)=0),"",(W9-R9-Y9)/(R9+Y9))</f>
+        <f>IF(OR(W9="",R9=""),"",IF((R9+N(Y9))=0,"",(W9-R9-N(Y9))/(R9+N(Y9))))</f>
         <v/>
       </c>
       <c r="AB9" s="12">
@@ -1847,7 +1847,7 @@
         <v/>
       </c>
       <c r="AF9" s="13">
-        <f>IF(OR(AB9="",W9="",(W9+AD9)=0),"",(AB9-W9-AD9)/(W9+AD9))</f>
+        <f>IF(OR(AB9="",W9=""),"",IF((W9+N(AD9))=0,"",(AB9-W9-N(AD9))/(W9+N(AD9))))</f>
         <v/>
       </c>
       <c r="AG9" s="12">
@@ -1867,7 +1867,7 @@
         <v/>
       </c>
       <c r="AK9" s="13">
-        <f>IF(OR(AG9="",AB9="",(AB9+AI9)=0),"",(AG9-AB9-AI9)/(AB9+AI9))</f>
+        <f>IF(OR(AG9="",AB9=""),"",IF((AB9+N(AI9))=0,"",(AG9-AB9-N(AI9))/(AB9+N(AI9))))</f>
         <v/>
       </c>
       <c r="AL9" s="12">
@@ -1887,7 +1887,7 @@
         <v/>
       </c>
       <c r="AP9" s="13">
-        <f>IF(OR(AL9="",AG9="",(AG9+AN9)=0),"",(AL9-AG9-AN9)/(AG9+AN9))</f>
+        <f>IF(OR(AL9="",AG9=""),"",IF((AG9+N(AN9))=0,"",(AL9-AG9-N(AN9))/(AG9+N(AN9))))</f>
         <v/>
       </c>
       <c r="AQ9" s="12">
@@ -1907,7 +1907,7 @@
         <v/>
       </c>
       <c r="AU9" s="13">
-        <f>IF(OR(AQ9="",AL9="",(AL9+AS9)=0),"",(AQ9-AL9-AS9)/(AL9+AS9))</f>
+        <f>IF(OR(AQ9="",AL9=""),"",IF((AL9+N(AS9))=0,"",(AQ9-AL9-N(AS9))/(AL9+N(AS9))))</f>
         <v/>
       </c>
       <c r="AV9" s="12">
@@ -1927,7 +1927,7 @@
         <v/>
       </c>
       <c r="AZ9" s="13">
-        <f>IF(OR(AV9="",AQ9="",(AQ9+AX9)=0),"",(AV9-AQ9-AX9)/(AQ9+AX9))</f>
+        <f>IF(OR(AV9="",AQ9=""),"",IF((AQ9+N(AX9))=0,"",(AV9-AQ9-N(AX9))/(AQ9+N(AX9))))</f>
         <v/>
       </c>
       <c r="BA9" s="12">
@@ -1947,7 +1947,7 @@
         <v/>
       </c>
       <c r="BE9" s="13">
-        <f>IF(OR(BA9="",AV9="",(AV9+BC9)=0),"",(BA9-AV9-BC9)/(AV9+BC9))</f>
+        <f>IF(OR(BA9="",AV9=""),"",IF((AV9+N(BC9))=0,"",(BA9-AV9-N(BC9))/(AV9+N(BC9))))</f>
         <v/>
       </c>
       <c r="BF9" s="12">
@@ -1967,7 +1967,7 @@
         <v/>
       </c>
       <c r="BJ9" s="13">
-        <f>IF(OR(BF9="",BA9="",(BA9+BH9)=0),"",(BF9-BA9-BH9)/(BA9+BH9))</f>
+        <f>IF(OR(BF9="",BA9=""),"",IF((BA9+N(BH9))=0,"",(BF9-BA9-N(BH9))/(BA9+N(BH9))))</f>
         <v/>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v/>
       </c>
       <c r="G10" s="16">
-        <f>IF(OR(C10="",B10="",(B10+E10)=0),"",(C10-B10-E10)/(B10+E10))</f>
+        <f>IF(OR(C10="",B10=""),"",IF((B10+N(E10))=0,"",(C10-B10-N(E10))/(B10+N(E10))))</f>
         <v/>
       </c>
       <c r="H10" s="15" t="n"/>
@@ -1993,7 +1993,7 @@
         <v/>
       </c>
       <c r="L10" s="16">
-        <f>IF(OR(H10="",C10="",(C10+J10)=0),"",(H10-C10-J10)/(C10+J10))</f>
+        <f>IF(OR(H10="",C10=""),"",IF((C10+N(J10))=0,"",(H10-C10-N(J10))/(C10+N(J10))))</f>
         <v/>
       </c>
       <c r="M10" s="15" t="n"/>
@@ -2004,7 +2004,7 @@
         <v/>
       </c>
       <c r="Q10" s="16">
-        <f>IF(OR(M10="",H10="",(H10+O10)=0),"",(M10-H10-O10)/(H10+O10))</f>
+        <f>IF(OR(M10="",H10=""),"",IF((H10+N(O10))=0,"",(M10-H10-N(O10))/(H10+N(O10))))</f>
         <v/>
       </c>
       <c r="R10" s="15" t="n"/>
@@ -2015,7 +2015,7 @@
         <v/>
       </c>
       <c r="V10" s="16">
-        <f>IF(OR(R10="",M10="",(M10+T10)=0),"",(R10-M10-T10)/(M10+T10))</f>
+        <f>IF(OR(R10="",M10=""),"",IF((M10+N(T10))=0,"",(R10-M10-N(T10))/(M10+N(T10))))</f>
         <v/>
       </c>
       <c r="W10" s="15" t="n"/>
@@ -2026,7 +2026,7 @@
         <v/>
       </c>
       <c r="AA10" s="16">
-        <f>IF(OR(W10="",R10="",(R10+Y10)=0),"",(W10-R10-Y10)/(R10+Y10))</f>
+        <f>IF(OR(W10="",R10=""),"",IF((R10+N(Y10))=0,"",(W10-R10-N(Y10))/(R10+N(Y10))))</f>
         <v/>
       </c>
       <c r="AB10" s="15" t="n"/>
@@ -2037,7 +2037,7 @@
         <v/>
       </c>
       <c r="AF10" s="16">
-        <f>IF(OR(AB10="",W10="",(W10+AD10)=0),"",(AB10-W10-AD10)/(W10+AD10))</f>
+        <f>IF(OR(AB10="",W10=""),"",IF((W10+N(AD10))=0,"",(AB10-W10-N(AD10))/(W10+N(AD10))))</f>
         <v/>
       </c>
       <c r="AG10" s="15" t="n"/>
@@ -2048,7 +2048,7 @@
         <v/>
       </c>
       <c r="AK10" s="16">
-        <f>IF(OR(AG10="",AB10="",(AB10+AI10)=0),"",(AG10-AB10-AI10)/(AB10+AI10))</f>
+        <f>IF(OR(AG10="",AB10=""),"",IF((AB10+N(AI10))=0,"",(AG10-AB10-N(AI10))/(AB10+N(AI10))))</f>
         <v/>
       </c>
       <c r="AL10" s="15" t="n"/>
@@ -2059,7 +2059,7 @@
         <v/>
       </c>
       <c r="AP10" s="16">
-        <f>IF(OR(AL10="",AG10="",(AG10+AN10)=0),"",(AL10-AG10-AN10)/(AG10+AN10))</f>
+        <f>IF(OR(AL10="",AG10=""),"",IF((AG10+N(AN10))=0,"",(AL10-AG10-N(AN10))/(AG10+N(AN10))))</f>
         <v/>
       </c>
       <c r="AQ10" s="15" t="n"/>
@@ -2070,7 +2070,7 @@
         <v/>
       </c>
       <c r="AU10" s="16">
-        <f>IF(OR(AQ10="",AL10="",(AL10+AS10)=0),"",(AQ10-AL10-AS10)/(AL10+AS10))</f>
+        <f>IF(OR(AQ10="",AL10=""),"",IF((AL10+N(AS10))=0,"",(AQ10-AL10-N(AS10))/(AL10+N(AS10))))</f>
         <v/>
       </c>
       <c r="AV10" s="15" t="n"/>
@@ -2081,7 +2081,7 @@
         <v/>
       </c>
       <c r="AZ10" s="16">
-        <f>IF(OR(AV10="",AQ10="",(AQ10+AX10)=0),"",(AV10-AQ10-AX10)/(AQ10+AX10))</f>
+        <f>IF(OR(AV10="",AQ10=""),"",IF((AQ10+N(AX10))=0,"",(AV10-AQ10-N(AX10))/(AQ10+N(AX10))))</f>
         <v/>
       </c>
       <c r="BA10" s="15" t="n"/>
@@ -2092,7 +2092,7 @@
         <v/>
       </c>
       <c r="BE10" s="16">
-        <f>IF(OR(BA10="",AV10="",(AV10+BC10)=0),"",(BA10-AV10-BC10)/(AV10+BC10))</f>
+        <f>IF(OR(BA10="",AV10=""),"",IF((AV10+N(BC10))=0,"",(BA10-AV10-N(BC10))/(AV10+N(BC10))))</f>
         <v/>
       </c>
       <c r="BF10" s="15" t="n"/>
@@ -2103,7 +2103,7 @@
         <v/>
       </c>
       <c r="BJ10" s="16">
-        <f>IF(OR(BF10="",BA10="",(BA10+BH10)=0),"",(BF10-BA10-BH10)/(BA10+BH10))</f>
+        <f>IF(OR(BF10="",BA10=""),"",IF((BA10+N(BH10))=0,"",(BF10-BA10-N(BH10))/(BA10+N(BH10))))</f>
         <v/>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
         <v/>
       </c>
       <c r="G11" s="19">
-        <f>IF(OR(C11="",B11="",(B11+E11)=0),"",(C11-B11-E11)/(B11+E11))</f>
+        <f>IF(OR(C11="",B11=""),"",IF((B11+N(E11))=0,"",(C11-B11-N(E11))/(B11+N(E11))))</f>
         <v/>
       </c>
       <c r="H11" s="18" t="n"/>
@@ -2129,7 +2129,7 @@
         <v/>
       </c>
       <c r="L11" s="19">
-        <f>IF(OR(H11="",C11="",(C11+J11)=0),"",(H11-C11-J11)/(C11+J11))</f>
+        <f>IF(OR(H11="",C11=""),"",IF((C11+N(J11))=0,"",(H11-C11-N(J11))/(C11+N(J11))))</f>
         <v/>
       </c>
       <c r="M11" s="18" t="n"/>
@@ -2140,7 +2140,7 @@
         <v/>
       </c>
       <c r="Q11" s="19">
-        <f>IF(OR(M11="",H11="",(H11+O11)=0),"",(M11-H11-O11)/(H11+O11))</f>
+        <f>IF(OR(M11="",H11=""),"",IF((H11+N(O11))=0,"",(M11-H11-N(O11))/(H11+N(O11))))</f>
         <v/>
       </c>
       <c r="R11" s="18" t="n"/>
@@ -2151,7 +2151,7 @@
         <v/>
       </c>
       <c r="V11" s="19">
-        <f>IF(OR(R11="",M11="",(M11+T11)=0),"",(R11-M11-T11)/(M11+T11))</f>
+        <f>IF(OR(R11="",M11=""),"",IF((M11+N(T11))=0,"",(R11-M11-N(T11))/(M11+N(T11))))</f>
         <v/>
       </c>
       <c r="W11" s="18" t="n"/>
@@ -2162,7 +2162,7 @@
         <v/>
       </c>
       <c r="AA11" s="19">
-        <f>IF(OR(W11="",R11="",(R11+Y11)=0),"",(W11-R11-Y11)/(R11+Y11))</f>
+        <f>IF(OR(W11="",R11=""),"",IF((R11+N(Y11))=0,"",(W11-R11-N(Y11))/(R11+N(Y11))))</f>
         <v/>
       </c>
       <c r="AB11" s="18" t="n"/>
@@ -2173,7 +2173,7 @@
         <v/>
       </c>
       <c r="AF11" s="19">
-        <f>IF(OR(AB11="",W11="",(W11+AD11)=0),"",(AB11-W11-AD11)/(W11+AD11))</f>
+        <f>IF(OR(AB11="",W11=""),"",IF((W11+N(AD11))=0,"",(AB11-W11-N(AD11))/(W11+N(AD11))))</f>
         <v/>
       </c>
       <c r="AG11" s="18" t="n"/>
@@ -2184,7 +2184,7 @@
         <v/>
       </c>
       <c r="AK11" s="19">
-        <f>IF(OR(AG11="",AB11="",(AB11+AI11)=0),"",(AG11-AB11-AI11)/(AB11+AI11))</f>
+        <f>IF(OR(AG11="",AB11=""),"",IF((AB11+N(AI11))=0,"",(AG11-AB11-N(AI11))/(AB11+N(AI11))))</f>
         <v/>
       </c>
       <c r="AL11" s="18" t="n"/>
@@ -2195,7 +2195,7 @@
         <v/>
       </c>
       <c r="AP11" s="19">
-        <f>IF(OR(AL11="",AG11="",(AG11+AN11)=0),"",(AL11-AG11-AN11)/(AG11+AN11))</f>
+        <f>IF(OR(AL11="",AG11=""),"",IF((AG11+N(AN11))=0,"",(AL11-AG11-N(AN11))/(AG11+N(AN11))))</f>
         <v/>
       </c>
       <c r="AQ11" s="18" t="n"/>
@@ -2206,7 +2206,7 @@
         <v/>
       </c>
       <c r="AU11" s="19">
-        <f>IF(OR(AQ11="",AL11="",(AL11+AS11)=0),"",(AQ11-AL11-AS11)/(AL11+AS11))</f>
+        <f>IF(OR(AQ11="",AL11=""),"",IF((AL11+N(AS11))=0,"",(AQ11-AL11-N(AS11))/(AL11+N(AS11))))</f>
         <v/>
       </c>
       <c r="AV11" s="18" t="n"/>
@@ -2217,7 +2217,7 @@
         <v/>
       </c>
       <c r="AZ11" s="19">
-        <f>IF(OR(AV11="",AQ11="",(AQ11+AX11)=0),"",(AV11-AQ11-AX11)/(AQ11+AX11))</f>
+        <f>IF(OR(AV11="",AQ11=""),"",IF((AQ11+N(AX11))=0,"",(AV11-AQ11-N(AX11))/(AQ11+N(AX11))))</f>
         <v/>
       </c>
       <c r="BA11" s="18" t="n"/>
@@ -2228,7 +2228,7 @@
         <v/>
       </c>
       <c r="BE11" s="19">
-        <f>IF(OR(BA11="",AV11="",(AV11+BC11)=0),"",(BA11-AV11-BC11)/(AV11+BC11))</f>
+        <f>IF(OR(BA11="",AV11=""),"",IF((AV11+N(BC11))=0,"",(BA11-AV11-N(BC11))/(AV11+N(BC11))))</f>
         <v/>
       </c>
       <c r="BF11" s="18" t="n"/>
@@ -2239,7 +2239,7 @@
         <v/>
       </c>
       <c r="BJ11" s="19">
-        <f>IF(OR(BF11="",BA11="",(BA11+BH11)=0),"",(BF11-BA11-BH11)/(BA11+BH11))</f>
+        <f>IF(OR(BF11="",BA11=""),"",IF((BA11+N(BH11))=0,"",(BF11-BA11-N(BH11))/(BA11+N(BH11))))</f>
         <v/>
       </c>
     </row>
@@ -2254,7 +2254,7 @@
         <v/>
       </c>
       <c r="G12" s="16">
-        <f>IF(OR(C12="",B12="",(B12+E12)=0),"",(C12-B12-E12)/(B12+E12))</f>
+        <f>IF(OR(C12="",B12=""),"",IF((B12+N(E12))=0,"",(C12-B12-N(E12))/(B12+N(E12))))</f>
         <v/>
       </c>
       <c r="H12" s="15" t="n"/>
@@ -2265,7 +2265,7 @@
         <v/>
       </c>
       <c r="L12" s="16">
-        <f>IF(OR(H12="",C12="",(C12+J12)=0),"",(H12-C12-J12)/(C12+J12))</f>
+        <f>IF(OR(H12="",C12=""),"",IF((C12+N(J12))=0,"",(H12-C12-N(J12))/(C12+N(J12))))</f>
         <v/>
       </c>
       <c r="M12" s="15" t="n"/>
@@ -2276,7 +2276,7 @@
         <v/>
       </c>
       <c r="Q12" s="16">
-        <f>IF(OR(M12="",H12="",(H12+O12)=0),"",(M12-H12-O12)/(H12+O12))</f>
+        <f>IF(OR(M12="",H12=""),"",IF((H12+N(O12))=0,"",(M12-H12-N(O12))/(H12+N(O12))))</f>
         <v/>
       </c>
       <c r="R12" s="15" t="n"/>
@@ -2287,7 +2287,7 @@
         <v/>
       </c>
       <c r="V12" s="16">
-        <f>IF(OR(R12="",M12="",(M12+T12)=0),"",(R12-M12-T12)/(M12+T12))</f>
+        <f>IF(OR(R12="",M12=""),"",IF((M12+N(T12))=0,"",(R12-M12-N(T12))/(M12+N(T12))))</f>
         <v/>
       </c>
       <c r="W12" s="15" t="n"/>
@@ -2298,7 +2298,7 @@
         <v/>
       </c>
       <c r="AA12" s="16">
-        <f>IF(OR(W12="",R12="",(R12+Y12)=0),"",(W12-R12-Y12)/(R12+Y12))</f>
+        <f>IF(OR(W12="",R12=""),"",IF((R12+N(Y12))=0,"",(W12-R12-N(Y12))/(R12+N(Y12))))</f>
         <v/>
       </c>
       <c r="AB12" s="15" t="n"/>
@@ -2309,7 +2309,7 @@
         <v/>
       </c>
       <c r="AF12" s="16">
-        <f>IF(OR(AB12="",W12="",(W12+AD12)=0),"",(AB12-W12-AD12)/(W12+AD12))</f>
+        <f>IF(OR(AB12="",W12=""),"",IF((W12+N(AD12))=0,"",(AB12-W12-N(AD12))/(W12+N(AD12))))</f>
         <v/>
       </c>
       <c r="AG12" s="15" t="n"/>
@@ -2320,7 +2320,7 @@
         <v/>
       </c>
       <c r="AK12" s="16">
-        <f>IF(OR(AG12="",AB12="",(AB12+AI12)=0),"",(AG12-AB12-AI12)/(AB12+AI12))</f>
+        <f>IF(OR(AG12="",AB12=""),"",IF((AB12+N(AI12))=0,"",(AG12-AB12-N(AI12))/(AB12+N(AI12))))</f>
         <v/>
       </c>
       <c r="AL12" s="15" t="n"/>
@@ -2331,7 +2331,7 @@
         <v/>
       </c>
       <c r="AP12" s="16">
-        <f>IF(OR(AL12="",AG12="",(AG12+AN12)=0),"",(AL12-AG12-AN12)/(AG12+AN12))</f>
+        <f>IF(OR(AL12="",AG12=""),"",IF((AG12+N(AN12))=0,"",(AL12-AG12-N(AN12))/(AG12+N(AN12))))</f>
         <v/>
       </c>
       <c r="AQ12" s="15" t="n"/>
@@ -2342,7 +2342,7 @@
         <v/>
       </c>
       <c r="AU12" s="16">
-        <f>IF(OR(AQ12="",AL12="",(AL12+AS12)=0),"",(AQ12-AL12-AS12)/(AL12+AS12))</f>
+        <f>IF(OR(AQ12="",AL12=""),"",IF((AL12+N(AS12))=0,"",(AQ12-AL12-N(AS12))/(AL12+N(AS12))))</f>
         <v/>
       </c>
       <c r="AV12" s="15" t="n"/>
@@ -2353,7 +2353,7 @@
         <v/>
       </c>
       <c r="AZ12" s="16">
-        <f>IF(OR(AV12="",AQ12="",(AQ12+AX12)=0),"",(AV12-AQ12-AX12)/(AQ12+AX12))</f>
+        <f>IF(OR(AV12="",AQ12=""),"",IF((AQ12+N(AX12))=0,"",(AV12-AQ12-N(AX12))/(AQ12+N(AX12))))</f>
         <v/>
       </c>
       <c r="BA12" s="15" t="n"/>
@@ -2364,7 +2364,7 @@
         <v/>
       </c>
       <c r="BE12" s="16">
-        <f>IF(OR(BA12="",AV12="",(AV12+BC12)=0),"",(BA12-AV12-BC12)/(AV12+BC12))</f>
+        <f>IF(OR(BA12="",AV12=""),"",IF((AV12+N(BC12))=0,"",(BA12-AV12-N(BC12))/(AV12+N(BC12))))</f>
         <v/>
       </c>
       <c r="BF12" s="15" t="n"/>
@@ -2375,7 +2375,7 @@
         <v/>
       </c>
       <c r="BJ12" s="16">
-        <f>IF(OR(BF12="",BA12="",(BA12+BH12)=0),"",(BF12-BA12-BH12)/(BA12+BH12))</f>
+        <f>IF(OR(BF12="",BA12=""),"",IF((BA12+N(BH12))=0,"",(BF12-BA12-N(BH12))/(BA12+N(BH12))))</f>
         <v/>
       </c>
     </row>
@@ -2390,7 +2390,7 @@
         <v/>
       </c>
       <c r="G13" s="19">
-        <f>IF(OR(C13="",B13="",(B13+E13)=0),"",(C13-B13-E13)/(B13+E13))</f>
+        <f>IF(OR(C13="",B13=""),"",IF((B13+N(E13))=0,"",(C13-B13-N(E13))/(B13+N(E13))))</f>
         <v/>
       </c>
       <c r="H13" s="18" t="n"/>
@@ -2401,7 +2401,7 @@
         <v/>
       </c>
       <c r="L13" s="19">
-        <f>IF(OR(H13="",C13="",(C13+J13)=0),"",(H13-C13-J13)/(C13+J13))</f>
+        <f>IF(OR(H13="",C13=""),"",IF((C13+N(J13))=0,"",(H13-C13-N(J13))/(C13+N(J13))))</f>
         <v/>
       </c>
       <c r="M13" s="18" t="n"/>
@@ -2412,7 +2412,7 @@
         <v/>
       </c>
       <c r="Q13" s="19">
-        <f>IF(OR(M13="",H13="",(H13+O13)=0),"",(M13-H13-O13)/(H13+O13))</f>
+        <f>IF(OR(M13="",H13=""),"",IF((H13+N(O13))=0,"",(M13-H13-N(O13))/(H13+N(O13))))</f>
         <v/>
       </c>
       <c r="R13" s="18" t="n"/>
@@ -2423,7 +2423,7 @@
         <v/>
       </c>
       <c r="V13" s="19">
-        <f>IF(OR(R13="",M13="",(M13+T13)=0),"",(R13-M13-T13)/(M13+T13))</f>
+        <f>IF(OR(R13="",M13=""),"",IF((M13+N(T13))=0,"",(R13-M13-N(T13))/(M13+N(T13))))</f>
         <v/>
       </c>
       <c r="W13" s="18" t="n"/>
@@ -2434,7 +2434,7 @@
         <v/>
       </c>
       <c r="AA13" s="19">
-        <f>IF(OR(W13="",R13="",(R13+Y13)=0),"",(W13-R13-Y13)/(R13+Y13))</f>
+        <f>IF(OR(W13="",R13=""),"",IF((R13+N(Y13))=0,"",(W13-R13-N(Y13))/(R13+N(Y13))))</f>
         <v/>
       </c>
       <c r="AB13" s="18" t="n"/>
@@ -2445,7 +2445,7 @@
         <v/>
       </c>
       <c r="AF13" s="19">
-        <f>IF(OR(AB13="",W13="",(W13+AD13)=0),"",(AB13-W13-AD13)/(W13+AD13))</f>
+        <f>IF(OR(AB13="",W13=""),"",IF((W13+N(AD13))=0,"",(AB13-W13-N(AD13))/(W13+N(AD13))))</f>
         <v/>
       </c>
       <c r="AG13" s="18" t="n"/>
@@ -2456,7 +2456,7 @@
         <v/>
       </c>
       <c r="AK13" s="19">
-        <f>IF(OR(AG13="",AB13="",(AB13+AI13)=0),"",(AG13-AB13-AI13)/(AB13+AI13))</f>
+        <f>IF(OR(AG13="",AB13=""),"",IF((AB13+N(AI13))=0,"",(AG13-AB13-N(AI13))/(AB13+N(AI13))))</f>
         <v/>
       </c>
       <c r="AL13" s="18" t="n"/>
@@ -2467,7 +2467,7 @@
         <v/>
       </c>
       <c r="AP13" s="19">
-        <f>IF(OR(AL13="",AG13="",(AG13+AN13)=0),"",(AL13-AG13-AN13)/(AG13+AN13))</f>
+        <f>IF(OR(AL13="",AG13=""),"",IF((AG13+N(AN13))=0,"",(AL13-AG13-N(AN13))/(AG13+N(AN13))))</f>
         <v/>
       </c>
       <c r="AQ13" s="18" t="n"/>
@@ -2478,7 +2478,7 @@
         <v/>
       </c>
       <c r="AU13" s="19">
-        <f>IF(OR(AQ13="",AL13="",(AL13+AS13)=0),"",(AQ13-AL13-AS13)/(AL13+AS13))</f>
+        <f>IF(OR(AQ13="",AL13=""),"",IF((AL13+N(AS13))=0,"",(AQ13-AL13-N(AS13))/(AL13+N(AS13))))</f>
         <v/>
       </c>
       <c r="AV13" s="18" t="n"/>
@@ -2489,7 +2489,7 @@
         <v/>
       </c>
       <c r="AZ13" s="19">
-        <f>IF(OR(AV13="",AQ13="",(AQ13+AX13)=0),"",(AV13-AQ13-AX13)/(AQ13+AX13))</f>
+        <f>IF(OR(AV13="",AQ13=""),"",IF((AQ13+N(AX13))=0,"",(AV13-AQ13-N(AX13))/(AQ13+N(AX13))))</f>
         <v/>
       </c>
       <c r="BA13" s="18" t="n"/>
@@ -2500,7 +2500,7 @@
         <v/>
       </c>
       <c r="BE13" s="19">
-        <f>IF(OR(BA13="",AV13="",(AV13+BC13)=0),"",(BA13-AV13-BC13)/(AV13+BC13))</f>
+        <f>IF(OR(BA13="",AV13=""),"",IF((AV13+N(BC13))=0,"",(BA13-AV13-N(BC13))/(AV13+N(BC13))))</f>
         <v/>
       </c>
       <c r="BF13" s="18" t="n"/>
@@ -2511,7 +2511,7 @@
         <v/>
       </c>
       <c r="BJ13" s="19">
-        <f>IF(OR(BF13="",BA13="",(BA13+BH13)=0),"",(BF13-BA13-BH13)/(BA13+BH13))</f>
+        <f>IF(OR(BF13="",BA13=""),"",IF((BA13+N(BH13))=0,"",(BF13-BA13-N(BH13))/(BA13+N(BH13))))</f>
         <v/>
       </c>
     </row>
@@ -2526,7 +2526,7 @@
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IF(OR(C14="",B14="",(B14+E14)=0),"",(C14-B14-E14)/(B14+E14))</f>
+        <f>IF(OR(C14="",B14=""),"",IF((B14+N(E14))=0,"",(C14-B14-N(E14))/(B14+N(E14))))</f>
         <v/>
       </c>
       <c r="H14" s="15" t="n"/>
@@ -2537,7 +2537,7 @@
         <v/>
       </c>
       <c r="L14" s="16">
-        <f>IF(OR(H14="",C14="",(C14+J14)=0),"",(H14-C14-J14)/(C14+J14))</f>
+        <f>IF(OR(H14="",C14=""),"",IF((C14+N(J14))=0,"",(H14-C14-N(J14))/(C14+N(J14))))</f>
         <v/>
       </c>
       <c r="M14" s="15" t="n"/>
@@ -2548,7 +2548,7 @@
         <v/>
       </c>
       <c r="Q14" s="16">
-        <f>IF(OR(M14="",H14="",(H14+O14)=0),"",(M14-H14-O14)/(H14+O14))</f>
+        <f>IF(OR(M14="",H14=""),"",IF((H14+N(O14))=0,"",(M14-H14-N(O14))/(H14+N(O14))))</f>
         <v/>
       </c>
       <c r="R14" s="15" t="n"/>
@@ -2559,7 +2559,7 @@
         <v/>
       </c>
       <c r="V14" s="16">
-        <f>IF(OR(R14="",M14="",(M14+T14)=0),"",(R14-M14-T14)/(M14+T14))</f>
+        <f>IF(OR(R14="",M14=""),"",IF((M14+N(T14))=0,"",(R14-M14-N(T14))/(M14+N(T14))))</f>
         <v/>
       </c>
       <c r="W14" s="15" t="n"/>
@@ -2570,7 +2570,7 @@
         <v/>
       </c>
       <c r="AA14" s="16">
-        <f>IF(OR(W14="",R14="",(R14+Y14)=0),"",(W14-R14-Y14)/(R14+Y14))</f>
+        <f>IF(OR(W14="",R14=""),"",IF((R14+N(Y14))=0,"",(W14-R14-N(Y14))/(R14+N(Y14))))</f>
         <v/>
       </c>
       <c r="AB14" s="15" t="n"/>
@@ -2581,7 +2581,7 @@
         <v/>
       </c>
       <c r="AF14" s="16">
-        <f>IF(OR(AB14="",W14="",(W14+AD14)=0),"",(AB14-W14-AD14)/(W14+AD14))</f>
+        <f>IF(OR(AB14="",W14=""),"",IF((W14+N(AD14))=0,"",(AB14-W14-N(AD14))/(W14+N(AD14))))</f>
         <v/>
       </c>
       <c r="AG14" s="15" t="n"/>
@@ -2592,7 +2592,7 @@
         <v/>
       </c>
       <c r="AK14" s="16">
-        <f>IF(OR(AG14="",AB14="",(AB14+AI14)=0),"",(AG14-AB14-AI14)/(AB14+AI14))</f>
+        <f>IF(OR(AG14="",AB14=""),"",IF((AB14+N(AI14))=0,"",(AG14-AB14-N(AI14))/(AB14+N(AI14))))</f>
         <v/>
       </c>
       <c r="AL14" s="15" t="n"/>
@@ -2603,7 +2603,7 @@
         <v/>
       </c>
       <c r="AP14" s="16">
-        <f>IF(OR(AL14="",AG14="",(AG14+AN14)=0),"",(AL14-AG14-AN14)/(AG14+AN14))</f>
+        <f>IF(OR(AL14="",AG14=""),"",IF((AG14+N(AN14))=0,"",(AL14-AG14-N(AN14))/(AG14+N(AN14))))</f>
         <v/>
       </c>
       <c r="AQ14" s="15" t="n"/>
@@ -2614,7 +2614,7 @@
         <v/>
       </c>
       <c r="AU14" s="16">
-        <f>IF(OR(AQ14="",AL14="",(AL14+AS14)=0),"",(AQ14-AL14-AS14)/(AL14+AS14))</f>
+        <f>IF(OR(AQ14="",AL14=""),"",IF((AL14+N(AS14))=0,"",(AQ14-AL14-N(AS14))/(AL14+N(AS14))))</f>
         <v/>
       </c>
       <c r="AV14" s="15" t="n"/>
@@ -2625,7 +2625,7 @@
         <v/>
       </c>
       <c r="AZ14" s="16">
-        <f>IF(OR(AV14="",AQ14="",(AQ14+AX14)=0),"",(AV14-AQ14-AX14)/(AQ14+AX14))</f>
+        <f>IF(OR(AV14="",AQ14=""),"",IF((AQ14+N(AX14))=0,"",(AV14-AQ14-N(AX14))/(AQ14+N(AX14))))</f>
         <v/>
       </c>
       <c r="BA14" s="15" t="n"/>
@@ -2636,7 +2636,7 @@
         <v/>
       </c>
       <c r="BE14" s="16">
-        <f>IF(OR(BA14="",AV14="",(AV14+BC14)=0),"",(BA14-AV14-BC14)/(AV14+BC14))</f>
+        <f>IF(OR(BA14="",AV14=""),"",IF((AV14+N(BC14))=0,"",(BA14-AV14-N(BC14))/(AV14+N(BC14))))</f>
         <v/>
       </c>
       <c r="BF14" s="15" t="n"/>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="BJ14" s="16">
-        <f>IF(OR(BF14="",BA14="",(BA14+BH14)=0),"",(BF14-BA14-BH14)/(BA14+BH14))</f>
+        <f>IF(OR(BF14="",BA14=""),"",IF((BA14+N(BH14))=0,"",(BF14-BA14-N(BH14))/(BA14+N(BH14))))</f>
         <v/>
       </c>
     </row>
@@ -2662,7 +2662,7 @@
         <v/>
       </c>
       <c r="G15" s="19">
-        <f>IF(OR(C15="",B15="",(B15+E15)=0),"",(C15-B15-E15)/(B15+E15))</f>
+        <f>IF(OR(C15="",B15=""),"",IF((B15+N(E15))=0,"",(C15-B15-N(E15))/(B15+N(E15))))</f>
         <v/>
       </c>
       <c r="H15" s="18" t="n"/>
@@ -2673,7 +2673,7 @@
         <v/>
       </c>
       <c r="L15" s="19">
-        <f>IF(OR(H15="",C15="",(C15+J15)=0),"",(H15-C15-J15)/(C15+J15))</f>
+        <f>IF(OR(H15="",C15=""),"",IF((C15+N(J15))=0,"",(H15-C15-N(J15))/(C15+N(J15))))</f>
         <v/>
       </c>
       <c r="M15" s="18" t="n"/>
@@ -2684,7 +2684,7 @@
         <v/>
       </c>
       <c r="Q15" s="19">
-        <f>IF(OR(M15="",H15="",(H15+O15)=0),"",(M15-H15-O15)/(H15+O15))</f>
+        <f>IF(OR(M15="",H15=""),"",IF((H15+N(O15))=0,"",(M15-H15-N(O15))/(H15+N(O15))))</f>
         <v/>
       </c>
       <c r="R15" s="18" t="n"/>
@@ -2695,7 +2695,7 @@
         <v/>
       </c>
       <c r="V15" s="19">
-        <f>IF(OR(R15="",M15="",(M15+T15)=0),"",(R15-M15-T15)/(M15+T15))</f>
+        <f>IF(OR(R15="",M15=""),"",IF((M15+N(T15))=0,"",(R15-M15-N(T15))/(M15+N(T15))))</f>
         <v/>
       </c>
       <c r="W15" s="18" t="n"/>
@@ -2706,7 +2706,7 @@
         <v/>
       </c>
       <c r="AA15" s="19">
-        <f>IF(OR(W15="",R15="",(R15+Y15)=0),"",(W15-R15-Y15)/(R15+Y15))</f>
+        <f>IF(OR(W15="",R15=""),"",IF((R15+N(Y15))=0,"",(W15-R15-N(Y15))/(R15+N(Y15))))</f>
         <v/>
       </c>
       <c r="AB15" s="18" t="n"/>
@@ -2717,7 +2717,7 @@
         <v/>
       </c>
       <c r="AF15" s="19">
-        <f>IF(OR(AB15="",W15="",(W15+AD15)=0),"",(AB15-W15-AD15)/(W15+AD15))</f>
+        <f>IF(OR(AB15="",W15=""),"",IF((W15+N(AD15))=0,"",(AB15-W15-N(AD15))/(W15+N(AD15))))</f>
         <v/>
       </c>
       <c r="AG15" s="18" t="n"/>
@@ -2728,7 +2728,7 @@
         <v/>
       </c>
       <c r="AK15" s="19">
-        <f>IF(OR(AG15="",AB15="",(AB15+AI15)=0),"",(AG15-AB15-AI15)/(AB15+AI15))</f>
+        <f>IF(OR(AG15="",AB15=""),"",IF((AB15+N(AI15))=0,"",(AG15-AB15-N(AI15))/(AB15+N(AI15))))</f>
         <v/>
       </c>
       <c r="AL15" s="18" t="n"/>
@@ -2739,7 +2739,7 @@
         <v/>
       </c>
       <c r="AP15" s="19">
-        <f>IF(OR(AL15="",AG15="",(AG15+AN15)=0),"",(AL15-AG15-AN15)/(AG15+AN15))</f>
+        <f>IF(OR(AL15="",AG15=""),"",IF((AG15+N(AN15))=0,"",(AL15-AG15-N(AN15))/(AG15+N(AN15))))</f>
         <v/>
       </c>
       <c r="AQ15" s="18" t="n"/>
@@ -2750,7 +2750,7 @@
         <v/>
       </c>
       <c r="AU15" s="19">
-        <f>IF(OR(AQ15="",AL15="",(AL15+AS15)=0),"",(AQ15-AL15-AS15)/(AL15+AS15))</f>
+        <f>IF(OR(AQ15="",AL15=""),"",IF((AL15+N(AS15))=0,"",(AQ15-AL15-N(AS15))/(AL15+N(AS15))))</f>
         <v/>
       </c>
       <c r="AV15" s="18" t="n"/>
@@ -2761,7 +2761,7 @@
         <v/>
       </c>
       <c r="AZ15" s="19">
-        <f>IF(OR(AV15="",AQ15="",(AQ15+AX15)=0),"",(AV15-AQ15-AX15)/(AQ15+AX15))</f>
+        <f>IF(OR(AV15="",AQ15=""),"",IF((AQ15+N(AX15))=0,"",(AV15-AQ15-N(AX15))/(AQ15+N(AX15))))</f>
         <v/>
       </c>
       <c r="BA15" s="18" t="n"/>
@@ -2772,7 +2772,7 @@
         <v/>
       </c>
       <c r="BE15" s="19">
-        <f>IF(OR(BA15="",AV15="",(AV15+BC15)=0),"",(BA15-AV15-BC15)/(AV15+BC15))</f>
+        <f>IF(OR(BA15="",AV15=""),"",IF((AV15+N(BC15))=0,"",(BA15-AV15-N(BC15))/(AV15+N(BC15))))</f>
         <v/>
       </c>
       <c r="BF15" s="18" t="n"/>
@@ -2783,7 +2783,7 @@
         <v/>
       </c>
       <c r="BJ15" s="19">
-        <f>IF(OR(BF15="",BA15="",(BA15+BH15)=0),"",(BF15-BA15-BH15)/(BA15+BH15))</f>
+        <f>IF(OR(BF15="",BA15=""),"",IF((BA15+N(BH15))=0,"",(BF15-BA15-N(BH15))/(BA15+N(BH15))))</f>
         <v/>
       </c>
     </row>
@@ -2814,7 +2814,7 @@
         <v/>
       </c>
       <c r="G16" s="13">
-        <f>IF(OR(C16="",B16="",(B16+E16)=0),"",(C16-B16-E16)/(B16+E16))</f>
+        <f>IF(OR(C16="",B16=""),"",IF((B16+N(E16))=0,"",(C16-B16-N(E16))/(B16+N(E16))))</f>
         <v/>
       </c>
       <c r="H16" s="12">
@@ -2834,7 +2834,7 @@
         <v/>
       </c>
       <c r="L16" s="13">
-        <f>IF(OR(H16="",C16="",(C16+J16)=0),"",(H16-C16-J16)/(C16+J16))</f>
+        <f>IF(OR(H16="",C16=""),"",IF((C16+N(J16))=0,"",(H16-C16-N(J16))/(C16+N(J16))))</f>
         <v/>
       </c>
       <c r="M16" s="12">
@@ -2854,7 +2854,7 @@
         <v/>
       </c>
       <c r="Q16" s="13">
-        <f>IF(OR(M16="",H16="",(H16+O16)=0),"",(M16-H16-O16)/(H16+O16))</f>
+        <f>IF(OR(M16="",H16=""),"",IF((H16+N(O16))=0,"",(M16-H16-N(O16))/(H16+N(O16))))</f>
         <v/>
       </c>
       <c r="R16" s="12">
@@ -2874,7 +2874,7 @@
         <v/>
       </c>
       <c r="V16" s="13">
-        <f>IF(OR(R16="",M16="",(M16+T16)=0),"",(R16-M16-T16)/(M16+T16))</f>
+        <f>IF(OR(R16="",M16=""),"",IF((M16+N(T16))=0,"",(R16-M16-N(T16))/(M16+N(T16))))</f>
         <v/>
       </c>
       <c r="W16" s="12">
@@ -2894,7 +2894,7 @@
         <v/>
       </c>
       <c r="AA16" s="13">
-        <f>IF(OR(W16="",R16="",(R16+Y16)=0),"",(W16-R16-Y16)/(R16+Y16))</f>
+        <f>IF(OR(W16="",R16=""),"",IF((R16+N(Y16))=0,"",(W16-R16-N(Y16))/(R16+N(Y16))))</f>
         <v/>
       </c>
       <c r="AB16" s="12">
@@ -2914,7 +2914,7 @@
         <v/>
       </c>
       <c r="AF16" s="13">
-        <f>IF(OR(AB16="",W16="",(W16+AD16)=0),"",(AB16-W16-AD16)/(W16+AD16))</f>
+        <f>IF(OR(AB16="",W16=""),"",IF((W16+N(AD16))=0,"",(AB16-W16-N(AD16))/(W16+N(AD16))))</f>
         <v/>
       </c>
       <c r="AG16" s="12">
@@ -2934,7 +2934,7 @@
         <v/>
       </c>
       <c r="AK16" s="13">
-        <f>IF(OR(AG16="",AB16="",(AB16+AI16)=0),"",(AG16-AB16-AI16)/(AB16+AI16))</f>
+        <f>IF(OR(AG16="",AB16=""),"",IF((AB16+N(AI16))=0,"",(AG16-AB16-N(AI16))/(AB16+N(AI16))))</f>
         <v/>
       </c>
       <c r="AL16" s="12">
@@ -2954,7 +2954,7 @@
         <v/>
       </c>
       <c r="AP16" s="13">
-        <f>IF(OR(AL16="",AG16="",(AG16+AN16)=0),"",(AL16-AG16-AN16)/(AG16+AN16))</f>
+        <f>IF(OR(AL16="",AG16=""),"",IF((AG16+N(AN16))=0,"",(AL16-AG16-N(AN16))/(AG16+N(AN16))))</f>
         <v/>
       </c>
       <c r="AQ16" s="12">
@@ -2974,7 +2974,7 @@
         <v/>
       </c>
       <c r="AU16" s="13">
-        <f>IF(OR(AQ16="",AL16="",(AL16+AS16)=0),"",(AQ16-AL16-AS16)/(AL16+AS16))</f>
+        <f>IF(OR(AQ16="",AL16=""),"",IF((AL16+N(AS16))=0,"",(AQ16-AL16-N(AS16))/(AL16+N(AS16))))</f>
         <v/>
       </c>
       <c r="AV16" s="12">
@@ -2994,7 +2994,7 @@
         <v/>
       </c>
       <c r="AZ16" s="13">
-        <f>IF(OR(AV16="",AQ16="",(AQ16+AX16)=0),"",(AV16-AQ16-AX16)/(AQ16+AX16))</f>
+        <f>IF(OR(AV16="",AQ16=""),"",IF((AQ16+N(AX16))=0,"",(AV16-AQ16-N(AX16))/(AQ16+N(AX16))))</f>
         <v/>
       </c>
       <c r="BA16" s="12">
@@ -3014,7 +3014,7 @@
         <v/>
       </c>
       <c r="BE16" s="13">
-        <f>IF(OR(BA16="",AV16="",(AV16+BC16)=0),"",(BA16-AV16-BC16)/(AV16+BC16))</f>
+        <f>IF(OR(BA16="",AV16=""),"",IF((AV16+N(BC16))=0,"",(BA16-AV16-N(BC16))/(AV16+N(BC16))))</f>
         <v/>
       </c>
       <c r="BF16" s="12">
@@ -3034,7 +3034,7 @@
         <v/>
       </c>
       <c r="BJ16" s="13">
-        <f>IF(OR(BF16="",BA16="",(BA16+BH16)=0),"",(BF16-BA16-BH16)/(BA16+BH16))</f>
+        <f>IF(OR(BF16="",BA16=""),"",IF((BA16+N(BH16))=0,"",(BF16-BA16-N(BH16))/(BA16+N(BH16))))</f>
         <v/>
       </c>
     </row>
@@ -3049,7 +3049,7 @@
         <v/>
       </c>
       <c r="G17" s="16">
-        <f>IF(OR(C17="",B17="",(B17+E17)=0),"",(C17-B17-E17)/(B17+E17))</f>
+        <f>IF(OR(C17="",B17=""),"",IF((B17+N(E17))=0,"",(C17-B17-N(E17))/(B17+N(E17))))</f>
         <v/>
       </c>
       <c r="H17" s="15" t="n"/>
@@ -3060,7 +3060,7 @@
         <v/>
       </c>
       <c r="L17" s="16">
-        <f>IF(OR(H17="",C17="",(C17+J17)=0),"",(H17-C17-J17)/(C17+J17))</f>
+        <f>IF(OR(H17="",C17=""),"",IF((C17+N(J17))=0,"",(H17-C17-N(J17))/(C17+N(J17))))</f>
         <v/>
       </c>
       <c r="M17" s="15" t="n"/>
@@ -3071,7 +3071,7 @@
         <v/>
       </c>
       <c r="Q17" s="16">
-        <f>IF(OR(M17="",H17="",(H17+O17)=0),"",(M17-H17-O17)/(H17+O17))</f>
+        <f>IF(OR(M17="",H17=""),"",IF((H17+N(O17))=0,"",(M17-H17-N(O17))/(H17+N(O17))))</f>
         <v/>
       </c>
       <c r="R17" s="15" t="n"/>
@@ -3082,7 +3082,7 @@
         <v/>
       </c>
       <c r="V17" s="16">
-        <f>IF(OR(R17="",M17="",(M17+T17)=0),"",(R17-M17-T17)/(M17+T17))</f>
+        <f>IF(OR(R17="",M17=""),"",IF((M17+N(T17))=0,"",(R17-M17-N(T17))/(M17+N(T17))))</f>
         <v/>
       </c>
       <c r="W17" s="15" t="n"/>
@@ -3093,7 +3093,7 @@
         <v/>
       </c>
       <c r="AA17" s="16">
-        <f>IF(OR(W17="",R17="",(R17+Y17)=0),"",(W17-R17-Y17)/(R17+Y17))</f>
+        <f>IF(OR(W17="",R17=""),"",IF((R17+N(Y17))=0,"",(W17-R17-N(Y17))/(R17+N(Y17))))</f>
         <v/>
       </c>
       <c r="AB17" s="15" t="n"/>
@@ -3104,7 +3104,7 @@
         <v/>
       </c>
       <c r="AF17" s="16">
-        <f>IF(OR(AB17="",W17="",(W17+AD17)=0),"",(AB17-W17-AD17)/(W17+AD17))</f>
+        <f>IF(OR(AB17="",W17=""),"",IF((W17+N(AD17))=0,"",(AB17-W17-N(AD17))/(W17+N(AD17))))</f>
         <v/>
       </c>
       <c r="AG17" s="15" t="n"/>
@@ -3115,7 +3115,7 @@
         <v/>
       </c>
       <c r="AK17" s="16">
-        <f>IF(OR(AG17="",AB17="",(AB17+AI17)=0),"",(AG17-AB17-AI17)/(AB17+AI17))</f>
+        <f>IF(OR(AG17="",AB17=""),"",IF((AB17+N(AI17))=0,"",(AG17-AB17-N(AI17))/(AB17+N(AI17))))</f>
         <v/>
       </c>
       <c r="AL17" s="15" t="n"/>
@@ -3126,7 +3126,7 @@
         <v/>
       </c>
       <c r="AP17" s="16">
-        <f>IF(OR(AL17="",AG17="",(AG17+AN17)=0),"",(AL17-AG17-AN17)/(AG17+AN17))</f>
+        <f>IF(OR(AL17="",AG17=""),"",IF((AG17+N(AN17))=0,"",(AL17-AG17-N(AN17))/(AG17+N(AN17))))</f>
         <v/>
       </c>
       <c r="AQ17" s="15" t="n"/>
@@ -3137,7 +3137,7 @@
         <v/>
       </c>
       <c r="AU17" s="16">
-        <f>IF(OR(AQ17="",AL17="",(AL17+AS17)=0),"",(AQ17-AL17-AS17)/(AL17+AS17))</f>
+        <f>IF(OR(AQ17="",AL17=""),"",IF((AL17+N(AS17))=0,"",(AQ17-AL17-N(AS17))/(AL17+N(AS17))))</f>
         <v/>
       </c>
       <c r="AV17" s="15" t="n"/>
@@ -3148,7 +3148,7 @@
         <v/>
       </c>
       <c r="AZ17" s="16">
-        <f>IF(OR(AV17="",AQ17="",(AQ17+AX17)=0),"",(AV17-AQ17-AX17)/(AQ17+AX17))</f>
+        <f>IF(OR(AV17="",AQ17=""),"",IF((AQ17+N(AX17))=0,"",(AV17-AQ17-N(AX17))/(AQ17+N(AX17))))</f>
         <v/>
       </c>
       <c r="BA17" s="15" t="n"/>
@@ -3159,7 +3159,7 @@
         <v/>
       </c>
       <c r="BE17" s="16">
-        <f>IF(OR(BA17="",AV17="",(AV17+BC17)=0),"",(BA17-AV17-BC17)/(AV17+BC17))</f>
+        <f>IF(OR(BA17="",AV17=""),"",IF((AV17+N(BC17))=0,"",(BA17-AV17-N(BC17))/(AV17+N(BC17))))</f>
         <v/>
       </c>
       <c r="BF17" s="15" t="n"/>
@@ -3170,7 +3170,7 @@
         <v/>
       </c>
       <c r="BJ17" s="16">
-        <f>IF(OR(BF17="",BA17="",(BA17+BH17)=0),"",(BF17-BA17-BH17)/(BA17+BH17))</f>
+        <f>IF(OR(BF17="",BA17=""),"",IF((BA17+N(BH17))=0,"",(BF17-BA17-N(BH17))/(BA17+N(BH17))))</f>
         <v/>
       </c>
     </row>
@@ -3185,7 +3185,7 @@
         <v/>
       </c>
       <c r="G18" s="19">
-        <f>IF(OR(C18="",B18="",(B18+E18)=0),"",(C18-B18-E18)/(B18+E18))</f>
+        <f>IF(OR(C18="",B18=""),"",IF((B18+N(E18))=0,"",(C18-B18-N(E18))/(B18+N(E18))))</f>
         <v/>
       </c>
       <c r="H18" s="18" t="n"/>
@@ -3196,7 +3196,7 @@
         <v/>
       </c>
       <c r="L18" s="19">
-        <f>IF(OR(H18="",C18="",(C18+J18)=0),"",(H18-C18-J18)/(C18+J18))</f>
+        <f>IF(OR(H18="",C18=""),"",IF((C18+N(J18))=0,"",(H18-C18-N(J18))/(C18+N(J18))))</f>
         <v/>
       </c>
       <c r="M18" s="18" t="n"/>
@@ -3207,7 +3207,7 @@
         <v/>
       </c>
       <c r="Q18" s="19">
-        <f>IF(OR(M18="",H18="",(H18+O18)=0),"",(M18-H18-O18)/(H18+O18))</f>
+        <f>IF(OR(M18="",H18=""),"",IF((H18+N(O18))=0,"",(M18-H18-N(O18))/(H18+N(O18))))</f>
         <v/>
       </c>
       <c r="R18" s="18" t="n"/>
@@ -3218,7 +3218,7 @@
         <v/>
       </c>
       <c r="V18" s="19">
-        <f>IF(OR(R18="",M18="",(M18+T18)=0),"",(R18-M18-T18)/(M18+T18))</f>
+        <f>IF(OR(R18="",M18=""),"",IF((M18+N(T18))=0,"",(R18-M18-N(T18))/(M18+N(T18))))</f>
         <v/>
       </c>
       <c r="W18" s="18" t="n"/>
@@ -3229,7 +3229,7 @@
         <v/>
       </c>
       <c r="AA18" s="19">
-        <f>IF(OR(W18="",R18="",(R18+Y18)=0),"",(W18-R18-Y18)/(R18+Y18))</f>
+        <f>IF(OR(W18="",R18=""),"",IF((R18+N(Y18))=0,"",(W18-R18-N(Y18))/(R18+N(Y18))))</f>
         <v/>
       </c>
       <c r="AB18" s="18" t="n"/>
@@ -3240,7 +3240,7 @@
         <v/>
       </c>
       <c r="AF18" s="19">
-        <f>IF(OR(AB18="",W18="",(W18+AD18)=0),"",(AB18-W18-AD18)/(W18+AD18))</f>
+        <f>IF(OR(AB18="",W18=""),"",IF((W18+N(AD18))=0,"",(AB18-W18-N(AD18))/(W18+N(AD18))))</f>
         <v/>
       </c>
       <c r="AG18" s="18" t="n"/>
@@ -3251,7 +3251,7 @@
         <v/>
       </c>
       <c r="AK18" s="19">
-        <f>IF(OR(AG18="",AB18="",(AB18+AI18)=0),"",(AG18-AB18-AI18)/(AB18+AI18))</f>
+        <f>IF(OR(AG18="",AB18=""),"",IF((AB18+N(AI18))=0,"",(AG18-AB18-N(AI18))/(AB18+N(AI18))))</f>
         <v/>
       </c>
       <c r="AL18" s="18" t="n"/>
@@ -3262,7 +3262,7 @@
         <v/>
       </c>
       <c r="AP18" s="19">
-        <f>IF(OR(AL18="",AG18="",(AG18+AN18)=0),"",(AL18-AG18-AN18)/(AG18+AN18))</f>
+        <f>IF(OR(AL18="",AG18=""),"",IF((AG18+N(AN18))=0,"",(AL18-AG18-N(AN18))/(AG18+N(AN18))))</f>
         <v/>
       </c>
       <c r="AQ18" s="18" t="n"/>
@@ -3273,7 +3273,7 @@
         <v/>
       </c>
       <c r="AU18" s="19">
-        <f>IF(OR(AQ18="",AL18="",(AL18+AS18)=0),"",(AQ18-AL18-AS18)/(AL18+AS18))</f>
+        <f>IF(OR(AQ18="",AL18=""),"",IF((AL18+N(AS18))=0,"",(AQ18-AL18-N(AS18))/(AL18+N(AS18))))</f>
         <v/>
       </c>
       <c r="AV18" s="18" t="n"/>
@@ -3284,7 +3284,7 @@
         <v/>
       </c>
       <c r="AZ18" s="19">
-        <f>IF(OR(AV18="",AQ18="",(AQ18+AX18)=0),"",(AV18-AQ18-AX18)/(AQ18+AX18))</f>
+        <f>IF(OR(AV18="",AQ18=""),"",IF((AQ18+N(AX18))=0,"",(AV18-AQ18-N(AX18))/(AQ18+N(AX18))))</f>
         <v/>
       </c>
       <c r="BA18" s="18" t="n"/>
@@ -3295,7 +3295,7 @@
         <v/>
       </c>
       <c r="BE18" s="19">
-        <f>IF(OR(BA18="",AV18="",(AV18+BC18)=0),"",(BA18-AV18-BC18)/(AV18+BC18))</f>
+        <f>IF(OR(BA18="",AV18=""),"",IF((AV18+N(BC18))=0,"",(BA18-AV18-N(BC18))/(AV18+N(BC18))))</f>
         <v/>
       </c>
       <c r="BF18" s="18" t="n"/>
@@ -3306,7 +3306,7 @@
         <v/>
       </c>
       <c r="BJ18" s="19">
-        <f>IF(OR(BF18="",BA18="",(BA18+BH18)=0),"",(BF18-BA18-BH18)/(BA18+BH18))</f>
+        <f>IF(OR(BF18="",BA18=""),"",IF((BA18+N(BH18))=0,"",(BF18-BA18-N(BH18))/(BA18+N(BH18))))</f>
         <v/>
       </c>
     </row>
@@ -3321,7 +3321,7 @@
         <v/>
       </c>
       <c r="G19" s="16">
-        <f>IF(OR(C19="",B19="",(B19+E19)=0),"",(C19-B19-E19)/(B19+E19))</f>
+        <f>IF(OR(C19="",B19=""),"",IF((B19+N(E19))=0,"",(C19-B19-N(E19))/(B19+N(E19))))</f>
         <v/>
       </c>
       <c r="H19" s="15" t="n"/>
@@ -3332,7 +3332,7 @@
         <v/>
       </c>
       <c r="L19" s="16">
-        <f>IF(OR(H19="",C19="",(C19+J19)=0),"",(H19-C19-J19)/(C19+J19))</f>
+        <f>IF(OR(H19="",C19=""),"",IF((C19+N(J19))=0,"",(H19-C19-N(J19))/(C19+N(J19))))</f>
         <v/>
       </c>
       <c r="M19" s="15" t="n"/>
@@ -3343,7 +3343,7 @@
         <v/>
       </c>
       <c r="Q19" s="16">
-        <f>IF(OR(M19="",H19="",(H19+O19)=0),"",(M19-H19-O19)/(H19+O19))</f>
+        <f>IF(OR(M19="",H19=""),"",IF((H19+N(O19))=0,"",(M19-H19-N(O19))/(H19+N(O19))))</f>
         <v/>
       </c>
       <c r="R19" s="15" t="n"/>
@@ -3354,7 +3354,7 @@
         <v/>
       </c>
       <c r="V19" s="16">
-        <f>IF(OR(R19="",M19="",(M19+T19)=0),"",(R19-M19-T19)/(M19+T19))</f>
+        <f>IF(OR(R19="",M19=""),"",IF((M19+N(T19))=0,"",(R19-M19-N(T19))/(M19+N(T19))))</f>
         <v/>
       </c>
       <c r="W19" s="15" t="n"/>
@@ -3365,7 +3365,7 @@
         <v/>
       </c>
       <c r="AA19" s="16">
-        <f>IF(OR(W19="",R19="",(R19+Y19)=0),"",(W19-R19-Y19)/(R19+Y19))</f>
+        <f>IF(OR(W19="",R19=""),"",IF((R19+N(Y19))=0,"",(W19-R19-N(Y19))/(R19+N(Y19))))</f>
         <v/>
       </c>
       <c r="AB19" s="15" t="n"/>
@@ -3376,7 +3376,7 @@
         <v/>
       </c>
       <c r="AF19" s="16">
-        <f>IF(OR(AB19="",W19="",(W19+AD19)=0),"",(AB19-W19-AD19)/(W19+AD19))</f>
+        <f>IF(OR(AB19="",W19=""),"",IF((W19+N(AD19))=0,"",(AB19-W19-N(AD19))/(W19+N(AD19))))</f>
         <v/>
       </c>
       <c r="AG19" s="15" t="n"/>
@@ -3387,7 +3387,7 @@
         <v/>
       </c>
       <c r="AK19" s="16">
-        <f>IF(OR(AG19="",AB19="",(AB19+AI19)=0),"",(AG19-AB19-AI19)/(AB19+AI19))</f>
+        <f>IF(OR(AG19="",AB19=""),"",IF((AB19+N(AI19))=0,"",(AG19-AB19-N(AI19))/(AB19+N(AI19))))</f>
         <v/>
       </c>
       <c r="AL19" s="15" t="n"/>
@@ -3398,7 +3398,7 @@
         <v/>
       </c>
       <c r="AP19" s="16">
-        <f>IF(OR(AL19="",AG19="",(AG19+AN19)=0),"",(AL19-AG19-AN19)/(AG19+AN19))</f>
+        <f>IF(OR(AL19="",AG19=""),"",IF((AG19+N(AN19))=0,"",(AL19-AG19-N(AN19))/(AG19+N(AN19))))</f>
         <v/>
       </c>
       <c r="AQ19" s="15" t="n"/>
@@ -3409,7 +3409,7 @@
         <v/>
       </c>
       <c r="AU19" s="16">
-        <f>IF(OR(AQ19="",AL19="",(AL19+AS19)=0),"",(AQ19-AL19-AS19)/(AL19+AS19))</f>
+        <f>IF(OR(AQ19="",AL19=""),"",IF((AL19+N(AS19))=0,"",(AQ19-AL19-N(AS19))/(AL19+N(AS19))))</f>
         <v/>
       </c>
       <c r="AV19" s="15" t="n"/>
@@ -3420,7 +3420,7 @@
         <v/>
       </c>
       <c r="AZ19" s="16">
-        <f>IF(OR(AV19="",AQ19="",(AQ19+AX19)=0),"",(AV19-AQ19-AX19)/(AQ19+AX19))</f>
+        <f>IF(OR(AV19="",AQ19=""),"",IF((AQ19+N(AX19))=0,"",(AV19-AQ19-N(AX19))/(AQ19+N(AX19))))</f>
         <v/>
       </c>
       <c r="BA19" s="15" t="n"/>
@@ -3431,7 +3431,7 @@
         <v/>
       </c>
       <c r="BE19" s="16">
-        <f>IF(OR(BA19="",AV19="",(AV19+BC19)=0),"",(BA19-AV19-BC19)/(AV19+BC19))</f>
+        <f>IF(OR(BA19="",AV19=""),"",IF((AV19+N(BC19))=0,"",(BA19-AV19-N(BC19))/(AV19+N(BC19))))</f>
         <v/>
       </c>
       <c r="BF19" s="15" t="n"/>
@@ -3442,7 +3442,7 @@
         <v/>
       </c>
       <c r="BJ19" s="16">
-        <f>IF(OR(BF19="",BA19="",(BA19+BH19)=0),"",(BF19-BA19-BH19)/(BA19+BH19))</f>
+        <f>IF(OR(BF19="",BA19=""),"",IF((BA19+N(BH19))=0,"",(BF19-BA19-N(BH19))/(BA19+N(BH19))))</f>
         <v/>
       </c>
     </row>
@@ -3457,7 +3457,7 @@
         <v/>
       </c>
       <c r="G20" s="19">
-        <f>IF(OR(C20="",B20="",(B20+E20)=0),"",(C20-B20-E20)/(B20+E20))</f>
+        <f>IF(OR(C20="",B20=""),"",IF((B20+N(E20))=0,"",(C20-B20-N(E20))/(B20+N(E20))))</f>
         <v/>
       </c>
       <c r="H20" s="18" t="n"/>
@@ -3468,7 +3468,7 @@
         <v/>
       </c>
       <c r="L20" s="19">
-        <f>IF(OR(H20="",C20="",(C20+J20)=0),"",(H20-C20-J20)/(C20+J20))</f>
+        <f>IF(OR(H20="",C20=""),"",IF((C20+N(J20))=0,"",(H20-C20-N(J20))/(C20+N(J20))))</f>
         <v/>
       </c>
       <c r="M20" s="18" t="n"/>
@@ -3479,7 +3479,7 @@
         <v/>
       </c>
       <c r="Q20" s="19">
-        <f>IF(OR(M20="",H20="",(H20+O20)=0),"",(M20-H20-O20)/(H20+O20))</f>
+        <f>IF(OR(M20="",H20=""),"",IF((H20+N(O20))=0,"",(M20-H20-N(O20))/(H20+N(O20))))</f>
         <v/>
       </c>
       <c r="R20" s="18" t="n"/>
@@ -3490,7 +3490,7 @@
         <v/>
       </c>
       <c r="V20" s="19">
-        <f>IF(OR(R20="",M20="",(M20+T20)=0),"",(R20-M20-T20)/(M20+T20))</f>
+        <f>IF(OR(R20="",M20=""),"",IF((M20+N(T20))=0,"",(R20-M20-N(T20))/(M20+N(T20))))</f>
         <v/>
       </c>
       <c r="W20" s="18" t="n"/>
@@ -3501,7 +3501,7 @@
         <v/>
       </c>
       <c r="AA20" s="19">
-        <f>IF(OR(W20="",R20="",(R20+Y20)=0),"",(W20-R20-Y20)/(R20+Y20))</f>
+        <f>IF(OR(W20="",R20=""),"",IF((R20+N(Y20))=0,"",(W20-R20-N(Y20))/(R20+N(Y20))))</f>
         <v/>
       </c>
       <c r="AB20" s="18" t="n"/>
@@ -3512,7 +3512,7 @@
         <v/>
       </c>
       <c r="AF20" s="19">
-        <f>IF(OR(AB20="",W20="",(W20+AD20)=0),"",(AB20-W20-AD20)/(W20+AD20))</f>
+        <f>IF(OR(AB20="",W20=""),"",IF((W20+N(AD20))=0,"",(AB20-W20-N(AD20))/(W20+N(AD20))))</f>
         <v/>
       </c>
       <c r="AG20" s="18" t="n"/>
@@ -3523,7 +3523,7 @@
         <v/>
       </c>
       <c r="AK20" s="19">
-        <f>IF(OR(AG20="",AB20="",(AB20+AI20)=0),"",(AG20-AB20-AI20)/(AB20+AI20))</f>
+        <f>IF(OR(AG20="",AB20=""),"",IF((AB20+N(AI20))=0,"",(AG20-AB20-N(AI20))/(AB20+N(AI20))))</f>
         <v/>
       </c>
       <c r="AL20" s="18" t="n"/>
@@ -3534,7 +3534,7 @@
         <v/>
       </c>
       <c r="AP20" s="19">
-        <f>IF(OR(AL20="",AG20="",(AG20+AN20)=0),"",(AL20-AG20-AN20)/(AG20+AN20))</f>
+        <f>IF(OR(AL20="",AG20=""),"",IF((AG20+N(AN20))=0,"",(AL20-AG20-N(AN20))/(AG20+N(AN20))))</f>
         <v/>
       </c>
       <c r="AQ20" s="18" t="n"/>
@@ -3545,7 +3545,7 @@
         <v/>
       </c>
       <c r="AU20" s="19">
-        <f>IF(OR(AQ20="",AL20="",(AL20+AS20)=0),"",(AQ20-AL20-AS20)/(AL20+AS20))</f>
+        <f>IF(OR(AQ20="",AL20=""),"",IF((AL20+N(AS20))=0,"",(AQ20-AL20-N(AS20))/(AL20+N(AS20))))</f>
         <v/>
       </c>
       <c r="AV20" s="18" t="n"/>
@@ -3556,7 +3556,7 @@
         <v/>
       </c>
       <c r="AZ20" s="19">
-        <f>IF(OR(AV20="",AQ20="",(AQ20+AX20)=0),"",(AV20-AQ20-AX20)/(AQ20+AX20))</f>
+        <f>IF(OR(AV20="",AQ20=""),"",IF((AQ20+N(AX20))=0,"",(AV20-AQ20-N(AX20))/(AQ20+N(AX20))))</f>
         <v/>
       </c>
       <c r="BA20" s="18" t="n"/>
@@ -3567,7 +3567,7 @@
         <v/>
       </c>
       <c r="BE20" s="19">
-        <f>IF(OR(BA20="",AV20="",(AV20+BC20)=0),"",(BA20-AV20-BC20)/(AV20+BC20))</f>
+        <f>IF(OR(BA20="",AV20=""),"",IF((AV20+N(BC20))=0,"",(BA20-AV20-N(BC20))/(AV20+N(BC20))))</f>
         <v/>
       </c>
       <c r="BF20" s="18" t="n"/>
@@ -3578,7 +3578,7 @@
         <v/>
       </c>
       <c r="BJ20" s="19">
-        <f>IF(OR(BF20="",BA20="",(BA20+BH20)=0),"",(BF20-BA20-BH20)/(BA20+BH20))</f>
+        <f>IF(OR(BF20="",BA20=""),"",IF((BA20+N(BH20))=0,"",(BF20-BA20-N(BH20))/(BA20+N(BH20))))</f>
         <v/>
       </c>
     </row>
@@ -3593,7 +3593,7 @@
         <v/>
       </c>
       <c r="G21" s="16">
-        <f>IF(OR(C21="",B21="",(B21+E21)=0),"",(C21-B21-E21)/(B21+E21))</f>
+        <f>IF(OR(C21="",B21=""),"",IF((B21+N(E21))=0,"",(C21-B21-N(E21))/(B21+N(E21))))</f>
         <v/>
       </c>
       <c r="H21" s="15" t="n"/>
@@ -3604,7 +3604,7 @@
         <v/>
       </c>
       <c r="L21" s="16">
-        <f>IF(OR(H21="",C21="",(C21+J21)=0),"",(H21-C21-J21)/(C21+J21))</f>
+        <f>IF(OR(H21="",C21=""),"",IF((C21+N(J21))=0,"",(H21-C21-N(J21))/(C21+N(J21))))</f>
         <v/>
       </c>
       <c r="M21" s="15" t="n"/>
@@ -3615,7 +3615,7 @@
         <v/>
       </c>
       <c r="Q21" s="16">
-        <f>IF(OR(M21="",H21="",(H21+O21)=0),"",(M21-H21-O21)/(H21+O21))</f>
+        <f>IF(OR(M21="",H21=""),"",IF((H21+N(O21))=0,"",(M21-H21-N(O21))/(H21+N(O21))))</f>
         <v/>
       </c>
       <c r="R21" s="15" t="n"/>
@@ -3626,7 +3626,7 @@
         <v/>
       </c>
       <c r="V21" s="16">
-        <f>IF(OR(R21="",M21="",(M21+T21)=0),"",(R21-M21-T21)/(M21+T21))</f>
+        <f>IF(OR(R21="",M21=""),"",IF((M21+N(T21))=0,"",(R21-M21-N(T21))/(M21+N(T21))))</f>
         <v/>
       </c>
       <c r="W21" s="15" t="n"/>
@@ -3637,7 +3637,7 @@
         <v/>
       </c>
       <c r="AA21" s="16">
-        <f>IF(OR(W21="",R21="",(R21+Y21)=0),"",(W21-R21-Y21)/(R21+Y21))</f>
+        <f>IF(OR(W21="",R21=""),"",IF((R21+N(Y21))=0,"",(W21-R21-N(Y21))/(R21+N(Y21))))</f>
         <v/>
       </c>
       <c r="AB21" s="15" t="n"/>
@@ -3648,7 +3648,7 @@
         <v/>
       </c>
       <c r="AF21" s="16">
-        <f>IF(OR(AB21="",W21="",(W21+AD21)=0),"",(AB21-W21-AD21)/(W21+AD21))</f>
+        <f>IF(OR(AB21="",W21=""),"",IF((W21+N(AD21))=0,"",(AB21-W21-N(AD21))/(W21+N(AD21))))</f>
         <v/>
       </c>
       <c r="AG21" s="15" t="n"/>
@@ -3659,7 +3659,7 @@
         <v/>
       </c>
       <c r="AK21" s="16">
-        <f>IF(OR(AG21="",AB21="",(AB21+AI21)=0),"",(AG21-AB21-AI21)/(AB21+AI21))</f>
+        <f>IF(OR(AG21="",AB21=""),"",IF((AB21+N(AI21))=0,"",(AG21-AB21-N(AI21))/(AB21+N(AI21))))</f>
         <v/>
       </c>
       <c r="AL21" s="15" t="n"/>
@@ -3670,7 +3670,7 @@
         <v/>
       </c>
       <c r="AP21" s="16">
-        <f>IF(OR(AL21="",AG21="",(AG21+AN21)=0),"",(AL21-AG21-AN21)/(AG21+AN21))</f>
+        <f>IF(OR(AL21="",AG21=""),"",IF((AG21+N(AN21))=0,"",(AL21-AG21-N(AN21))/(AG21+N(AN21))))</f>
         <v/>
       </c>
       <c r="AQ21" s="15" t="n"/>
@@ -3681,7 +3681,7 @@
         <v/>
       </c>
       <c r="AU21" s="16">
-        <f>IF(OR(AQ21="",AL21="",(AL21+AS21)=0),"",(AQ21-AL21-AS21)/(AL21+AS21))</f>
+        <f>IF(OR(AQ21="",AL21=""),"",IF((AL21+N(AS21))=0,"",(AQ21-AL21-N(AS21))/(AL21+N(AS21))))</f>
         <v/>
       </c>
       <c r="AV21" s="15" t="n"/>
@@ -3692,7 +3692,7 @@
         <v/>
       </c>
       <c r="AZ21" s="16">
-        <f>IF(OR(AV21="",AQ21="",(AQ21+AX21)=0),"",(AV21-AQ21-AX21)/(AQ21+AX21))</f>
+        <f>IF(OR(AV21="",AQ21=""),"",IF((AQ21+N(AX21))=0,"",(AV21-AQ21-N(AX21))/(AQ21+N(AX21))))</f>
         <v/>
       </c>
       <c r="BA21" s="15" t="n"/>
@@ -3703,7 +3703,7 @@
         <v/>
       </c>
       <c r="BE21" s="16">
-        <f>IF(OR(BA21="",AV21="",(AV21+BC21)=0),"",(BA21-AV21-BC21)/(AV21+BC21))</f>
+        <f>IF(OR(BA21="",AV21=""),"",IF((AV21+N(BC21))=0,"",(BA21-AV21-N(BC21))/(AV21+N(BC21))))</f>
         <v/>
       </c>
       <c r="BF21" s="15" t="n"/>
@@ -3714,7 +3714,7 @@
         <v/>
       </c>
       <c r="BJ21" s="16">
-        <f>IF(OR(BF21="",BA21="",(BA21+BH21)=0),"",(BF21-BA21-BH21)/(BA21+BH21))</f>
+        <f>IF(OR(BF21="",BA21=""),"",IF((BA21+N(BH21))=0,"",(BF21-BA21-N(BH21))/(BA21+N(BH21))))</f>
         <v/>
       </c>
     </row>
@@ -3729,7 +3729,7 @@
         <v/>
       </c>
       <c r="G22" s="19">
-        <f>IF(OR(C22="",B22="",(B22+E22)=0),"",(C22-B22-E22)/(B22+E22))</f>
+        <f>IF(OR(C22="",B22=""),"",IF((B22+N(E22))=0,"",(C22-B22-N(E22))/(B22+N(E22))))</f>
         <v/>
       </c>
       <c r="H22" s="18" t="n"/>
@@ -3740,7 +3740,7 @@
         <v/>
       </c>
       <c r="L22" s="19">
-        <f>IF(OR(H22="",C22="",(C22+J22)=0),"",(H22-C22-J22)/(C22+J22))</f>
+        <f>IF(OR(H22="",C22=""),"",IF((C22+N(J22))=0,"",(H22-C22-N(J22))/(C22+N(J22))))</f>
         <v/>
       </c>
       <c r="M22" s="18" t="n"/>
@@ -3751,7 +3751,7 @@
         <v/>
       </c>
       <c r="Q22" s="19">
-        <f>IF(OR(M22="",H22="",(H22+O22)=0),"",(M22-H22-O22)/(H22+O22))</f>
+        <f>IF(OR(M22="",H22=""),"",IF((H22+N(O22))=0,"",(M22-H22-N(O22))/(H22+N(O22))))</f>
         <v/>
       </c>
       <c r="R22" s="18" t="n"/>
@@ -3762,7 +3762,7 @@
         <v/>
       </c>
       <c r="V22" s="19">
-        <f>IF(OR(R22="",M22="",(M22+T22)=0),"",(R22-M22-T22)/(M22+T22))</f>
+        <f>IF(OR(R22="",M22=""),"",IF((M22+N(T22))=0,"",(R22-M22-N(T22))/(M22+N(T22))))</f>
         <v/>
       </c>
       <c r="W22" s="18" t="n"/>
@@ -3773,7 +3773,7 @@
         <v/>
       </c>
       <c r="AA22" s="19">
-        <f>IF(OR(W22="",R22="",(R22+Y22)=0),"",(W22-R22-Y22)/(R22+Y22))</f>
+        <f>IF(OR(W22="",R22=""),"",IF((R22+N(Y22))=0,"",(W22-R22-N(Y22))/(R22+N(Y22))))</f>
         <v/>
       </c>
       <c r="AB22" s="18" t="n"/>
@@ -3784,7 +3784,7 @@
         <v/>
       </c>
       <c r="AF22" s="19">
-        <f>IF(OR(AB22="",W22="",(W22+AD22)=0),"",(AB22-W22-AD22)/(W22+AD22))</f>
+        <f>IF(OR(AB22="",W22=""),"",IF((W22+N(AD22))=0,"",(AB22-W22-N(AD22))/(W22+N(AD22))))</f>
         <v/>
       </c>
       <c r="AG22" s="18" t="n"/>
@@ -3795,7 +3795,7 @@
         <v/>
       </c>
       <c r="AK22" s="19">
-        <f>IF(OR(AG22="",AB22="",(AB22+AI22)=0),"",(AG22-AB22-AI22)/(AB22+AI22))</f>
+        <f>IF(OR(AG22="",AB22=""),"",IF((AB22+N(AI22))=0,"",(AG22-AB22-N(AI22))/(AB22+N(AI22))))</f>
         <v/>
       </c>
       <c r="AL22" s="18" t="n"/>
@@ -3806,7 +3806,7 @@
         <v/>
       </c>
       <c r="AP22" s="19">
-        <f>IF(OR(AL22="",AG22="",(AG22+AN22)=0),"",(AL22-AG22-AN22)/(AG22+AN22))</f>
+        <f>IF(OR(AL22="",AG22=""),"",IF((AG22+N(AN22))=0,"",(AL22-AG22-N(AN22))/(AG22+N(AN22))))</f>
         <v/>
       </c>
       <c r="AQ22" s="18" t="n"/>
@@ -3817,7 +3817,7 @@
         <v/>
       </c>
       <c r="AU22" s="19">
-        <f>IF(OR(AQ22="",AL22="",(AL22+AS22)=0),"",(AQ22-AL22-AS22)/(AL22+AS22))</f>
+        <f>IF(OR(AQ22="",AL22=""),"",IF((AL22+N(AS22))=0,"",(AQ22-AL22-N(AS22))/(AL22+N(AS22))))</f>
         <v/>
       </c>
       <c r="AV22" s="18" t="n"/>
@@ -3828,7 +3828,7 @@
         <v/>
       </c>
       <c r="AZ22" s="19">
-        <f>IF(OR(AV22="",AQ22="",(AQ22+AX22)=0),"",(AV22-AQ22-AX22)/(AQ22+AX22))</f>
+        <f>IF(OR(AV22="",AQ22=""),"",IF((AQ22+N(AX22))=0,"",(AV22-AQ22-N(AX22))/(AQ22+N(AX22))))</f>
         <v/>
       </c>
       <c r="BA22" s="18" t="n"/>
@@ -3839,7 +3839,7 @@
         <v/>
       </c>
       <c r="BE22" s="19">
-        <f>IF(OR(BA22="",AV22="",(AV22+BC22)=0),"",(BA22-AV22-BC22)/(AV22+BC22))</f>
+        <f>IF(OR(BA22="",AV22=""),"",IF((AV22+N(BC22))=0,"",(BA22-AV22-N(BC22))/(AV22+N(BC22))))</f>
         <v/>
       </c>
       <c r="BF22" s="18" t="n"/>
@@ -3850,7 +3850,7 @@
         <v/>
       </c>
       <c r="BJ22" s="19">
-        <f>IF(OR(BF22="",BA22="",(BA22+BH22)=0),"",(BF22-BA22-BH22)/(BA22+BH22))</f>
+        <f>IF(OR(BF22="",BA22=""),"",IF((BA22+N(BH22))=0,"",(BF22-BA22-N(BH22))/(BA22+N(BH22))))</f>
         <v/>
       </c>
     </row>
@@ -3881,7 +3881,7 @@
         <v/>
       </c>
       <c r="G23" s="13">
-        <f>IF(OR(C23="",B23="",(B23+E23)=0),"",(C23-B23-E23)/(B23+E23))</f>
+        <f>IF(OR(C23="",B23=""),"",IF((B23+N(E23))=0,"",(C23-B23-N(E23))/(B23+N(E23))))</f>
         <v/>
       </c>
       <c r="H23" s="12">
@@ -3901,7 +3901,7 @@
         <v/>
       </c>
       <c r="L23" s="13">
-        <f>IF(OR(H23="",C23="",(C23+J23)=0),"",(H23-C23-J23)/(C23+J23))</f>
+        <f>IF(OR(H23="",C23=""),"",IF((C23+N(J23))=0,"",(H23-C23-N(J23))/(C23+N(J23))))</f>
         <v/>
       </c>
       <c r="M23" s="12">
@@ -3921,7 +3921,7 @@
         <v/>
       </c>
       <c r="Q23" s="13">
-        <f>IF(OR(M23="",H23="",(H23+O23)=0),"",(M23-H23-O23)/(H23+O23))</f>
+        <f>IF(OR(M23="",H23=""),"",IF((H23+N(O23))=0,"",(M23-H23-N(O23))/(H23+N(O23))))</f>
         <v/>
       </c>
       <c r="R23" s="12">
@@ -3941,7 +3941,7 @@
         <v/>
       </c>
       <c r="V23" s="13">
-        <f>IF(OR(R23="",M23="",(M23+T23)=0),"",(R23-M23-T23)/(M23+T23))</f>
+        <f>IF(OR(R23="",M23=""),"",IF((M23+N(T23))=0,"",(R23-M23-N(T23))/(M23+N(T23))))</f>
         <v/>
       </c>
       <c r="W23" s="12">
@@ -3961,7 +3961,7 @@
         <v/>
       </c>
       <c r="AA23" s="13">
-        <f>IF(OR(W23="",R23="",(R23+Y23)=0),"",(W23-R23-Y23)/(R23+Y23))</f>
+        <f>IF(OR(W23="",R23=""),"",IF((R23+N(Y23))=0,"",(W23-R23-N(Y23))/(R23+N(Y23))))</f>
         <v/>
       </c>
       <c r="AB23" s="12">
@@ -3981,7 +3981,7 @@
         <v/>
       </c>
       <c r="AF23" s="13">
-        <f>IF(OR(AB23="",W23="",(W23+AD23)=0),"",(AB23-W23-AD23)/(W23+AD23))</f>
+        <f>IF(OR(AB23="",W23=""),"",IF((W23+N(AD23))=0,"",(AB23-W23-N(AD23))/(W23+N(AD23))))</f>
         <v/>
       </c>
       <c r="AG23" s="12">
@@ -4001,7 +4001,7 @@
         <v/>
       </c>
       <c r="AK23" s="13">
-        <f>IF(OR(AG23="",AB23="",(AB23+AI23)=0),"",(AG23-AB23-AI23)/(AB23+AI23))</f>
+        <f>IF(OR(AG23="",AB23=""),"",IF((AB23+N(AI23))=0,"",(AG23-AB23-N(AI23))/(AB23+N(AI23))))</f>
         <v/>
       </c>
       <c r="AL23" s="12">
@@ -4021,7 +4021,7 @@
         <v/>
       </c>
       <c r="AP23" s="13">
-        <f>IF(OR(AL23="",AG23="",(AG23+AN23)=0),"",(AL23-AG23-AN23)/(AG23+AN23))</f>
+        <f>IF(OR(AL23="",AG23=""),"",IF((AG23+N(AN23))=0,"",(AL23-AG23-N(AN23))/(AG23+N(AN23))))</f>
         <v/>
       </c>
       <c r="AQ23" s="12">
@@ -4041,7 +4041,7 @@
         <v/>
       </c>
       <c r="AU23" s="13">
-        <f>IF(OR(AQ23="",AL23="",(AL23+AS23)=0),"",(AQ23-AL23-AS23)/(AL23+AS23))</f>
+        <f>IF(OR(AQ23="",AL23=""),"",IF((AL23+N(AS23))=0,"",(AQ23-AL23-N(AS23))/(AL23+N(AS23))))</f>
         <v/>
       </c>
       <c r="AV23" s="12">
@@ -4061,7 +4061,7 @@
         <v/>
       </c>
       <c r="AZ23" s="13">
-        <f>IF(OR(AV23="",AQ23="",(AQ23+AX23)=0),"",(AV23-AQ23-AX23)/(AQ23+AX23))</f>
+        <f>IF(OR(AV23="",AQ23=""),"",IF((AQ23+N(AX23))=0,"",(AV23-AQ23-N(AX23))/(AQ23+N(AX23))))</f>
         <v/>
       </c>
       <c r="BA23" s="12">
@@ -4081,7 +4081,7 @@
         <v/>
       </c>
       <c r="BE23" s="13">
-        <f>IF(OR(BA23="",AV23="",(AV23+BC23)=0),"",(BA23-AV23-BC23)/(AV23+BC23))</f>
+        <f>IF(OR(BA23="",AV23=""),"",IF((AV23+N(BC23))=0,"",(BA23-AV23-N(BC23))/(AV23+N(BC23))))</f>
         <v/>
       </c>
       <c r="BF23" s="12">
@@ -4101,7 +4101,7 @@
         <v/>
       </c>
       <c r="BJ23" s="13">
-        <f>IF(OR(BF23="",BA23="",(BA23+BH23)=0),"",(BF23-BA23-BH23)/(BA23+BH23))</f>
+        <f>IF(OR(BF23="",BA23=""),"",IF((BA23+N(BH23))=0,"",(BF23-BA23-N(BH23))/(BA23+N(BH23))))</f>
         <v/>
       </c>
     </row>
@@ -4116,7 +4116,7 @@
         <v/>
       </c>
       <c r="G24" s="16">
-        <f>IF(OR(C24="",B24="",(B24+E24)=0),"",(C24-B24-E24)/(B24+E24))</f>
+        <f>IF(OR(C24="",B24=""),"",IF((B24+N(E24))=0,"",(C24-B24-N(E24))/(B24+N(E24))))</f>
         <v/>
       </c>
       <c r="H24" s="15" t="n"/>
@@ -4127,7 +4127,7 @@
         <v/>
       </c>
       <c r="L24" s="16">
-        <f>IF(OR(H24="",C24="",(C24+J24)=0),"",(H24-C24-J24)/(C24+J24))</f>
+        <f>IF(OR(H24="",C24=""),"",IF((C24+N(J24))=0,"",(H24-C24-N(J24))/(C24+N(J24))))</f>
         <v/>
       </c>
       <c r="M24" s="15" t="n"/>
@@ -4138,7 +4138,7 @@
         <v/>
       </c>
       <c r="Q24" s="16">
-        <f>IF(OR(M24="",H24="",(H24+O24)=0),"",(M24-H24-O24)/(H24+O24))</f>
+        <f>IF(OR(M24="",H24=""),"",IF((H24+N(O24))=0,"",(M24-H24-N(O24))/(H24+N(O24))))</f>
         <v/>
       </c>
       <c r="R24" s="15" t="n"/>
@@ -4149,7 +4149,7 @@
         <v/>
       </c>
       <c r="V24" s="16">
-        <f>IF(OR(R24="",M24="",(M24+T24)=0),"",(R24-M24-T24)/(M24+T24))</f>
+        <f>IF(OR(R24="",M24=""),"",IF((M24+N(T24))=0,"",(R24-M24-N(T24))/(M24+N(T24))))</f>
         <v/>
       </c>
       <c r="W24" s="15" t="n"/>
@@ -4160,7 +4160,7 @@
         <v/>
       </c>
       <c r="AA24" s="16">
-        <f>IF(OR(W24="",R24="",(R24+Y24)=0),"",(W24-R24-Y24)/(R24+Y24))</f>
+        <f>IF(OR(W24="",R24=""),"",IF((R24+N(Y24))=0,"",(W24-R24-N(Y24))/(R24+N(Y24))))</f>
         <v/>
       </c>
       <c r="AB24" s="15" t="n"/>
@@ -4171,7 +4171,7 @@
         <v/>
       </c>
       <c r="AF24" s="16">
-        <f>IF(OR(AB24="",W24="",(W24+AD24)=0),"",(AB24-W24-AD24)/(W24+AD24))</f>
+        <f>IF(OR(AB24="",W24=""),"",IF((W24+N(AD24))=0,"",(AB24-W24-N(AD24))/(W24+N(AD24))))</f>
         <v/>
       </c>
       <c r="AG24" s="15" t="n"/>
@@ -4182,7 +4182,7 @@
         <v/>
       </c>
       <c r="AK24" s="16">
-        <f>IF(OR(AG24="",AB24="",(AB24+AI24)=0),"",(AG24-AB24-AI24)/(AB24+AI24))</f>
+        <f>IF(OR(AG24="",AB24=""),"",IF((AB24+N(AI24))=0,"",(AG24-AB24-N(AI24))/(AB24+N(AI24))))</f>
         <v/>
       </c>
       <c r="AL24" s="15" t="n"/>
@@ -4193,7 +4193,7 @@
         <v/>
       </c>
       <c r="AP24" s="16">
-        <f>IF(OR(AL24="",AG24="",(AG24+AN24)=0),"",(AL24-AG24-AN24)/(AG24+AN24))</f>
+        <f>IF(OR(AL24="",AG24=""),"",IF((AG24+N(AN24))=0,"",(AL24-AG24-N(AN24))/(AG24+N(AN24))))</f>
         <v/>
       </c>
       <c r="AQ24" s="15" t="n"/>
@@ -4204,7 +4204,7 @@
         <v/>
       </c>
       <c r="AU24" s="16">
-        <f>IF(OR(AQ24="",AL24="",(AL24+AS24)=0),"",(AQ24-AL24-AS24)/(AL24+AS24))</f>
+        <f>IF(OR(AQ24="",AL24=""),"",IF((AL24+N(AS24))=0,"",(AQ24-AL24-N(AS24))/(AL24+N(AS24))))</f>
         <v/>
       </c>
       <c r="AV24" s="15" t="n"/>
@@ -4215,7 +4215,7 @@
         <v/>
       </c>
       <c r="AZ24" s="16">
-        <f>IF(OR(AV24="",AQ24="",(AQ24+AX24)=0),"",(AV24-AQ24-AX24)/(AQ24+AX24))</f>
+        <f>IF(OR(AV24="",AQ24=""),"",IF((AQ24+N(AX24))=0,"",(AV24-AQ24-N(AX24))/(AQ24+N(AX24))))</f>
         <v/>
       </c>
       <c r="BA24" s="15" t="n"/>
@@ -4226,7 +4226,7 @@
         <v/>
       </c>
       <c r="BE24" s="16">
-        <f>IF(OR(BA24="",AV24="",(AV24+BC24)=0),"",(BA24-AV24-BC24)/(AV24+BC24))</f>
+        <f>IF(OR(BA24="",AV24=""),"",IF((AV24+N(BC24))=0,"",(BA24-AV24-N(BC24))/(AV24+N(BC24))))</f>
         <v/>
       </c>
       <c r="BF24" s="15" t="n"/>
@@ -4237,7 +4237,7 @@
         <v/>
       </c>
       <c r="BJ24" s="16">
-        <f>IF(OR(BF24="",BA24="",(BA24+BH24)=0),"",(BF24-BA24-BH24)/(BA24+BH24))</f>
+        <f>IF(OR(BF24="",BA24=""),"",IF((BA24+N(BH24))=0,"",(BF24-BA24-N(BH24))/(BA24+N(BH24))))</f>
         <v/>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v/>
       </c>
       <c r="G25" s="19">
-        <f>IF(OR(C25="",B25="",(B25+E25)=0),"",(C25-B25-E25)/(B25+E25))</f>
+        <f>IF(OR(C25="",B25=""),"",IF((B25+N(E25))=0,"",(C25-B25-N(E25))/(B25+N(E25))))</f>
         <v/>
       </c>
       <c r="H25" s="18" t="n"/>
@@ -4263,7 +4263,7 @@
         <v/>
       </c>
       <c r="L25" s="19">
-        <f>IF(OR(H25="",C25="",(C25+J25)=0),"",(H25-C25-J25)/(C25+J25))</f>
+        <f>IF(OR(H25="",C25=""),"",IF((C25+N(J25))=0,"",(H25-C25-N(J25))/(C25+N(J25))))</f>
         <v/>
       </c>
       <c r="M25" s="18" t="n"/>
@@ -4274,7 +4274,7 @@
         <v/>
       </c>
       <c r="Q25" s="19">
-        <f>IF(OR(M25="",H25="",(H25+O25)=0),"",(M25-H25-O25)/(H25+O25))</f>
+        <f>IF(OR(M25="",H25=""),"",IF((H25+N(O25))=0,"",(M25-H25-N(O25))/(H25+N(O25))))</f>
         <v/>
       </c>
       <c r="R25" s="18" t="n"/>
@@ -4285,7 +4285,7 @@
         <v/>
       </c>
       <c r="V25" s="19">
-        <f>IF(OR(R25="",M25="",(M25+T25)=0),"",(R25-M25-T25)/(M25+T25))</f>
+        <f>IF(OR(R25="",M25=""),"",IF((M25+N(T25))=0,"",(R25-M25-N(T25))/(M25+N(T25))))</f>
         <v/>
       </c>
       <c r="W25" s="18" t="n"/>
@@ -4296,7 +4296,7 @@
         <v/>
       </c>
       <c r="AA25" s="19">
-        <f>IF(OR(W25="",R25="",(R25+Y25)=0),"",(W25-R25-Y25)/(R25+Y25))</f>
+        <f>IF(OR(W25="",R25=""),"",IF((R25+N(Y25))=0,"",(W25-R25-N(Y25))/(R25+N(Y25))))</f>
         <v/>
       </c>
       <c r="AB25" s="18" t="n"/>
@@ -4307,7 +4307,7 @@
         <v/>
       </c>
       <c r="AF25" s="19">
-        <f>IF(OR(AB25="",W25="",(W25+AD25)=0),"",(AB25-W25-AD25)/(W25+AD25))</f>
+        <f>IF(OR(AB25="",W25=""),"",IF((W25+N(AD25))=0,"",(AB25-W25-N(AD25))/(W25+N(AD25))))</f>
         <v/>
       </c>
       <c r="AG25" s="18" t="n"/>
@@ -4318,7 +4318,7 @@
         <v/>
       </c>
       <c r="AK25" s="19">
-        <f>IF(OR(AG25="",AB25="",(AB25+AI25)=0),"",(AG25-AB25-AI25)/(AB25+AI25))</f>
+        <f>IF(OR(AG25="",AB25=""),"",IF((AB25+N(AI25))=0,"",(AG25-AB25-N(AI25))/(AB25+N(AI25))))</f>
         <v/>
       </c>
       <c r="AL25" s="18" t="n"/>
@@ -4329,7 +4329,7 @@
         <v/>
       </c>
       <c r="AP25" s="19">
-        <f>IF(OR(AL25="",AG25="",(AG25+AN25)=0),"",(AL25-AG25-AN25)/(AG25+AN25))</f>
+        <f>IF(OR(AL25="",AG25=""),"",IF((AG25+N(AN25))=0,"",(AL25-AG25-N(AN25))/(AG25+N(AN25))))</f>
         <v/>
       </c>
       <c r="AQ25" s="18" t="n"/>
@@ -4340,7 +4340,7 @@
         <v/>
       </c>
       <c r="AU25" s="19">
-        <f>IF(OR(AQ25="",AL25="",(AL25+AS25)=0),"",(AQ25-AL25-AS25)/(AL25+AS25))</f>
+        <f>IF(OR(AQ25="",AL25=""),"",IF((AL25+N(AS25))=0,"",(AQ25-AL25-N(AS25))/(AL25+N(AS25))))</f>
         <v/>
       </c>
       <c r="AV25" s="18" t="n"/>
@@ -4351,7 +4351,7 @@
         <v/>
       </c>
       <c r="AZ25" s="19">
-        <f>IF(OR(AV25="",AQ25="",(AQ25+AX25)=0),"",(AV25-AQ25-AX25)/(AQ25+AX25))</f>
+        <f>IF(OR(AV25="",AQ25=""),"",IF((AQ25+N(AX25))=0,"",(AV25-AQ25-N(AX25))/(AQ25+N(AX25))))</f>
         <v/>
       </c>
       <c r="BA25" s="18" t="n"/>
@@ -4362,7 +4362,7 @@
         <v/>
       </c>
       <c r="BE25" s="19">
-        <f>IF(OR(BA25="",AV25="",(AV25+BC25)=0),"",(BA25-AV25-BC25)/(AV25+BC25))</f>
+        <f>IF(OR(BA25="",AV25=""),"",IF((AV25+N(BC25))=0,"",(BA25-AV25-N(BC25))/(AV25+N(BC25))))</f>
         <v/>
       </c>
       <c r="BF25" s="18" t="n"/>
@@ -4373,7 +4373,7 @@
         <v/>
       </c>
       <c r="BJ25" s="19">
-        <f>IF(OR(BF25="",BA25="",(BA25+BH25)=0),"",(BF25-BA25-BH25)/(BA25+BH25))</f>
+        <f>IF(OR(BF25="",BA25=""),"",IF((BA25+N(BH25))=0,"",(BF25-BA25-N(BH25))/(BA25+N(BH25))))</f>
         <v/>
       </c>
     </row>
@@ -4388,7 +4388,7 @@
         <v/>
       </c>
       <c r="G26" s="16">
-        <f>IF(OR(C26="",B26="",(B26+E26)=0),"",(C26-B26-E26)/(B26+E26))</f>
+        <f>IF(OR(C26="",B26=""),"",IF((B26+N(E26))=0,"",(C26-B26-N(E26))/(B26+N(E26))))</f>
         <v/>
       </c>
       <c r="H26" s="15" t="n"/>
@@ -4399,7 +4399,7 @@
         <v/>
       </c>
       <c r="L26" s="16">
-        <f>IF(OR(H26="",C26="",(C26+J26)=0),"",(H26-C26-J26)/(C26+J26))</f>
+        <f>IF(OR(H26="",C26=""),"",IF((C26+N(J26))=0,"",(H26-C26-N(J26))/(C26+N(J26))))</f>
         <v/>
       </c>
       <c r="M26" s="15" t="n"/>
@@ -4410,7 +4410,7 @@
         <v/>
       </c>
       <c r="Q26" s="16">
-        <f>IF(OR(M26="",H26="",(H26+O26)=0),"",(M26-H26-O26)/(H26+O26))</f>
+        <f>IF(OR(M26="",H26=""),"",IF((H26+N(O26))=0,"",(M26-H26-N(O26))/(H26+N(O26))))</f>
         <v/>
       </c>
       <c r="R26" s="15" t="n"/>
@@ -4421,7 +4421,7 @@
         <v/>
       </c>
       <c r="V26" s="16">
-        <f>IF(OR(R26="",M26="",(M26+T26)=0),"",(R26-M26-T26)/(M26+T26))</f>
+        <f>IF(OR(R26="",M26=""),"",IF((M26+N(T26))=0,"",(R26-M26-N(T26))/(M26+N(T26))))</f>
         <v/>
       </c>
       <c r="W26" s="15" t="n"/>
@@ -4432,7 +4432,7 @@
         <v/>
       </c>
       <c r="AA26" s="16">
-        <f>IF(OR(W26="",R26="",(R26+Y26)=0),"",(W26-R26-Y26)/(R26+Y26))</f>
+        <f>IF(OR(W26="",R26=""),"",IF((R26+N(Y26))=0,"",(W26-R26-N(Y26))/(R26+N(Y26))))</f>
         <v/>
       </c>
       <c r="AB26" s="15" t="n"/>
@@ -4443,7 +4443,7 @@
         <v/>
       </c>
       <c r="AF26" s="16">
-        <f>IF(OR(AB26="",W26="",(W26+AD26)=0),"",(AB26-W26-AD26)/(W26+AD26))</f>
+        <f>IF(OR(AB26="",W26=""),"",IF((W26+N(AD26))=0,"",(AB26-W26-N(AD26))/(W26+N(AD26))))</f>
         <v/>
       </c>
       <c r="AG26" s="15" t="n"/>
@@ -4454,7 +4454,7 @@
         <v/>
       </c>
       <c r="AK26" s="16">
-        <f>IF(OR(AG26="",AB26="",(AB26+AI26)=0),"",(AG26-AB26-AI26)/(AB26+AI26))</f>
+        <f>IF(OR(AG26="",AB26=""),"",IF((AB26+N(AI26))=0,"",(AG26-AB26-N(AI26))/(AB26+N(AI26))))</f>
         <v/>
       </c>
       <c r="AL26" s="15" t="n"/>
@@ -4465,7 +4465,7 @@
         <v/>
       </c>
       <c r="AP26" s="16">
-        <f>IF(OR(AL26="",AG26="",(AG26+AN26)=0),"",(AL26-AG26-AN26)/(AG26+AN26))</f>
+        <f>IF(OR(AL26="",AG26=""),"",IF((AG26+N(AN26))=0,"",(AL26-AG26-N(AN26))/(AG26+N(AN26))))</f>
         <v/>
       </c>
       <c r="AQ26" s="15" t="n"/>
@@ -4476,7 +4476,7 @@
         <v/>
       </c>
       <c r="AU26" s="16">
-        <f>IF(OR(AQ26="",AL26="",(AL26+AS26)=0),"",(AQ26-AL26-AS26)/(AL26+AS26))</f>
+        <f>IF(OR(AQ26="",AL26=""),"",IF((AL26+N(AS26))=0,"",(AQ26-AL26-N(AS26))/(AL26+N(AS26))))</f>
         <v/>
       </c>
       <c r="AV26" s="15" t="n"/>
@@ -4487,7 +4487,7 @@
         <v/>
       </c>
       <c r="AZ26" s="16">
-        <f>IF(OR(AV26="",AQ26="",(AQ26+AX26)=0),"",(AV26-AQ26-AX26)/(AQ26+AX26))</f>
+        <f>IF(OR(AV26="",AQ26=""),"",IF((AQ26+N(AX26))=0,"",(AV26-AQ26-N(AX26))/(AQ26+N(AX26))))</f>
         <v/>
       </c>
       <c r="BA26" s="15" t="n"/>
@@ -4498,7 +4498,7 @@
         <v/>
       </c>
       <c r="BE26" s="16">
-        <f>IF(OR(BA26="",AV26="",(AV26+BC26)=0),"",(BA26-AV26-BC26)/(AV26+BC26))</f>
+        <f>IF(OR(BA26="",AV26=""),"",IF((AV26+N(BC26))=0,"",(BA26-AV26-N(BC26))/(AV26+N(BC26))))</f>
         <v/>
       </c>
       <c r="BF26" s="15" t="n"/>
@@ -4509,7 +4509,7 @@
         <v/>
       </c>
       <c r="BJ26" s="16">
-        <f>IF(OR(BF26="",BA26="",(BA26+BH26)=0),"",(BF26-BA26-BH26)/(BA26+BH26))</f>
+        <f>IF(OR(BF26="",BA26=""),"",IF((BA26+N(BH26))=0,"",(BF26-BA26-N(BH26))/(BA26+N(BH26))))</f>
         <v/>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
         <v/>
       </c>
       <c r="G27" s="19">
-        <f>IF(OR(C27="",B27="",(B27+E27)=0),"",(C27-B27-E27)/(B27+E27))</f>
+        <f>IF(OR(C27="",B27=""),"",IF((B27+N(E27))=0,"",(C27-B27-N(E27))/(B27+N(E27))))</f>
         <v/>
       </c>
       <c r="H27" s="18" t="n"/>
@@ -4535,7 +4535,7 @@
         <v/>
       </c>
       <c r="L27" s="19">
-        <f>IF(OR(H27="",C27="",(C27+J27)=0),"",(H27-C27-J27)/(C27+J27))</f>
+        <f>IF(OR(H27="",C27=""),"",IF((C27+N(J27))=0,"",(H27-C27-N(J27))/(C27+N(J27))))</f>
         <v/>
       </c>
       <c r="M27" s="18" t="n"/>
@@ -4546,7 +4546,7 @@
         <v/>
       </c>
       <c r="Q27" s="19">
-        <f>IF(OR(M27="",H27="",(H27+O27)=0),"",(M27-H27-O27)/(H27+O27))</f>
+        <f>IF(OR(M27="",H27=""),"",IF((H27+N(O27))=0,"",(M27-H27-N(O27))/(H27+N(O27))))</f>
         <v/>
       </c>
       <c r="R27" s="18" t="n"/>
@@ -4557,7 +4557,7 @@
         <v/>
       </c>
       <c r="V27" s="19">
-        <f>IF(OR(R27="",M27="",(M27+T27)=0),"",(R27-M27-T27)/(M27+T27))</f>
+        <f>IF(OR(R27="",M27=""),"",IF((M27+N(T27))=0,"",(R27-M27-N(T27))/(M27+N(T27))))</f>
         <v/>
       </c>
       <c r="W27" s="18" t="n"/>
@@ -4568,7 +4568,7 @@
         <v/>
       </c>
       <c r="AA27" s="19">
-        <f>IF(OR(W27="",R27="",(R27+Y27)=0),"",(W27-R27-Y27)/(R27+Y27))</f>
+        <f>IF(OR(W27="",R27=""),"",IF((R27+N(Y27))=0,"",(W27-R27-N(Y27))/(R27+N(Y27))))</f>
         <v/>
       </c>
       <c r="AB27" s="18" t="n"/>
@@ -4579,7 +4579,7 @@
         <v/>
       </c>
       <c r="AF27" s="19">
-        <f>IF(OR(AB27="",W27="",(W27+AD27)=0),"",(AB27-W27-AD27)/(W27+AD27))</f>
+        <f>IF(OR(AB27="",W27=""),"",IF((W27+N(AD27))=0,"",(AB27-W27-N(AD27))/(W27+N(AD27))))</f>
         <v/>
       </c>
       <c r="AG27" s="18" t="n"/>
@@ -4590,7 +4590,7 @@
         <v/>
       </c>
       <c r="AK27" s="19">
-        <f>IF(OR(AG27="",AB27="",(AB27+AI27)=0),"",(AG27-AB27-AI27)/(AB27+AI27))</f>
+        <f>IF(OR(AG27="",AB27=""),"",IF((AB27+N(AI27))=0,"",(AG27-AB27-N(AI27))/(AB27+N(AI27))))</f>
         <v/>
       </c>
       <c r="AL27" s="18" t="n"/>
@@ -4601,7 +4601,7 @@
         <v/>
       </c>
       <c r="AP27" s="19">
-        <f>IF(OR(AL27="",AG27="",(AG27+AN27)=0),"",(AL27-AG27-AN27)/(AG27+AN27))</f>
+        <f>IF(OR(AL27="",AG27=""),"",IF((AG27+N(AN27))=0,"",(AL27-AG27-N(AN27))/(AG27+N(AN27))))</f>
         <v/>
       </c>
       <c r="AQ27" s="18" t="n"/>
@@ -4612,7 +4612,7 @@
         <v/>
       </c>
       <c r="AU27" s="19">
-        <f>IF(OR(AQ27="",AL27="",(AL27+AS27)=0),"",(AQ27-AL27-AS27)/(AL27+AS27))</f>
+        <f>IF(OR(AQ27="",AL27=""),"",IF((AL27+N(AS27))=0,"",(AQ27-AL27-N(AS27))/(AL27+N(AS27))))</f>
         <v/>
       </c>
       <c r="AV27" s="18" t="n"/>
@@ -4623,7 +4623,7 @@
         <v/>
       </c>
       <c r="AZ27" s="19">
-        <f>IF(OR(AV27="",AQ27="",(AQ27+AX27)=0),"",(AV27-AQ27-AX27)/(AQ27+AX27))</f>
+        <f>IF(OR(AV27="",AQ27=""),"",IF((AQ27+N(AX27))=0,"",(AV27-AQ27-N(AX27))/(AQ27+N(AX27))))</f>
         <v/>
       </c>
       <c r="BA27" s="18" t="n"/>
@@ -4634,7 +4634,7 @@
         <v/>
       </c>
       <c r="BE27" s="19">
-        <f>IF(OR(BA27="",AV27="",(AV27+BC27)=0),"",(BA27-AV27-BC27)/(AV27+BC27))</f>
+        <f>IF(OR(BA27="",AV27=""),"",IF((AV27+N(BC27))=0,"",(BA27-AV27-N(BC27))/(AV27+N(BC27))))</f>
         <v/>
       </c>
       <c r="BF27" s="18" t="n"/>
@@ -4645,7 +4645,7 @@
         <v/>
       </c>
       <c r="BJ27" s="19">
-        <f>IF(OR(BF27="",BA27="",(BA27+BH27)=0),"",(BF27-BA27-BH27)/(BA27+BH27))</f>
+        <f>IF(OR(BF27="",BA27=""),"",IF((BA27+N(BH27))=0,"",(BF27-BA27-N(BH27))/(BA27+N(BH27))))</f>
         <v/>
       </c>
     </row>
@@ -4660,7 +4660,7 @@
         <v/>
       </c>
       <c r="G28" s="16">
-        <f>IF(OR(C28="",B28="",(B28+E28)=0),"",(C28-B28-E28)/(B28+E28))</f>
+        <f>IF(OR(C28="",B28=""),"",IF((B28+N(E28))=0,"",(C28-B28-N(E28))/(B28+N(E28))))</f>
         <v/>
       </c>
       <c r="H28" s="15" t="n"/>
@@ -4671,7 +4671,7 @@
         <v/>
       </c>
       <c r="L28" s="16">
-        <f>IF(OR(H28="",C28="",(C28+J28)=0),"",(H28-C28-J28)/(C28+J28))</f>
+        <f>IF(OR(H28="",C28=""),"",IF((C28+N(J28))=0,"",(H28-C28-N(J28))/(C28+N(J28))))</f>
         <v/>
       </c>
       <c r="M28" s="15" t="n"/>
@@ -4682,7 +4682,7 @@
         <v/>
       </c>
       <c r="Q28" s="16">
-        <f>IF(OR(M28="",H28="",(H28+O28)=0),"",(M28-H28-O28)/(H28+O28))</f>
+        <f>IF(OR(M28="",H28=""),"",IF((H28+N(O28))=0,"",(M28-H28-N(O28))/(H28+N(O28))))</f>
         <v/>
       </c>
       <c r="R28" s="15" t="n"/>
@@ -4693,7 +4693,7 @@
         <v/>
       </c>
       <c r="V28" s="16">
-        <f>IF(OR(R28="",M28="",(M28+T28)=0),"",(R28-M28-T28)/(M28+T28))</f>
+        <f>IF(OR(R28="",M28=""),"",IF((M28+N(T28))=0,"",(R28-M28-N(T28))/(M28+N(T28))))</f>
         <v/>
       </c>
       <c r="W28" s="15" t="n"/>
@@ -4704,7 +4704,7 @@
         <v/>
       </c>
       <c r="AA28" s="16">
-        <f>IF(OR(W28="",R28="",(R28+Y28)=0),"",(W28-R28-Y28)/(R28+Y28))</f>
+        <f>IF(OR(W28="",R28=""),"",IF((R28+N(Y28))=0,"",(W28-R28-N(Y28))/(R28+N(Y28))))</f>
         <v/>
       </c>
       <c r="AB28" s="15" t="n"/>
@@ -4715,7 +4715,7 @@
         <v/>
       </c>
       <c r="AF28" s="16">
-        <f>IF(OR(AB28="",W28="",(W28+AD28)=0),"",(AB28-W28-AD28)/(W28+AD28))</f>
+        <f>IF(OR(AB28="",W28=""),"",IF((W28+N(AD28))=0,"",(AB28-W28-N(AD28))/(W28+N(AD28))))</f>
         <v/>
       </c>
       <c r="AG28" s="15" t="n"/>
@@ -4726,7 +4726,7 @@
         <v/>
       </c>
       <c r="AK28" s="16">
-        <f>IF(OR(AG28="",AB28="",(AB28+AI28)=0),"",(AG28-AB28-AI28)/(AB28+AI28))</f>
+        <f>IF(OR(AG28="",AB28=""),"",IF((AB28+N(AI28))=0,"",(AG28-AB28-N(AI28))/(AB28+N(AI28))))</f>
         <v/>
       </c>
       <c r="AL28" s="15" t="n"/>
@@ -4737,7 +4737,7 @@
         <v/>
       </c>
       <c r="AP28" s="16">
-        <f>IF(OR(AL28="",AG28="",(AG28+AN28)=0),"",(AL28-AG28-AN28)/(AG28+AN28))</f>
+        <f>IF(OR(AL28="",AG28=""),"",IF((AG28+N(AN28))=0,"",(AL28-AG28-N(AN28))/(AG28+N(AN28))))</f>
         <v/>
       </c>
       <c r="AQ28" s="15" t="n"/>
@@ -4748,7 +4748,7 @@
         <v/>
       </c>
       <c r="AU28" s="16">
-        <f>IF(OR(AQ28="",AL28="",(AL28+AS28)=0),"",(AQ28-AL28-AS28)/(AL28+AS28))</f>
+        <f>IF(OR(AQ28="",AL28=""),"",IF((AL28+N(AS28))=0,"",(AQ28-AL28-N(AS28))/(AL28+N(AS28))))</f>
         <v/>
       </c>
       <c r="AV28" s="15" t="n"/>
@@ -4759,7 +4759,7 @@
         <v/>
       </c>
       <c r="AZ28" s="16">
-        <f>IF(OR(AV28="",AQ28="",(AQ28+AX28)=0),"",(AV28-AQ28-AX28)/(AQ28+AX28))</f>
+        <f>IF(OR(AV28="",AQ28=""),"",IF((AQ28+N(AX28))=0,"",(AV28-AQ28-N(AX28))/(AQ28+N(AX28))))</f>
         <v/>
       </c>
       <c r="BA28" s="15" t="n"/>
@@ -4770,7 +4770,7 @@
         <v/>
       </c>
       <c r="BE28" s="16">
-        <f>IF(OR(BA28="",AV28="",(AV28+BC28)=0),"",(BA28-AV28-BC28)/(AV28+BC28))</f>
+        <f>IF(OR(BA28="",AV28=""),"",IF((AV28+N(BC28))=0,"",(BA28-AV28-N(BC28))/(AV28+N(BC28))))</f>
         <v/>
       </c>
       <c r="BF28" s="15" t="n"/>
@@ -4781,7 +4781,7 @@
         <v/>
       </c>
       <c r="BJ28" s="16">
-        <f>IF(OR(BF28="",BA28="",(BA28+BH28)=0),"",(BF28-BA28-BH28)/(BA28+BH28))</f>
+        <f>IF(OR(BF28="",BA28=""),"",IF((BA28+N(BH28))=0,"",(BF28-BA28-N(BH28))/(BA28+N(BH28))))</f>
         <v/>
       </c>
     </row>
@@ -4796,7 +4796,7 @@
         <v/>
       </c>
       <c r="G29" s="19">
-        <f>IF(OR(C29="",B29="",(B29+E29)=0),"",(C29-B29-E29)/(B29+E29))</f>
+        <f>IF(OR(C29="",B29=""),"",IF((B29+N(E29))=0,"",(C29-B29-N(E29))/(B29+N(E29))))</f>
         <v/>
       </c>
       <c r="H29" s="18" t="n"/>
@@ -4807,7 +4807,7 @@
         <v/>
       </c>
       <c r="L29" s="19">
-        <f>IF(OR(H29="",C29="",(C29+J29)=0),"",(H29-C29-J29)/(C29+J29))</f>
+        <f>IF(OR(H29="",C29=""),"",IF((C29+N(J29))=0,"",(H29-C29-N(J29))/(C29+N(J29))))</f>
         <v/>
       </c>
       <c r="M29" s="18" t="n"/>
@@ -4818,7 +4818,7 @@
         <v/>
       </c>
       <c r="Q29" s="19">
-        <f>IF(OR(M29="",H29="",(H29+O29)=0),"",(M29-H29-O29)/(H29+O29))</f>
+        <f>IF(OR(M29="",H29=""),"",IF((H29+N(O29))=0,"",(M29-H29-N(O29))/(H29+N(O29))))</f>
         <v/>
       </c>
       <c r="R29" s="18" t="n"/>
@@ -4829,7 +4829,7 @@
         <v/>
       </c>
       <c r="V29" s="19">
-        <f>IF(OR(R29="",M29="",(M29+T29)=0),"",(R29-M29-T29)/(M29+T29))</f>
+        <f>IF(OR(R29="",M29=""),"",IF((M29+N(T29))=0,"",(R29-M29-N(T29))/(M29+N(T29))))</f>
         <v/>
       </c>
       <c r="W29" s="18" t="n"/>
@@ -4840,7 +4840,7 @@
         <v/>
       </c>
       <c r="AA29" s="19">
-        <f>IF(OR(W29="",R29="",(R29+Y29)=0),"",(W29-R29-Y29)/(R29+Y29))</f>
+        <f>IF(OR(W29="",R29=""),"",IF((R29+N(Y29))=0,"",(W29-R29-N(Y29))/(R29+N(Y29))))</f>
         <v/>
       </c>
       <c r="AB29" s="18" t="n"/>
@@ -4851,7 +4851,7 @@
         <v/>
       </c>
       <c r="AF29" s="19">
-        <f>IF(OR(AB29="",W29="",(W29+AD29)=0),"",(AB29-W29-AD29)/(W29+AD29))</f>
+        <f>IF(OR(AB29="",W29=""),"",IF((W29+N(AD29))=0,"",(AB29-W29-N(AD29))/(W29+N(AD29))))</f>
         <v/>
       </c>
       <c r="AG29" s="18" t="n"/>
@@ -4862,7 +4862,7 @@
         <v/>
       </c>
       <c r="AK29" s="19">
-        <f>IF(OR(AG29="",AB29="",(AB29+AI29)=0),"",(AG29-AB29-AI29)/(AB29+AI29))</f>
+        <f>IF(OR(AG29="",AB29=""),"",IF((AB29+N(AI29))=0,"",(AG29-AB29-N(AI29))/(AB29+N(AI29))))</f>
         <v/>
       </c>
       <c r="AL29" s="18" t="n"/>
@@ -4873,7 +4873,7 @@
         <v/>
       </c>
       <c r="AP29" s="19">
-        <f>IF(OR(AL29="",AG29="",(AG29+AN29)=0),"",(AL29-AG29-AN29)/(AG29+AN29))</f>
+        <f>IF(OR(AL29="",AG29=""),"",IF((AG29+N(AN29))=0,"",(AL29-AG29-N(AN29))/(AG29+N(AN29))))</f>
         <v/>
       </c>
       <c r="AQ29" s="18" t="n"/>
@@ -4884,7 +4884,7 @@
         <v/>
       </c>
       <c r="AU29" s="19">
-        <f>IF(OR(AQ29="",AL29="",(AL29+AS29)=0),"",(AQ29-AL29-AS29)/(AL29+AS29))</f>
+        <f>IF(OR(AQ29="",AL29=""),"",IF((AL29+N(AS29))=0,"",(AQ29-AL29-N(AS29))/(AL29+N(AS29))))</f>
         <v/>
       </c>
       <c r="AV29" s="18" t="n"/>
@@ -4895,7 +4895,7 @@
         <v/>
       </c>
       <c r="AZ29" s="19">
-        <f>IF(OR(AV29="",AQ29="",(AQ29+AX29)=0),"",(AV29-AQ29-AX29)/(AQ29+AX29))</f>
+        <f>IF(OR(AV29="",AQ29=""),"",IF((AQ29+N(AX29))=0,"",(AV29-AQ29-N(AX29))/(AQ29+N(AX29))))</f>
         <v/>
       </c>
       <c r="BA29" s="18" t="n"/>
@@ -4906,7 +4906,7 @@
         <v/>
       </c>
       <c r="BE29" s="19">
-        <f>IF(OR(BA29="",AV29="",(AV29+BC29)=0),"",(BA29-AV29-BC29)/(AV29+BC29))</f>
+        <f>IF(OR(BA29="",AV29=""),"",IF((AV29+N(BC29))=0,"",(BA29-AV29-N(BC29))/(AV29+N(BC29))))</f>
         <v/>
       </c>
       <c r="BF29" s="18" t="n"/>
@@ -4917,7 +4917,7 @@
         <v/>
       </c>
       <c r="BJ29" s="19">
-        <f>IF(OR(BF29="",BA29="",(BA29+BH29)=0),"",(BF29-BA29-BH29)/(BA29+BH29))</f>
+        <f>IF(OR(BF29="",BA29=""),"",IF((BA29+N(BH29))=0,"",(BF29-BA29-N(BH29))/(BA29+N(BH29))))</f>
         <v/>
       </c>
     </row>
@@ -4948,7 +4948,7 @@
         <v/>
       </c>
       <c r="G30" s="13">
-        <f>IF(OR(C30="",B30="",(B30+E30)=0),"",(C30-B30-E30)/(B30+E30))</f>
+        <f>IF(OR(C30="",B30=""),"",IF((B30+N(E30))=0,"",(C30-B30-N(E30))/(B30+N(E30))))</f>
         <v/>
       </c>
       <c r="H30" s="12">
@@ -4968,7 +4968,7 @@
         <v/>
       </c>
       <c r="L30" s="13">
-        <f>IF(OR(H30="",C30="",(C30+J30)=0),"",(H30-C30-J30)/(C30+J30))</f>
+        <f>IF(OR(H30="",C30=""),"",IF((C30+N(J30))=0,"",(H30-C30-N(J30))/(C30+N(J30))))</f>
         <v/>
       </c>
       <c r="M30" s="12">
@@ -4988,7 +4988,7 @@
         <v/>
       </c>
       <c r="Q30" s="13">
-        <f>IF(OR(M30="",H30="",(H30+O30)=0),"",(M30-H30-O30)/(H30+O30))</f>
+        <f>IF(OR(M30="",H30=""),"",IF((H30+N(O30))=0,"",(M30-H30-N(O30))/(H30+N(O30))))</f>
         <v/>
       </c>
       <c r="R30" s="12">
@@ -5008,7 +5008,7 @@
         <v/>
       </c>
       <c r="V30" s="13">
-        <f>IF(OR(R30="",M30="",(M30+T30)=0),"",(R30-M30-T30)/(M30+T30))</f>
+        <f>IF(OR(R30="",M30=""),"",IF((M30+N(T30))=0,"",(R30-M30-N(T30))/(M30+N(T30))))</f>
         <v/>
       </c>
       <c r="W30" s="12">
@@ -5028,7 +5028,7 @@
         <v/>
       </c>
       <c r="AA30" s="13">
-        <f>IF(OR(W30="",R30="",(R30+Y30)=0),"",(W30-R30-Y30)/(R30+Y30))</f>
+        <f>IF(OR(W30="",R30=""),"",IF((R30+N(Y30))=0,"",(W30-R30-N(Y30))/(R30+N(Y30))))</f>
         <v/>
       </c>
       <c r="AB30" s="12">
@@ -5048,7 +5048,7 @@
         <v/>
       </c>
       <c r="AF30" s="13">
-        <f>IF(OR(AB30="",W30="",(W30+AD30)=0),"",(AB30-W30-AD30)/(W30+AD30))</f>
+        <f>IF(OR(AB30="",W30=""),"",IF((W30+N(AD30))=0,"",(AB30-W30-N(AD30))/(W30+N(AD30))))</f>
         <v/>
       </c>
       <c r="AG30" s="12">
@@ -5068,7 +5068,7 @@
         <v/>
       </c>
       <c r="AK30" s="13">
-        <f>IF(OR(AG30="",AB30="",(AB30+AI30)=0),"",(AG30-AB30-AI30)/(AB30+AI30))</f>
+        <f>IF(OR(AG30="",AB30=""),"",IF((AB30+N(AI30))=0,"",(AG30-AB30-N(AI30))/(AB30+N(AI30))))</f>
         <v/>
       </c>
       <c r="AL30" s="12">
@@ -5088,7 +5088,7 @@
         <v/>
       </c>
       <c r="AP30" s="13">
-        <f>IF(OR(AL30="",AG30="",(AG30+AN30)=0),"",(AL30-AG30-AN30)/(AG30+AN30))</f>
+        <f>IF(OR(AL30="",AG30=""),"",IF((AG30+N(AN30))=0,"",(AL30-AG30-N(AN30))/(AG30+N(AN30))))</f>
         <v/>
       </c>
       <c r="AQ30" s="12">
@@ -5108,7 +5108,7 @@
         <v/>
       </c>
       <c r="AU30" s="13">
-        <f>IF(OR(AQ30="",AL30="",(AL30+AS30)=0),"",(AQ30-AL30-AS30)/(AL30+AS30))</f>
+        <f>IF(OR(AQ30="",AL30=""),"",IF((AL30+N(AS30))=0,"",(AQ30-AL30-N(AS30))/(AL30+N(AS30))))</f>
         <v/>
       </c>
       <c r="AV30" s="12">
@@ -5128,7 +5128,7 @@
         <v/>
       </c>
       <c r="AZ30" s="13">
-        <f>IF(OR(AV30="",AQ30="",(AQ30+AX30)=0),"",(AV30-AQ30-AX30)/(AQ30+AX30))</f>
+        <f>IF(OR(AV30="",AQ30=""),"",IF((AQ30+N(AX30))=0,"",(AV30-AQ30-N(AX30))/(AQ30+N(AX30))))</f>
         <v/>
       </c>
       <c r="BA30" s="12">
@@ -5148,7 +5148,7 @@
         <v/>
       </c>
       <c r="BE30" s="13">
-        <f>IF(OR(BA30="",AV30="",(AV30+BC30)=0),"",(BA30-AV30-BC30)/(AV30+BC30))</f>
+        <f>IF(OR(BA30="",AV30=""),"",IF((AV30+N(BC30))=0,"",(BA30-AV30-N(BC30))/(AV30+N(BC30))))</f>
         <v/>
       </c>
       <c r="BF30" s="12">
@@ -5168,7 +5168,7 @@
         <v/>
       </c>
       <c r="BJ30" s="13">
-        <f>IF(OR(BF30="",BA30="",(BA30+BH30)=0),"",(BF30-BA30-BH30)/(BA30+BH30))</f>
+        <f>IF(OR(BF30="",BA30=""),"",IF((BA30+N(BH30))=0,"",(BF30-BA30-N(BH30))/(BA30+N(BH30))))</f>
         <v/>
       </c>
     </row>
@@ -5183,7 +5183,7 @@
         <v/>
       </c>
       <c r="G31" s="16">
-        <f>IF(OR(C31="",B31="",(B31+E31)=0),"",(C31-B31-E31)/(B31+E31))</f>
+        <f>IF(OR(C31="",B31=""),"",IF((B31+N(E31))=0,"",(C31-B31-N(E31))/(B31+N(E31))))</f>
         <v/>
       </c>
       <c r="H31" s="15" t="n"/>
@@ -5194,7 +5194,7 @@
         <v/>
       </c>
       <c r="L31" s="16">
-        <f>IF(OR(H31="",C31="",(C31+J31)=0),"",(H31-C31-J31)/(C31+J31))</f>
+        <f>IF(OR(H31="",C31=""),"",IF((C31+N(J31))=0,"",(H31-C31-N(J31))/(C31+N(J31))))</f>
         <v/>
       </c>
       <c r="M31" s="15" t="n"/>
@@ -5205,7 +5205,7 @@
         <v/>
       </c>
       <c r="Q31" s="16">
-        <f>IF(OR(M31="",H31="",(H31+O31)=0),"",(M31-H31-O31)/(H31+O31))</f>
+        <f>IF(OR(M31="",H31=""),"",IF((H31+N(O31))=0,"",(M31-H31-N(O31))/(H31+N(O31))))</f>
         <v/>
       </c>
       <c r="R31" s="15" t="n"/>
@@ -5216,7 +5216,7 @@
         <v/>
       </c>
       <c r="V31" s="16">
-        <f>IF(OR(R31="",M31="",(M31+T31)=0),"",(R31-M31-T31)/(M31+T31))</f>
+        <f>IF(OR(R31="",M31=""),"",IF((M31+N(T31))=0,"",(R31-M31-N(T31))/(M31+N(T31))))</f>
         <v/>
       </c>
       <c r="W31" s="15" t="n"/>
@@ -5227,7 +5227,7 @@
         <v/>
       </c>
       <c r="AA31" s="16">
-        <f>IF(OR(W31="",R31="",(R31+Y31)=0),"",(W31-R31-Y31)/(R31+Y31))</f>
+        <f>IF(OR(W31="",R31=""),"",IF((R31+N(Y31))=0,"",(W31-R31-N(Y31))/(R31+N(Y31))))</f>
         <v/>
       </c>
       <c r="AB31" s="15" t="n"/>
@@ -5238,7 +5238,7 @@
         <v/>
       </c>
       <c r="AF31" s="16">
-        <f>IF(OR(AB31="",W31="",(W31+AD31)=0),"",(AB31-W31-AD31)/(W31+AD31))</f>
+        <f>IF(OR(AB31="",W31=""),"",IF((W31+N(AD31))=0,"",(AB31-W31-N(AD31))/(W31+N(AD31))))</f>
         <v/>
       </c>
       <c r="AG31" s="15" t="n"/>
@@ -5249,7 +5249,7 @@
         <v/>
       </c>
       <c r="AK31" s="16">
-        <f>IF(OR(AG31="",AB31="",(AB31+AI31)=0),"",(AG31-AB31-AI31)/(AB31+AI31))</f>
+        <f>IF(OR(AG31="",AB31=""),"",IF((AB31+N(AI31))=0,"",(AG31-AB31-N(AI31))/(AB31+N(AI31))))</f>
         <v/>
       </c>
       <c r="AL31" s="15" t="n"/>
@@ -5260,7 +5260,7 @@
         <v/>
       </c>
       <c r="AP31" s="16">
-        <f>IF(OR(AL31="",AG31="",(AG31+AN31)=0),"",(AL31-AG31-AN31)/(AG31+AN31))</f>
+        <f>IF(OR(AL31="",AG31=""),"",IF((AG31+N(AN31))=0,"",(AL31-AG31-N(AN31))/(AG31+N(AN31))))</f>
         <v/>
       </c>
       <c r="AQ31" s="15" t="n"/>
@@ -5271,7 +5271,7 @@
         <v/>
       </c>
       <c r="AU31" s="16">
-        <f>IF(OR(AQ31="",AL31="",(AL31+AS31)=0),"",(AQ31-AL31-AS31)/(AL31+AS31))</f>
+        <f>IF(OR(AQ31="",AL31=""),"",IF((AL31+N(AS31))=0,"",(AQ31-AL31-N(AS31))/(AL31+N(AS31))))</f>
         <v/>
       </c>
       <c r="AV31" s="15" t="n"/>
@@ -5282,7 +5282,7 @@
         <v/>
       </c>
       <c r="AZ31" s="16">
-        <f>IF(OR(AV31="",AQ31="",(AQ31+AX31)=0),"",(AV31-AQ31-AX31)/(AQ31+AX31))</f>
+        <f>IF(OR(AV31="",AQ31=""),"",IF((AQ31+N(AX31))=0,"",(AV31-AQ31-N(AX31))/(AQ31+N(AX31))))</f>
         <v/>
       </c>
       <c r="BA31" s="15" t="n"/>
@@ -5293,7 +5293,7 @@
         <v/>
       </c>
       <c r="BE31" s="16">
-        <f>IF(OR(BA31="",AV31="",(AV31+BC31)=0),"",(BA31-AV31-BC31)/(AV31+BC31))</f>
+        <f>IF(OR(BA31="",AV31=""),"",IF((AV31+N(BC31))=0,"",(BA31-AV31-N(BC31))/(AV31+N(BC31))))</f>
         <v/>
       </c>
       <c r="BF31" s="15" t="n"/>
@@ -5304,7 +5304,7 @@
         <v/>
       </c>
       <c r="BJ31" s="16">
-        <f>IF(OR(BF31="",BA31="",(BA31+BH31)=0),"",(BF31-BA31-BH31)/(BA31+BH31))</f>
+        <f>IF(OR(BF31="",BA31=""),"",IF((BA31+N(BH31))=0,"",(BF31-BA31-N(BH31))/(BA31+N(BH31))))</f>
         <v/>
       </c>
     </row>
@@ -5319,7 +5319,7 @@
         <v/>
       </c>
       <c r="G32" s="19">
-        <f>IF(OR(C32="",B32="",(B32+E32)=0),"",(C32-B32-E32)/(B32+E32))</f>
+        <f>IF(OR(C32="",B32=""),"",IF((B32+N(E32))=0,"",(C32-B32-N(E32))/(B32+N(E32))))</f>
         <v/>
       </c>
       <c r="H32" s="18" t="n"/>
@@ -5330,7 +5330,7 @@
         <v/>
       </c>
       <c r="L32" s="19">
-        <f>IF(OR(H32="",C32="",(C32+J32)=0),"",(H32-C32-J32)/(C32+J32))</f>
+        <f>IF(OR(H32="",C32=""),"",IF((C32+N(J32))=0,"",(H32-C32-N(J32))/(C32+N(J32))))</f>
         <v/>
       </c>
       <c r="M32" s="18" t="n"/>
@@ -5341,7 +5341,7 @@
         <v/>
       </c>
       <c r="Q32" s="19">
-        <f>IF(OR(M32="",H32="",(H32+O32)=0),"",(M32-H32-O32)/(H32+O32))</f>
+        <f>IF(OR(M32="",H32=""),"",IF((H32+N(O32))=0,"",(M32-H32-N(O32))/(H32+N(O32))))</f>
         <v/>
       </c>
       <c r="R32" s="18" t="n"/>
@@ -5352,7 +5352,7 @@
         <v/>
       </c>
       <c r="V32" s="19">
-        <f>IF(OR(R32="",M32="",(M32+T32)=0),"",(R32-M32-T32)/(M32+T32))</f>
+        <f>IF(OR(R32="",M32=""),"",IF((M32+N(T32))=0,"",(R32-M32-N(T32))/(M32+N(T32))))</f>
         <v/>
       </c>
       <c r="W32" s="18" t="n"/>
@@ -5363,7 +5363,7 @@
         <v/>
       </c>
       <c r="AA32" s="19">
-        <f>IF(OR(W32="",R32="",(R32+Y32)=0),"",(W32-R32-Y32)/(R32+Y32))</f>
+        <f>IF(OR(W32="",R32=""),"",IF((R32+N(Y32))=0,"",(W32-R32-N(Y32))/(R32+N(Y32))))</f>
         <v/>
       </c>
       <c r="AB32" s="18" t="n"/>
@@ -5374,7 +5374,7 @@
         <v/>
       </c>
       <c r="AF32" s="19">
-        <f>IF(OR(AB32="",W32="",(W32+AD32)=0),"",(AB32-W32-AD32)/(W32+AD32))</f>
+        <f>IF(OR(AB32="",W32=""),"",IF((W32+N(AD32))=0,"",(AB32-W32-N(AD32))/(W32+N(AD32))))</f>
         <v/>
       </c>
       <c r="AG32" s="18" t="n"/>
@@ -5385,7 +5385,7 @@
         <v/>
       </c>
       <c r="AK32" s="19">
-        <f>IF(OR(AG32="",AB32="",(AB32+AI32)=0),"",(AG32-AB32-AI32)/(AB32+AI32))</f>
+        <f>IF(OR(AG32="",AB32=""),"",IF((AB32+N(AI32))=0,"",(AG32-AB32-N(AI32))/(AB32+N(AI32))))</f>
         <v/>
       </c>
       <c r="AL32" s="18" t="n"/>
@@ -5396,7 +5396,7 @@
         <v/>
       </c>
       <c r="AP32" s="19">
-        <f>IF(OR(AL32="",AG32="",(AG32+AN32)=0),"",(AL32-AG32-AN32)/(AG32+AN32))</f>
+        <f>IF(OR(AL32="",AG32=""),"",IF((AG32+N(AN32))=0,"",(AL32-AG32-N(AN32))/(AG32+N(AN32))))</f>
         <v/>
       </c>
       <c r="AQ32" s="18" t="n"/>
@@ -5407,7 +5407,7 @@
         <v/>
       </c>
       <c r="AU32" s="19">
-        <f>IF(OR(AQ32="",AL32="",(AL32+AS32)=0),"",(AQ32-AL32-AS32)/(AL32+AS32))</f>
+        <f>IF(OR(AQ32="",AL32=""),"",IF((AL32+N(AS32))=0,"",(AQ32-AL32-N(AS32))/(AL32+N(AS32))))</f>
         <v/>
       </c>
       <c r="AV32" s="18" t="n"/>
@@ -5418,7 +5418,7 @@
         <v/>
       </c>
       <c r="AZ32" s="19">
-        <f>IF(OR(AV32="",AQ32="",(AQ32+AX32)=0),"",(AV32-AQ32-AX32)/(AQ32+AX32))</f>
+        <f>IF(OR(AV32="",AQ32=""),"",IF((AQ32+N(AX32))=0,"",(AV32-AQ32-N(AX32))/(AQ32+N(AX32))))</f>
         <v/>
       </c>
       <c r="BA32" s="18" t="n"/>
@@ -5429,7 +5429,7 @@
         <v/>
       </c>
       <c r="BE32" s="19">
-        <f>IF(OR(BA32="",AV32="",(AV32+BC32)=0),"",(BA32-AV32-BC32)/(AV32+BC32))</f>
+        <f>IF(OR(BA32="",AV32=""),"",IF((AV32+N(BC32))=0,"",(BA32-AV32-N(BC32))/(AV32+N(BC32))))</f>
         <v/>
       </c>
       <c r="BF32" s="18" t="n"/>
@@ -5440,7 +5440,7 @@
         <v/>
       </c>
       <c r="BJ32" s="19">
-        <f>IF(OR(BF32="",BA32="",(BA32+BH32)=0),"",(BF32-BA32-BH32)/(BA32+BH32))</f>
+        <f>IF(OR(BF32="",BA32=""),"",IF((BA32+N(BH32))=0,"",(BF32-BA32-N(BH32))/(BA32+N(BH32))))</f>
         <v/>
       </c>
     </row>
@@ -5455,7 +5455,7 @@
         <v/>
       </c>
       <c r="G33" s="16">
-        <f>IF(OR(C33="",B33="",(B33+E33)=0),"",(C33-B33-E33)/(B33+E33))</f>
+        <f>IF(OR(C33="",B33=""),"",IF((B33+N(E33))=0,"",(C33-B33-N(E33))/(B33+N(E33))))</f>
         <v/>
       </c>
       <c r="H33" s="15" t="n"/>
@@ -5466,7 +5466,7 @@
         <v/>
       </c>
       <c r="L33" s="16">
-        <f>IF(OR(H33="",C33="",(C33+J33)=0),"",(H33-C33-J33)/(C33+J33))</f>
+        <f>IF(OR(H33="",C33=""),"",IF((C33+N(J33))=0,"",(H33-C33-N(J33))/(C33+N(J33))))</f>
         <v/>
       </c>
       <c r="M33" s="15" t="n"/>
@@ -5477,7 +5477,7 @@
         <v/>
       </c>
       <c r="Q33" s="16">
-        <f>IF(OR(M33="",H33="",(H33+O33)=0),"",(M33-H33-O33)/(H33+O33))</f>
+        <f>IF(OR(M33="",H33=""),"",IF((H33+N(O33))=0,"",(M33-H33-N(O33))/(H33+N(O33))))</f>
         <v/>
       </c>
       <c r="R33" s="15" t="n"/>
@@ -5488,7 +5488,7 @@
         <v/>
       </c>
       <c r="V33" s="16">
-        <f>IF(OR(R33="",M33="",(M33+T33)=0),"",(R33-M33-T33)/(M33+T33))</f>
+        <f>IF(OR(R33="",M33=""),"",IF((M33+N(T33))=0,"",(R33-M33-N(T33))/(M33+N(T33))))</f>
         <v/>
       </c>
       <c r="W33" s="15" t="n"/>
@@ -5499,7 +5499,7 @@
         <v/>
       </c>
       <c r="AA33" s="16">
-        <f>IF(OR(W33="",R33="",(R33+Y33)=0),"",(W33-R33-Y33)/(R33+Y33))</f>
+        <f>IF(OR(W33="",R33=""),"",IF((R33+N(Y33))=0,"",(W33-R33-N(Y33))/(R33+N(Y33))))</f>
         <v/>
       </c>
       <c r="AB33" s="15" t="n"/>
@@ -5510,7 +5510,7 @@
         <v/>
       </c>
       <c r="AF33" s="16">
-        <f>IF(OR(AB33="",W33="",(W33+AD33)=0),"",(AB33-W33-AD33)/(W33+AD33))</f>
+        <f>IF(OR(AB33="",W33=""),"",IF((W33+N(AD33))=0,"",(AB33-W33-N(AD33))/(W33+N(AD33))))</f>
         <v/>
       </c>
       <c r="AG33" s="15" t="n"/>
@@ -5521,7 +5521,7 @@
         <v/>
       </c>
       <c r="AK33" s="16">
-        <f>IF(OR(AG33="",AB33="",(AB33+AI33)=0),"",(AG33-AB33-AI33)/(AB33+AI33))</f>
+        <f>IF(OR(AG33="",AB33=""),"",IF((AB33+N(AI33))=0,"",(AG33-AB33-N(AI33))/(AB33+N(AI33))))</f>
         <v/>
       </c>
       <c r="AL33" s="15" t="n"/>
@@ -5532,7 +5532,7 @@
         <v/>
       </c>
       <c r="AP33" s="16">
-        <f>IF(OR(AL33="",AG33="",(AG33+AN33)=0),"",(AL33-AG33-AN33)/(AG33+AN33))</f>
+        <f>IF(OR(AL33="",AG33=""),"",IF((AG33+N(AN33))=0,"",(AL33-AG33-N(AN33))/(AG33+N(AN33))))</f>
         <v/>
       </c>
       <c r="AQ33" s="15" t="n"/>
@@ -5543,7 +5543,7 @@
         <v/>
       </c>
       <c r="AU33" s="16">
-        <f>IF(OR(AQ33="",AL33="",(AL33+AS33)=0),"",(AQ33-AL33-AS33)/(AL33+AS33))</f>
+        <f>IF(OR(AQ33="",AL33=""),"",IF((AL33+N(AS33))=0,"",(AQ33-AL33-N(AS33))/(AL33+N(AS33))))</f>
         <v/>
       </c>
       <c r="AV33" s="15" t="n"/>
@@ -5554,7 +5554,7 @@
         <v/>
       </c>
       <c r="AZ33" s="16">
-        <f>IF(OR(AV33="",AQ33="",(AQ33+AX33)=0),"",(AV33-AQ33-AX33)/(AQ33+AX33))</f>
+        <f>IF(OR(AV33="",AQ33=""),"",IF((AQ33+N(AX33))=0,"",(AV33-AQ33-N(AX33))/(AQ33+N(AX33))))</f>
         <v/>
       </c>
       <c r="BA33" s="15" t="n"/>
@@ -5565,7 +5565,7 @@
         <v/>
       </c>
       <c r="BE33" s="16">
-        <f>IF(OR(BA33="",AV33="",(AV33+BC33)=0),"",(BA33-AV33-BC33)/(AV33+BC33))</f>
+        <f>IF(OR(BA33="",AV33=""),"",IF((AV33+N(BC33))=0,"",(BA33-AV33-N(BC33))/(AV33+N(BC33))))</f>
         <v/>
       </c>
       <c r="BF33" s="15" t="n"/>
@@ -5576,7 +5576,7 @@
         <v/>
       </c>
       <c r="BJ33" s="16">
-        <f>IF(OR(BF33="",BA33="",(BA33+BH33)=0),"",(BF33-BA33-BH33)/(BA33+BH33))</f>
+        <f>IF(OR(BF33="",BA33=""),"",IF((BA33+N(BH33))=0,"",(BF33-BA33-N(BH33))/(BA33+N(BH33))))</f>
         <v/>
       </c>
     </row>
@@ -5591,7 +5591,7 @@
         <v/>
       </c>
       <c r="G34" s="19">
-        <f>IF(OR(C34="",B34="",(B34+E34)=0),"",(C34-B34-E34)/(B34+E34))</f>
+        <f>IF(OR(C34="",B34=""),"",IF((B34+N(E34))=0,"",(C34-B34-N(E34))/(B34+N(E34))))</f>
         <v/>
       </c>
       <c r="H34" s="18" t="n"/>
@@ -5602,7 +5602,7 @@
         <v/>
       </c>
       <c r="L34" s="19">
-        <f>IF(OR(H34="",C34="",(C34+J34)=0),"",(H34-C34-J34)/(C34+J34))</f>
+        <f>IF(OR(H34="",C34=""),"",IF((C34+N(J34))=0,"",(H34-C34-N(J34))/(C34+N(J34))))</f>
         <v/>
       </c>
       <c r="M34" s="18" t="n"/>
@@ -5613,7 +5613,7 @@
         <v/>
       </c>
       <c r="Q34" s="19">
-        <f>IF(OR(M34="",H34="",(H34+O34)=0),"",(M34-H34-O34)/(H34+O34))</f>
+        <f>IF(OR(M34="",H34=""),"",IF((H34+N(O34))=0,"",(M34-H34-N(O34))/(H34+N(O34))))</f>
         <v/>
       </c>
       <c r="R34" s="18" t="n"/>
@@ -5624,7 +5624,7 @@
         <v/>
       </c>
       <c r="V34" s="19">
-        <f>IF(OR(R34="",M34="",(M34+T34)=0),"",(R34-M34-T34)/(M34+T34))</f>
+        <f>IF(OR(R34="",M34=""),"",IF((M34+N(T34))=0,"",(R34-M34-N(T34))/(M34+N(T34))))</f>
         <v/>
       </c>
       <c r="W34" s="18" t="n"/>
@@ -5635,7 +5635,7 @@
         <v/>
       </c>
       <c r="AA34" s="19">
-        <f>IF(OR(W34="",R34="",(R34+Y34)=0),"",(W34-R34-Y34)/(R34+Y34))</f>
+        <f>IF(OR(W34="",R34=""),"",IF((R34+N(Y34))=0,"",(W34-R34-N(Y34))/(R34+N(Y34))))</f>
         <v/>
       </c>
       <c r="AB34" s="18" t="n"/>
@@ -5646,7 +5646,7 @@
         <v/>
       </c>
       <c r="AF34" s="19">
-        <f>IF(OR(AB34="",W34="",(W34+AD34)=0),"",(AB34-W34-AD34)/(W34+AD34))</f>
+        <f>IF(OR(AB34="",W34=""),"",IF((W34+N(AD34))=0,"",(AB34-W34-N(AD34))/(W34+N(AD34))))</f>
         <v/>
       </c>
       <c r="AG34" s="18" t="n"/>
@@ -5657,7 +5657,7 @@
         <v/>
       </c>
       <c r="AK34" s="19">
-        <f>IF(OR(AG34="",AB34="",(AB34+AI34)=0),"",(AG34-AB34-AI34)/(AB34+AI34))</f>
+        <f>IF(OR(AG34="",AB34=""),"",IF((AB34+N(AI34))=0,"",(AG34-AB34-N(AI34))/(AB34+N(AI34))))</f>
         <v/>
       </c>
       <c r="AL34" s="18" t="n"/>
@@ -5668,7 +5668,7 @@
         <v/>
       </c>
       <c r="AP34" s="19">
-        <f>IF(OR(AL34="",AG34="",(AG34+AN34)=0),"",(AL34-AG34-AN34)/(AG34+AN34))</f>
+        <f>IF(OR(AL34="",AG34=""),"",IF((AG34+N(AN34))=0,"",(AL34-AG34-N(AN34))/(AG34+N(AN34))))</f>
         <v/>
       </c>
       <c r="AQ34" s="18" t="n"/>
@@ -5679,7 +5679,7 @@
         <v/>
       </c>
       <c r="AU34" s="19">
-        <f>IF(OR(AQ34="",AL34="",(AL34+AS34)=0),"",(AQ34-AL34-AS34)/(AL34+AS34))</f>
+        <f>IF(OR(AQ34="",AL34=""),"",IF((AL34+N(AS34))=0,"",(AQ34-AL34-N(AS34))/(AL34+N(AS34))))</f>
         <v/>
       </c>
       <c r="AV34" s="18" t="n"/>
@@ -5690,7 +5690,7 @@
         <v/>
       </c>
       <c r="AZ34" s="19">
-        <f>IF(OR(AV34="",AQ34="",(AQ34+AX34)=0),"",(AV34-AQ34-AX34)/(AQ34+AX34))</f>
+        <f>IF(OR(AV34="",AQ34=""),"",IF((AQ34+N(AX34))=0,"",(AV34-AQ34-N(AX34))/(AQ34+N(AX34))))</f>
         <v/>
       </c>
       <c r="BA34" s="18" t="n"/>
@@ -5701,7 +5701,7 @@
         <v/>
       </c>
       <c r="BE34" s="19">
-        <f>IF(OR(BA34="",AV34="",(AV34+BC34)=0),"",(BA34-AV34-BC34)/(AV34+BC34))</f>
+        <f>IF(OR(BA34="",AV34=""),"",IF((AV34+N(BC34))=0,"",(BA34-AV34-N(BC34))/(AV34+N(BC34))))</f>
         <v/>
       </c>
       <c r="BF34" s="18" t="n"/>
@@ -5712,7 +5712,7 @@
         <v/>
       </c>
       <c r="BJ34" s="19">
-        <f>IF(OR(BF34="",BA34="",(BA34+BH34)=0),"",(BF34-BA34-BH34)/(BA34+BH34))</f>
+        <f>IF(OR(BF34="",BA34=""),"",IF((BA34+N(BH34))=0,"",(BF34-BA34-N(BH34))/(BA34+N(BH34))))</f>
         <v/>
       </c>
     </row>
@@ -5743,7 +5743,7 @@
         <v/>
       </c>
       <c r="G35" s="13">
-        <f>IF(OR(C35="",B35="",(B35+E35)=0),"",(C35-B35-E35)/(B35+E35))</f>
+        <f>IF(OR(C35="",B35=""),"",IF((B35+N(E35))=0,"",(C35-B35-N(E35))/(B35+N(E35))))</f>
         <v/>
       </c>
       <c r="H35" s="12">
@@ -5763,7 +5763,7 @@
         <v/>
       </c>
       <c r="L35" s="13">
-        <f>IF(OR(H35="",C35="",(C35+J35)=0),"",(H35-C35-J35)/(C35+J35))</f>
+        <f>IF(OR(H35="",C35=""),"",IF((C35+N(J35))=0,"",(H35-C35-N(J35))/(C35+N(J35))))</f>
         <v/>
       </c>
       <c r="M35" s="12">
@@ -5783,7 +5783,7 @@
         <v/>
       </c>
       <c r="Q35" s="13">
-        <f>IF(OR(M35="",H35="",(H35+O35)=0),"",(M35-H35-O35)/(H35+O35))</f>
+        <f>IF(OR(M35="",H35=""),"",IF((H35+N(O35))=0,"",(M35-H35-N(O35))/(H35+N(O35))))</f>
         <v/>
       </c>
       <c r="R35" s="12">
@@ -5803,7 +5803,7 @@
         <v/>
       </c>
       <c r="V35" s="13">
-        <f>IF(OR(R35="",M35="",(M35+T35)=0),"",(R35-M35-T35)/(M35+T35))</f>
+        <f>IF(OR(R35="",M35=""),"",IF((M35+N(T35))=0,"",(R35-M35-N(T35))/(M35+N(T35))))</f>
         <v/>
       </c>
       <c r="W35" s="12">
@@ -5823,7 +5823,7 @@
         <v/>
       </c>
       <c r="AA35" s="13">
-        <f>IF(OR(W35="",R35="",(R35+Y35)=0),"",(W35-R35-Y35)/(R35+Y35))</f>
+        <f>IF(OR(W35="",R35=""),"",IF((R35+N(Y35))=0,"",(W35-R35-N(Y35))/(R35+N(Y35))))</f>
         <v/>
       </c>
       <c r="AB35" s="12">
@@ -5843,7 +5843,7 @@
         <v/>
       </c>
       <c r="AF35" s="13">
-        <f>IF(OR(AB35="",W35="",(W35+AD35)=0),"",(AB35-W35-AD35)/(W35+AD35))</f>
+        <f>IF(OR(AB35="",W35=""),"",IF((W35+N(AD35))=0,"",(AB35-W35-N(AD35))/(W35+N(AD35))))</f>
         <v/>
       </c>
       <c r="AG35" s="12">
@@ -5863,7 +5863,7 @@
         <v/>
       </c>
       <c r="AK35" s="13">
-        <f>IF(OR(AG35="",AB35="",(AB35+AI35)=0),"",(AG35-AB35-AI35)/(AB35+AI35))</f>
+        <f>IF(OR(AG35="",AB35=""),"",IF((AB35+N(AI35))=0,"",(AG35-AB35-N(AI35))/(AB35+N(AI35))))</f>
         <v/>
       </c>
       <c r="AL35" s="12">
@@ -5883,7 +5883,7 @@
         <v/>
       </c>
       <c r="AP35" s="13">
-        <f>IF(OR(AL35="",AG35="",(AG35+AN35)=0),"",(AL35-AG35-AN35)/(AG35+AN35))</f>
+        <f>IF(OR(AL35="",AG35=""),"",IF((AG35+N(AN35))=0,"",(AL35-AG35-N(AN35))/(AG35+N(AN35))))</f>
         <v/>
       </c>
       <c r="AQ35" s="12">
@@ -5903,7 +5903,7 @@
         <v/>
       </c>
       <c r="AU35" s="13">
-        <f>IF(OR(AQ35="",AL35="",(AL35+AS35)=0),"",(AQ35-AL35-AS35)/(AL35+AS35))</f>
+        <f>IF(OR(AQ35="",AL35=""),"",IF((AL35+N(AS35))=0,"",(AQ35-AL35-N(AS35))/(AL35+N(AS35))))</f>
         <v/>
       </c>
       <c r="AV35" s="12">
@@ -5923,7 +5923,7 @@
         <v/>
       </c>
       <c r="AZ35" s="13">
-        <f>IF(OR(AV35="",AQ35="",(AQ35+AX35)=0),"",(AV35-AQ35-AX35)/(AQ35+AX35))</f>
+        <f>IF(OR(AV35="",AQ35=""),"",IF((AQ35+N(AX35))=0,"",(AV35-AQ35-N(AX35))/(AQ35+N(AX35))))</f>
         <v/>
       </c>
       <c r="BA35" s="12">
@@ -5943,7 +5943,7 @@
         <v/>
       </c>
       <c r="BE35" s="13">
-        <f>IF(OR(BA35="",AV35="",(AV35+BC35)=0),"",(BA35-AV35-BC35)/(AV35+BC35))</f>
+        <f>IF(OR(BA35="",AV35=""),"",IF((AV35+N(BC35))=0,"",(BA35-AV35-N(BC35))/(AV35+N(BC35))))</f>
         <v/>
       </c>
       <c r="BF35" s="12">
@@ -5963,7 +5963,7 @@
         <v/>
       </c>
       <c r="BJ35" s="13">
-        <f>IF(OR(BF35="",BA35="",(BA35+BH35)=0),"",(BF35-BA35-BH35)/(BA35+BH35))</f>
+        <f>IF(OR(BF35="",BA35=""),"",IF((BA35+N(BH35))=0,"",(BF35-BA35-N(BH35))/(BA35+N(BH35))))</f>
         <v/>
       </c>
     </row>
@@ -5978,7 +5978,7 @@
         <v/>
       </c>
       <c r="G36" s="16">
-        <f>IF(OR(C36="",B36="",(B36+E36)=0),"",(C36-B36-E36)/(B36+E36))</f>
+        <f>IF(OR(C36="",B36=""),"",IF((B36+N(E36))=0,"",(C36-B36-N(E36))/(B36+N(E36))))</f>
         <v/>
       </c>
       <c r="H36" s="15" t="n"/>
@@ -5989,7 +5989,7 @@
         <v/>
       </c>
       <c r="L36" s="16">
-        <f>IF(OR(H36="",C36="",(C36+J36)=0),"",(H36-C36-J36)/(C36+J36))</f>
+        <f>IF(OR(H36="",C36=""),"",IF((C36+N(J36))=0,"",(H36-C36-N(J36))/(C36+N(J36))))</f>
         <v/>
       </c>
       <c r="M36" s="15" t="n"/>
@@ -6000,7 +6000,7 @@
         <v/>
       </c>
       <c r="Q36" s="16">
-        <f>IF(OR(M36="",H36="",(H36+O36)=0),"",(M36-H36-O36)/(H36+O36))</f>
+        <f>IF(OR(M36="",H36=""),"",IF((H36+N(O36))=0,"",(M36-H36-N(O36))/(H36+N(O36))))</f>
         <v/>
       </c>
       <c r="R36" s="15" t="n"/>
@@ -6011,7 +6011,7 @@
         <v/>
       </c>
       <c r="V36" s="16">
-        <f>IF(OR(R36="",M36="",(M36+T36)=0),"",(R36-M36-T36)/(M36+T36))</f>
+        <f>IF(OR(R36="",M36=""),"",IF((M36+N(T36))=0,"",(R36-M36-N(T36))/(M36+N(T36))))</f>
         <v/>
       </c>
       <c r="W36" s="15" t="n"/>
@@ -6022,7 +6022,7 @@
         <v/>
       </c>
       <c r="AA36" s="16">
-        <f>IF(OR(W36="",R36="",(R36+Y36)=0),"",(W36-R36-Y36)/(R36+Y36))</f>
+        <f>IF(OR(W36="",R36=""),"",IF((R36+N(Y36))=0,"",(W36-R36-N(Y36))/(R36+N(Y36))))</f>
         <v/>
       </c>
       <c r="AB36" s="15" t="n"/>
@@ -6033,7 +6033,7 @@
         <v/>
       </c>
       <c r="AF36" s="16">
-        <f>IF(OR(AB36="",W36="",(W36+AD36)=0),"",(AB36-W36-AD36)/(W36+AD36))</f>
+        <f>IF(OR(AB36="",W36=""),"",IF((W36+N(AD36))=0,"",(AB36-W36-N(AD36))/(W36+N(AD36))))</f>
         <v/>
       </c>
       <c r="AG36" s="15" t="n"/>
@@ -6044,7 +6044,7 @@
         <v/>
       </c>
       <c r="AK36" s="16">
-        <f>IF(OR(AG36="",AB36="",(AB36+AI36)=0),"",(AG36-AB36-AI36)/(AB36+AI36))</f>
+        <f>IF(OR(AG36="",AB36=""),"",IF((AB36+N(AI36))=0,"",(AG36-AB36-N(AI36))/(AB36+N(AI36))))</f>
         <v/>
       </c>
       <c r="AL36" s="15" t="n"/>
@@ -6055,7 +6055,7 @@
         <v/>
       </c>
       <c r="AP36" s="16">
-        <f>IF(OR(AL36="",AG36="",(AG36+AN36)=0),"",(AL36-AG36-AN36)/(AG36+AN36))</f>
+        <f>IF(OR(AL36="",AG36=""),"",IF((AG36+N(AN36))=0,"",(AL36-AG36-N(AN36))/(AG36+N(AN36))))</f>
         <v/>
       </c>
       <c r="AQ36" s="15" t="n"/>
@@ -6066,7 +6066,7 @@
         <v/>
       </c>
       <c r="AU36" s="16">
-        <f>IF(OR(AQ36="",AL36="",(AL36+AS36)=0),"",(AQ36-AL36-AS36)/(AL36+AS36))</f>
+        <f>IF(OR(AQ36="",AL36=""),"",IF((AL36+N(AS36))=0,"",(AQ36-AL36-N(AS36))/(AL36+N(AS36))))</f>
         <v/>
       </c>
       <c r="AV36" s="15" t="n"/>
@@ -6077,7 +6077,7 @@
         <v/>
       </c>
       <c r="AZ36" s="16">
-        <f>IF(OR(AV36="",AQ36="",(AQ36+AX36)=0),"",(AV36-AQ36-AX36)/(AQ36+AX36))</f>
+        <f>IF(OR(AV36="",AQ36=""),"",IF((AQ36+N(AX36))=0,"",(AV36-AQ36-N(AX36))/(AQ36+N(AX36))))</f>
         <v/>
       </c>
       <c r="BA36" s="15" t="n"/>
@@ -6088,7 +6088,7 @@
         <v/>
       </c>
       <c r="BE36" s="16">
-        <f>IF(OR(BA36="",AV36="",(AV36+BC36)=0),"",(BA36-AV36-BC36)/(AV36+BC36))</f>
+        <f>IF(OR(BA36="",AV36=""),"",IF((AV36+N(BC36))=0,"",(BA36-AV36-N(BC36))/(AV36+N(BC36))))</f>
         <v/>
       </c>
       <c r="BF36" s="15" t="n"/>
@@ -6099,7 +6099,7 @@
         <v/>
       </c>
       <c r="BJ36" s="16">
-        <f>IF(OR(BF36="",BA36="",(BA36+BH36)=0),"",(BF36-BA36-BH36)/(BA36+BH36))</f>
+        <f>IF(OR(BF36="",BA36=""),"",IF((BA36+N(BH36))=0,"",(BF36-BA36-N(BH36))/(BA36+N(BH36))))</f>
         <v/>
       </c>
     </row>
@@ -6114,7 +6114,7 @@
         <v/>
       </c>
       <c r="G37" s="19">
-        <f>IF(OR(C37="",B37="",(B37+E37)=0),"",(C37-B37-E37)/(B37+E37))</f>
+        <f>IF(OR(C37="",B37=""),"",IF((B37+N(E37))=0,"",(C37-B37-N(E37))/(B37+N(E37))))</f>
         <v/>
       </c>
       <c r="H37" s="18" t="n"/>
@@ -6125,7 +6125,7 @@
         <v/>
       </c>
       <c r="L37" s="19">
-        <f>IF(OR(H37="",C37="",(C37+J37)=0),"",(H37-C37-J37)/(C37+J37))</f>
+        <f>IF(OR(H37="",C37=""),"",IF((C37+N(J37))=0,"",(H37-C37-N(J37))/(C37+N(J37))))</f>
         <v/>
       </c>
       <c r="M37" s="18" t="n"/>
@@ -6136,7 +6136,7 @@
         <v/>
       </c>
       <c r="Q37" s="19">
-        <f>IF(OR(M37="",H37="",(H37+O37)=0),"",(M37-H37-O37)/(H37+O37))</f>
+        <f>IF(OR(M37="",H37=""),"",IF((H37+N(O37))=0,"",(M37-H37-N(O37))/(H37+N(O37))))</f>
         <v/>
       </c>
       <c r="R37" s="18" t="n"/>
@@ -6147,7 +6147,7 @@
         <v/>
       </c>
       <c r="V37" s="19">
-        <f>IF(OR(R37="",M37="",(M37+T37)=0),"",(R37-M37-T37)/(M37+T37))</f>
+        <f>IF(OR(R37="",M37=""),"",IF((M37+N(T37))=0,"",(R37-M37-N(T37))/(M37+N(T37))))</f>
         <v/>
       </c>
       <c r="W37" s="18" t="n"/>
@@ -6158,7 +6158,7 @@
         <v/>
       </c>
       <c r="AA37" s="19">
-        <f>IF(OR(W37="",R37="",(R37+Y37)=0),"",(W37-R37-Y37)/(R37+Y37))</f>
+        <f>IF(OR(W37="",R37=""),"",IF((R37+N(Y37))=0,"",(W37-R37-N(Y37))/(R37+N(Y37))))</f>
         <v/>
       </c>
       <c r="AB37" s="18" t="n"/>
@@ -6169,7 +6169,7 @@
         <v/>
       </c>
       <c r="AF37" s="19">
-        <f>IF(OR(AB37="",W37="",(W37+AD37)=0),"",(AB37-W37-AD37)/(W37+AD37))</f>
+        <f>IF(OR(AB37="",W37=""),"",IF((W37+N(AD37))=0,"",(AB37-W37-N(AD37))/(W37+N(AD37))))</f>
         <v/>
       </c>
       <c r="AG37" s="18" t="n"/>
@@ -6180,7 +6180,7 @@
         <v/>
       </c>
       <c r="AK37" s="19">
-        <f>IF(OR(AG37="",AB37="",(AB37+AI37)=0),"",(AG37-AB37-AI37)/(AB37+AI37))</f>
+        <f>IF(OR(AG37="",AB37=""),"",IF((AB37+N(AI37))=0,"",(AG37-AB37-N(AI37))/(AB37+N(AI37))))</f>
         <v/>
       </c>
       <c r="AL37" s="18" t="n"/>
@@ -6191,7 +6191,7 @@
         <v/>
       </c>
       <c r="AP37" s="19">
-        <f>IF(OR(AL37="",AG37="",(AG37+AN37)=0),"",(AL37-AG37-AN37)/(AG37+AN37))</f>
+        <f>IF(OR(AL37="",AG37=""),"",IF((AG37+N(AN37))=0,"",(AL37-AG37-N(AN37))/(AG37+N(AN37))))</f>
         <v/>
       </c>
       <c r="AQ37" s="18" t="n"/>
@@ -6202,7 +6202,7 @@
         <v/>
       </c>
       <c r="AU37" s="19">
-        <f>IF(OR(AQ37="",AL37="",(AL37+AS37)=0),"",(AQ37-AL37-AS37)/(AL37+AS37))</f>
+        <f>IF(OR(AQ37="",AL37=""),"",IF((AL37+N(AS37))=0,"",(AQ37-AL37-N(AS37))/(AL37+N(AS37))))</f>
         <v/>
       </c>
       <c r="AV37" s="18" t="n"/>
@@ -6213,7 +6213,7 @@
         <v/>
       </c>
       <c r="AZ37" s="19">
-        <f>IF(OR(AV37="",AQ37="",(AQ37+AX37)=0),"",(AV37-AQ37-AX37)/(AQ37+AX37))</f>
+        <f>IF(OR(AV37="",AQ37=""),"",IF((AQ37+N(AX37))=0,"",(AV37-AQ37-N(AX37))/(AQ37+N(AX37))))</f>
         <v/>
       </c>
       <c r="BA37" s="18" t="n"/>
@@ -6224,7 +6224,7 @@
         <v/>
       </c>
       <c r="BE37" s="19">
-        <f>IF(OR(BA37="",AV37="",(AV37+BC37)=0),"",(BA37-AV37-BC37)/(AV37+BC37))</f>
+        <f>IF(OR(BA37="",AV37=""),"",IF((AV37+N(BC37))=0,"",(BA37-AV37-N(BC37))/(AV37+N(BC37))))</f>
         <v/>
       </c>
       <c r="BF37" s="18" t="n"/>
@@ -6235,7 +6235,7 @@
         <v/>
       </c>
       <c r="BJ37" s="19">
-        <f>IF(OR(BF37="",BA37="",(BA37+BH37)=0),"",(BF37-BA37-BH37)/(BA37+BH37))</f>
+        <f>IF(OR(BF37="",BA37=""),"",IF((BA37+N(BH37))=0,"",(BF37-BA37-N(BH37))/(BA37+N(BH37))))</f>
         <v/>
       </c>
     </row>
@@ -6250,7 +6250,7 @@
         <v/>
       </c>
       <c r="G38" s="16">
-        <f>IF(OR(C38="",B38="",(B38+E38)=0),"",(C38-B38-E38)/(B38+E38))</f>
+        <f>IF(OR(C38="",B38=""),"",IF((B38+N(E38))=0,"",(C38-B38-N(E38))/(B38+N(E38))))</f>
         <v/>
       </c>
       <c r="H38" s="15" t="n"/>
@@ -6261,7 +6261,7 @@
         <v/>
       </c>
       <c r="L38" s="16">
-        <f>IF(OR(H38="",C38="",(C38+J38)=0),"",(H38-C38-J38)/(C38+J38))</f>
+        <f>IF(OR(H38="",C38=""),"",IF((C38+N(J38))=0,"",(H38-C38-N(J38))/(C38+N(J38))))</f>
         <v/>
       </c>
       <c r="M38" s="15" t="n"/>
@@ -6272,7 +6272,7 @@
         <v/>
       </c>
       <c r="Q38" s="16">
-        <f>IF(OR(M38="",H38="",(H38+O38)=0),"",(M38-H38-O38)/(H38+O38))</f>
+        <f>IF(OR(M38="",H38=""),"",IF((H38+N(O38))=0,"",(M38-H38-N(O38))/(H38+N(O38))))</f>
         <v/>
       </c>
       <c r="R38" s="15" t="n"/>
@@ -6283,7 +6283,7 @@
         <v/>
       </c>
       <c r="V38" s="16">
-        <f>IF(OR(R38="",M38="",(M38+T38)=0),"",(R38-M38-T38)/(M38+T38))</f>
+        <f>IF(OR(R38="",M38=""),"",IF((M38+N(T38))=0,"",(R38-M38-N(T38))/(M38+N(T38))))</f>
         <v/>
       </c>
       <c r="W38" s="15" t="n"/>
@@ -6294,7 +6294,7 @@
         <v/>
       </c>
       <c r="AA38" s="16">
-        <f>IF(OR(W38="",R38="",(R38+Y38)=0),"",(W38-R38-Y38)/(R38+Y38))</f>
+        <f>IF(OR(W38="",R38=""),"",IF((R38+N(Y38))=0,"",(W38-R38-N(Y38))/(R38+N(Y38))))</f>
         <v/>
       </c>
       <c r="AB38" s="15" t="n"/>
@@ -6305,7 +6305,7 @@
         <v/>
       </c>
       <c r="AF38" s="16">
-        <f>IF(OR(AB38="",W38="",(W38+AD38)=0),"",(AB38-W38-AD38)/(W38+AD38))</f>
+        <f>IF(OR(AB38="",W38=""),"",IF((W38+N(AD38))=0,"",(AB38-W38-N(AD38))/(W38+N(AD38))))</f>
         <v/>
       </c>
       <c r="AG38" s="15" t="n"/>
@@ -6316,7 +6316,7 @@
         <v/>
       </c>
       <c r="AK38" s="16">
-        <f>IF(OR(AG38="",AB38="",(AB38+AI38)=0),"",(AG38-AB38-AI38)/(AB38+AI38))</f>
+        <f>IF(OR(AG38="",AB38=""),"",IF((AB38+N(AI38))=0,"",(AG38-AB38-N(AI38))/(AB38+N(AI38))))</f>
         <v/>
       </c>
       <c r="AL38" s="15" t="n"/>
@@ -6327,7 +6327,7 @@
         <v/>
       </c>
       <c r="AP38" s="16">
-        <f>IF(OR(AL38="",AG38="",(AG38+AN38)=0),"",(AL38-AG38-AN38)/(AG38+AN38))</f>
+        <f>IF(OR(AL38="",AG38=""),"",IF((AG38+N(AN38))=0,"",(AL38-AG38-N(AN38))/(AG38+N(AN38))))</f>
         <v/>
       </c>
       <c r="AQ38" s="15" t="n"/>
@@ -6338,7 +6338,7 @@
         <v/>
       </c>
       <c r="AU38" s="16">
-        <f>IF(OR(AQ38="",AL38="",(AL38+AS38)=0),"",(AQ38-AL38-AS38)/(AL38+AS38))</f>
+        <f>IF(OR(AQ38="",AL38=""),"",IF((AL38+N(AS38))=0,"",(AQ38-AL38-N(AS38))/(AL38+N(AS38))))</f>
         <v/>
       </c>
       <c r="AV38" s="15" t="n"/>
@@ -6349,7 +6349,7 @@
         <v/>
       </c>
       <c r="AZ38" s="16">
-        <f>IF(OR(AV38="",AQ38="",(AQ38+AX38)=0),"",(AV38-AQ38-AX38)/(AQ38+AX38))</f>
+        <f>IF(OR(AV38="",AQ38=""),"",IF((AQ38+N(AX38))=0,"",(AV38-AQ38-N(AX38))/(AQ38+N(AX38))))</f>
         <v/>
       </c>
       <c r="BA38" s="15" t="n"/>
@@ -6360,7 +6360,7 @@
         <v/>
       </c>
       <c r="BE38" s="16">
-        <f>IF(OR(BA38="",AV38="",(AV38+BC38)=0),"",(BA38-AV38-BC38)/(AV38+BC38))</f>
+        <f>IF(OR(BA38="",AV38=""),"",IF((AV38+N(BC38))=0,"",(BA38-AV38-N(BC38))/(AV38+N(BC38))))</f>
         <v/>
       </c>
       <c r="BF38" s="15" t="n"/>
@@ -6371,7 +6371,7 @@
         <v/>
       </c>
       <c r="BJ38" s="16">
-        <f>IF(OR(BF38="",BA38="",(BA38+BH38)=0),"",(BF38-BA38-BH38)/(BA38+BH38))</f>
+        <f>IF(OR(BF38="",BA38=""),"",IF((BA38+N(BH38))=0,"",(BF38-BA38-N(BH38))/(BA38+N(BH38))))</f>
         <v/>
       </c>
     </row>
@@ -6386,7 +6386,7 @@
         <v/>
       </c>
       <c r="G39" s="19">
-        <f>IF(OR(C39="",B39="",(B39+E39)=0),"",(C39-B39-E39)/(B39+E39))</f>
+        <f>IF(OR(C39="",B39=""),"",IF((B39+N(E39))=0,"",(C39-B39-N(E39))/(B39+N(E39))))</f>
         <v/>
       </c>
       <c r="H39" s="18" t="n"/>
@@ -6397,7 +6397,7 @@
         <v/>
       </c>
       <c r="L39" s="19">
-        <f>IF(OR(H39="",C39="",(C39+J39)=0),"",(H39-C39-J39)/(C39+J39))</f>
+        <f>IF(OR(H39="",C39=""),"",IF((C39+N(J39))=0,"",(H39-C39-N(J39))/(C39+N(J39))))</f>
         <v/>
       </c>
       <c r="M39" s="18" t="n"/>
@@ -6408,7 +6408,7 @@
         <v/>
       </c>
       <c r="Q39" s="19">
-        <f>IF(OR(M39="",H39="",(H39+O39)=0),"",(M39-H39-O39)/(H39+O39))</f>
+        <f>IF(OR(M39="",H39=""),"",IF((H39+N(O39))=0,"",(M39-H39-N(O39))/(H39+N(O39))))</f>
         <v/>
       </c>
       <c r="R39" s="18" t="n"/>
@@ -6419,7 +6419,7 @@
         <v/>
       </c>
       <c r="V39" s="19">
-        <f>IF(OR(R39="",M39="",(M39+T39)=0),"",(R39-M39-T39)/(M39+T39))</f>
+        <f>IF(OR(R39="",M39=""),"",IF((M39+N(T39))=0,"",(R39-M39-N(T39))/(M39+N(T39))))</f>
         <v/>
       </c>
       <c r="W39" s="18" t="n"/>
@@ -6430,7 +6430,7 @@
         <v/>
       </c>
       <c r="AA39" s="19">
-        <f>IF(OR(W39="",R39="",(R39+Y39)=0),"",(W39-R39-Y39)/(R39+Y39))</f>
+        <f>IF(OR(W39="",R39=""),"",IF((R39+N(Y39))=0,"",(W39-R39-N(Y39))/(R39+N(Y39))))</f>
         <v/>
       </c>
       <c r="AB39" s="18" t="n"/>
@@ -6441,7 +6441,7 @@
         <v/>
       </c>
       <c r="AF39" s="19">
-        <f>IF(OR(AB39="",W39="",(W39+AD39)=0),"",(AB39-W39-AD39)/(W39+AD39))</f>
+        <f>IF(OR(AB39="",W39=""),"",IF((W39+N(AD39))=0,"",(AB39-W39-N(AD39))/(W39+N(AD39))))</f>
         <v/>
       </c>
       <c r="AG39" s="18" t="n"/>
@@ -6452,7 +6452,7 @@
         <v/>
       </c>
       <c r="AK39" s="19">
-        <f>IF(OR(AG39="",AB39="",(AB39+AI39)=0),"",(AG39-AB39-AI39)/(AB39+AI39))</f>
+        <f>IF(OR(AG39="",AB39=""),"",IF((AB39+N(AI39))=0,"",(AG39-AB39-N(AI39))/(AB39+N(AI39))))</f>
         <v/>
       </c>
       <c r="AL39" s="18" t="n"/>
@@ -6463,7 +6463,7 @@
         <v/>
       </c>
       <c r="AP39" s="19">
-        <f>IF(OR(AL39="",AG39="",(AG39+AN39)=0),"",(AL39-AG39-AN39)/(AG39+AN39))</f>
+        <f>IF(OR(AL39="",AG39=""),"",IF((AG39+N(AN39))=0,"",(AL39-AG39-N(AN39))/(AG39+N(AN39))))</f>
         <v/>
       </c>
       <c r="AQ39" s="18" t="n"/>
@@ -6474,7 +6474,7 @@
         <v/>
       </c>
       <c r="AU39" s="19">
-        <f>IF(OR(AQ39="",AL39="",(AL39+AS39)=0),"",(AQ39-AL39-AS39)/(AL39+AS39))</f>
+        <f>IF(OR(AQ39="",AL39=""),"",IF((AL39+N(AS39))=0,"",(AQ39-AL39-N(AS39))/(AL39+N(AS39))))</f>
         <v/>
       </c>
       <c r="AV39" s="18" t="n"/>
@@ -6485,7 +6485,7 @@
         <v/>
       </c>
       <c r="AZ39" s="19">
-        <f>IF(OR(AV39="",AQ39="",(AQ39+AX39)=0),"",(AV39-AQ39-AX39)/(AQ39+AX39))</f>
+        <f>IF(OR(AV39="",AQ39=""),"",IF((AQ39+N(AX39))=0,"",(AV39-AQ39-N(AX39))/(AQ39+N(AX39))))</f>
         <v/>
       </c>
       <c r="BA39" s="18" t="n"/>
@@ -6496,7 +6496,7 @@
         <v/>
       </c>
       <c r="BE39" s="19">
-        <f>IF(OR(BA39="",AV39="",(AV39+BC39)=0),"",(BA39-AV39-BC39)/(AV39+BC39))</f>
+        <f>IF(OR(BA39="",AV39=""),"",IF((AV39+N(BC39))=0,"",(BA39-AV39-N(BC39))/(AV39+N(BC39))))</f>
         <v/>
       </c>
       <c r="BF39" s="18" t="n"/>
@@ -6507,7 +6507,7 @@
         <v/>
       </c>
       <c r="BJ39" s="19">
-        <f>IF(OR(BF39="",BA39="",(BA39+BH39)=0),"",(BF39-BA39-BH39)/(BA39+BH39))</f>
+        <f>IF(OR(BF39="",BA39=""),"",IF((BA39+N(BH39))=0,"",(BF39-BA39-N(BH39))/(BA39+N(BH39))))</f>
         <v/>
       </c>
     </row>
@@ -6522,7 +6522,7 @@
         <v/>
       </c>
       <c r="G40" s="16">
-        <f>IF(OR(C40="",B40="",(B40+E40)=0),"",(C40-B40-E40)/(B40+E40))</f>
+        <f>IF(OR(C40="",B40=""),"",IF((B40+N(E40))=0,"",(C40-B40-N(E40))/(B40+N(E40))))</f>
         <v/>
       </c>
       <c r="H40" s="15" t="n"/>
@@ -6533,7 +6533,7 @@
         <v/>
       </c>
       <c r="L40" s="16">
-        <f>IF(OR(H40="",C40="",(C40+J40)=0),"",(H40-C40-J40)/(C40+J40))</f>
+        <f>IF(OR(H40="",C40=""),"",IF((C40+N(J40))=0,"",(H40-C40-N(J40))/(C40+N(J40))))</f>
         <v/>
       </c>
       <c r="M40" s="15" t="n"/>
@@ -6544,7 +6544,7 @@
         <v/>
       </c>
       <c r="Q40" s="16">
-        <f>IF(OR(M40="",H40="",(H40+O40)=0),"",(M40-H40-O40)/(H40+O40))</f>
+        <f>IF(OR(M40="",H40=""),"",IF((H40+N(O40))=0,"",(M40-H40-N(O40))/(H40+N(O40))))</f>
         <v/>
       </c>
       <c r="R40" s="15" t="n"/>
@@ -6555,7 +6555,7 @@
         <v/>
       </c>
       <c r="V40" s="16">
-        <f>IF(OR(R40="",M40="",(M40+T40)=0),"",(R40-M40-T40)/(M40+T40))</f>
+        <f>IF(OR(R40="",M40=""),"",IF((M40+N(T40))=0,"",(R40-M40-N(T40))/(M40+N(T40))))</f>
         <v/>
       </c>
       <c r="W40" s="15" t="n"/>
@@ -6566,7 +6566,7 @@
         <v/>
       </c>
       <c r="AA40" s="16">
-        <f>IF(OR(W40="",R40="",(R40+Y40)=0),"",(W40-R40-Y40)/(R40+Y40))</f>
+        <f>IF(OR(W40="",R40=""),"",IF((R40+N(Y40))=0,"",(W40-R40-N(Y40))/(R40+N(Y40))))</f>
         <v/>
       </c>
       <c r="AB40" s="15" t="n"/>
@@ -6577,7 +6577,7 @@
         <v/>
       </c>
       <c r="AF40" s="16">
-        <f>IF(OR(AB40="",W40="",(W40+AD40)=0),"",(AB40-W40-AD40)/(W40+AD40))</f>
+        <f>IF(OR(AB40="",W40=""),"",IF((W40+N(AD40))=0,"",(AB40-W40-N(AD40))/(W40+N(AD40))))</f>
         <v/>
       </c>
       <c r="AG40" s="15" t="n"/>
@@ -6588,7 +6588,7 @@
         <v/>
       </c>
       <c r="AK40" s="16">
-        <f>IF(OR(AG40="",AB40="",(AB40+AI40)=0),"",(AG40-AB40-AI40)/(AB40+AI40))</f>
+        <f>IF(OR(AG40="",AB40=""),"",IF((AB40+N(AI40))=0,"",(AG40-AB40-N(AI40))/(AB40+N(AI40))))</f>
         <v/>
       </c>
       <c r="AL40" s="15" t="n"/>
@@ -6599,7 +6599,7 @@
         <v/>
       </c>
       <c r="AP40" s="16">
-        <f>IF(OR(AL40="",AG40="",(AG40+AN40)=0),"",(AL40-AG40-AN40)/(AG40+AN40))</f>
+        <f>IF(OR(AL40="",AG40=""),"",IF((AG40+N(AN40))=0,"",(AL40-AG40-N(AN40))/(AG40+N(AN40))))</f>
         <v/>
       </c>
       <c r="AQ40" s="15" t="n"/>
@@ -6610,7 +6610,7 @@
         <v/>
       </c>
       <c r="AU40" s="16">
-        <f>IF(OR(AQ40="",AL40="",(AL40+AS40)=0),"",(AQ40-AL40-AS40)/(AL40+AS40))</f>
+        <f>IF(OR(AQ40="",AL40=""),"",IF((AL40+N(AS40))=0,"",(AQ40-AL40-N(AS40))/(AL40+N(AS40))))</f>
         <v/>
       </c>
       <c r="AV40" s="15" t="n"/>
@@ -6621,7 +6621,7 @@
         <v/>
       </c>
       <c r="AZ40" s="16">
-        <f>IF(OR(AV40="",AQ40="",(AQ40+AX40)=0),"",(AV40-AQ40-AX40)/(AQ40+AX40))</f>
+        <f>IF(OR(AV40="",AQ40=""),"",IF((AQ40+N(AX40))=0,"",(AV40-AQ40-N(AX40))/(AQ40+N(AX40))))</f>
         <v/>
       </c>
       <c r="BA40" s="15" t="n"/>
@@ -6632,7 +6632,7 @@
         <v/>
       </c>
       <c r="BE40" s="16">
-        <f>IF(OR(BA40="",AV40="",(AV40+BC40)=0),"",(BA40-AV40-BC40)/(AV40+BC40))</f>
+        <f>IF(OR(BA40="",AV40=""),"",IF((AV40+N(BC40))=0,"",(BA40-AV40-N(BC40))/(AV40+N(BC40))))</f>
         <v/>
       </c>
       <c r="BF40" s="15" t="n"/>
@@ -6643,7 +6643,7 @@
         <v/>
       </c>
       <c r="BJ40" s="16">
-        <f>IF(OR(BF40="",BA40="",(BA40+BH40)=0),"",(BF40-BA40-BH40)/(BA40+BH40))</f>
+        <f>IF(OR(BF40="",BA40=""),"",IF((BA40+N(BH40))=0,"",(BF40-BA40-N(BH40))/(BA40+N(BH40))))</f>
         <v/>
       </c>
     </row>
@@ -6658,7 +6658,7 @@
         <v/>
       </c>
       <c r="G41" s="19">
-        <f>IF(OR(C41="",B41="",(B41+E41)=0),"",(C41-B41-E41)/(B41+E41))</f>
+        <f>IF(OR(C41="",B41=""),"",IF((B41+N(E41))=0,"",(C41-B41-N(E41))/(B41+N(E41))))</f>
         <v/>
       </c>
       <c r="H41" s="18" t="n"/>
@@ -6669,7 +6669,7 @@
         <v/>
       </c>
       <c r="L41" s="19">
-        <f>IF(OR(H41="",C41="",(C41+J41)=0),"",(H41-C41-J41)/(C41+J41))</f>
+        <f>IF(OR(H41="",C41=""),"",IF((C41+N(J41))=0,"",(H41-C41-N(J41))/(C41+N(J41))))</f>
         <v/>
       </c>
       <c r="M41" s="18" t="n"/>
@@ -6680,7 +6680,7 @@
         <v/>
       </c>
       <c r="Q41" s="19">
-        <f>IF(OR(M41="",H41="",(H41+O41)=0),"",(M41-H41-O41)/(H41+O41))</f>
+        <f>IF(OR(M41="",H41=""),"",IF((H41+N(O41))=0,"",(M41-H41-N(O41))/(H41+N(O41))))</f>
         <v/>
       </c>
       <c r="R41" s="18" t="n"/>
@@ -6691,7 +6691,7 @@
         <v/>
       </c>
       <c r="V41" s="19">
-        <f>IF(OR(R41="",M41="",(M41+T41)=0),"",(R41-M41-T41)/(M41+T41))</f>
+        <f>IF(OR(R41="",M41=""),"",IF((M41+N(T41))=0,"",(R41-M41-N(T41))/(M41+N(T41))))</f>
         <v/>
       </c>
       <c r="W41" s="18" t="n"/>
@@ -6702,7 +6702,7 @@
         <v/>
       </c>
       <c r="AA41" s="19">
-        <f>IF(OR(W41="",R41="",(R41+Y41)=0),"",(W41-R41-Y41)/(R41+Y41))</f>
+        <f>IF(OR(W41="",R41=""),"",IF((R41+N(Y41))=0,"",(W41-R41-N(Y41))/(R41+N(Y41))))</f>
         <v/>
       </c>
       <c r="AB41" s="18" t="n"/>
@@ -6713,7 +6713,7 @@
         <v/>
       </c>
       <c r="AF41" s="19">
-        <f>IF(OR(AB41="",W41="",(W41+AD41)=0),"",(AB41-W41-AD41)/(W41+AD41))</f>
+        <f>IF(OR(AB41="",W41=""),"",IF((W41+N(AD41))=0,"",(AB41-W41-N(AD41))/(W41+N(AD41))))</f>
         <v/>
       </c>
       <c r="AG41" s="18" t="n"/>
@@ -6724,7 +6724,7 @@
         <v/>
       </c>
       <c r="AK41" s="19">
-        <f>IF(OR(AG41="",AB41="",(AB41+AI41)=0),"",(AG41-AB41-AI41)/(AB41+AI41))</f>
+        <f>IF(OR(AG41="",AB41=""),"",IF((AB41+N(AI41))=0,"",(AG41-AB41-N(AI41))/(AB41+N(AI41))))</f>
         <v/>
       </c>
       <c r="AL41" s="18" t="n"/>
@@ -6735,7 +6735,7 @@
         <v/>
       </c>
       <c r="AP41" s="19">
-        <f>IF(OR(AL41="",AG41="",(AG41+AN41)=0),"",(AL41-AG41-AN41)/(AG41+AN41))</f>
+        <f>IF(OR(AL41="",AG41=""),"",IF((AG41+N(AN41))=0,"",(AL41-AG41-N(AN41))/(AG41+N(AN41))))</f>
         <v/>
       </c>
       <c r="AQ41" s="18" t="n"/>
@@ -6746,7 +6746,7 @@
         <v/>
       </c>
       <c r="AU41" s="19">
-        <f>IF(OR(AQ41="",AL41="",(AL41+AS41)=0),"",(AQ41-AL41-AS41)/(AL41+AS41))</f>
+        <f>IF(OR(AQ41="",AL41=""),"",IF((AL41+N(AS41))=0,"",(AQ41-AL41-N(AS41))/(AL41+N(AS41))))</f>
         <v/>
       </c>
       <c r="AV41" s="18" t="n"/>
@@ -6757,7 +6757,7 @@
         <v/>
       </c>
       <c r="AZ41" s="19">
-        <f>IF(OR(AV41="",AQ41="",(AQ41+AX41)=0),"",(AV41-AQ41-AX41)/(AQ41+AX41))</f>
+        <f>IF(OR(AV41="",AQ41=""),"",IF((AQ41+N(AX41))=0,"",(AV41-AQ41-N(AX41))/(AQ41+N(AX41))))</f>
         <v/>
       </c>
       <c r="BA41" s="18" t="n"/>
@@ -6768,7 +6768,7 @@
         <v/>
       </c>
       <c r="BE41" s="19">
-        <f>IF(OR(BA41="",AV41="",(AV41+BC41)=0),"",(BA41-AV41-BC41)/(AV41+BC41))</f>
+        <f>IF(OR(BA41="",AV41=""),"",IF((AV41+N(BC41))=0,"",(BA41-AV41-N(BC41))/(AV41+N(BC41))))</f>
         <v/>
       </c>
       <c r="BF41" s="18" t="n"/>
@@ -6779,7 +6779,7 @@
         <v/>
       </c>
       <c r="BJ41" s="19">
-        <f>IF(OR(BF41="",BA41="",(BA41+BH41)=0),"",(BF41-BA41-BH41)/(BA41+BH41))</f>
+        <f>IF(OR(BF41="",BA41=""),"",IF((BA41+N(BH41))=0,"",(BF41-BA41-N(BH41))/(BA41+N(BH41))))</f>
         <v/>
       </c>
     </row>
@@ -6810,7 +6810,7 @@
         <v/>
       </c>
       <c r="G42" s="13">
-        <f>IF(OR(C42="",B42="",(B42+E42)=0),"",(C42-B42-E42)/(B42+E42))</f>
+        <f>IF(OR(C42="",B42=""),"",IF((B42+N(E42))=0,"",(C42-B42-N(E42))/(B42+N(E42))))</f>
         <v/>
       </c>
       <c r="H42" s="12">
@@ -6830,7 +6830,7 @@
         <v/>
       </c>
       <c r="L42" s="13">
-        <f>IF(OR(H42="",C42="",(C42+J42)=0),"",(H42-C42-J42)/(C42+J42))</f>
+        <f>IF(OR(H42="",C42=""),"",IF((C42+N(J42))=0,"",(H42-C42-N(J42))/(C42+N(J42))))</f>
         <v/>
       </c>
       <c r="M42" s="12">
@@ -6850,7 +6850,7 @@
         <v/>
       </c>
       <c r="Q42" s="13">
-        <f>IF(OR(M42="",H42="",(H42+O42)=0),"",(M42-H42-O42)/(H42+O42))</f>
+        <f>IF(OR(M42="",H42=""),"",IF((H42+N(O42))=0,"",(M42-H42-N(O42))/(H42+N(O42))))</f>
         <v/>
       </c>
       <c r="R42" s="12">
@@ -6870,7 +6870,7 @@
         <v/>
       </c>
       <c r="V42" s="13">
-        <f>IF(OR(R42="",M42="",(M42+T42)=0),"",(R42-M42-T42)/(M42+T42))</f>
+        <f>IF(OR(R42="",M42=""),"",IF((M42+N(T42))=0,"",(R42-M42-N(T42))/(M42+N(T42))))</f>
         <v/>
       </c>
       <c r="W42" s="12">
@@ -6890,7 +6890,7 @@
         <v/>
       </c>
       <c r="AA42" s="13">
-        <f>IF(OR(W42="",R42="",(R42+Y42)=0),"",(W42-R42-Y42)/(R42+Y42))</f>
+        <f>IF(OR(W42="",R42=""),"",IF((R42+N(Y42))=0,"",(W42-R42-N(Y42))/(R42+N(Y42))))</f>
         <v/>
       </c>
       <c r="AB42" s="12">
@@ -6910,7 +6910,7 @@
         <v/>
       </c>
       <c r="AF42" s="13">
-        <f>IF(OR(AB42="",W42="",(W42+AD42)=0),"",(AB42-W42-AD42)/(W42+AD42))</f>
+        <f>IF(OR(AB42="",W42=""),"",IF((W42+N(AD42))=0,"",(AB42-W42-N(AD42))/(W42+N(AD42))))</f>
         <v/>
       </c>
       <c r="AG42" s="12">
@@ -6930,7 +6930,7 @@
         <v/>
       </c>
       <c r="AK42" s="13">
-        <f>IF(OR(AG42="",AB42="",(AB42+AI42)=0),"",(AG42-AB42-AI42)/(AB42+AI42))</f>
+        <f>IF(OR(AG42="",AB42=""),"",IF((AB42+N(AI42))=0,"",(AG42-AB42-N(AI42))/(AB42+N(AI42))))</f>
         <v/>
       </c>
       <c r="AL42" s="12">
@@ -6950,7 +6950,7 @@
         <v/>
       </c>
       <c r="AP42" s="13">
-        <f>IF(OR(AL42="",AG42="",(AG42+AN42)=0),"",(AL42-AG42-AN42)/(AG42+AN42))</f>
+        <f>IF(OR(AL42="",AG42=""),"",IF((AG42+N(AN42))=0,"",(AL42-AG42-N(AN42))/(AG42+N(AN42))))</f>
         <v/>
       </c>
       <c r="AQ42" s="12">
@@ -6970,7 +6970,7 @@
         <v/>
       </c>
       <c r="AU42" s="13">
-        <f>IF(OR(AQ42="",AL42="",(AL42+AS42)=0),"",(AQ42-AL42-AS42)/(AL42+AS42))</f>
+        <f>IF(OR(AQ42="",AL42=""),"",IF((AL42+N(AS42))=0,"",(AQ42-AL42-N(AS42))/(AL42+N(AS42))))</f>
         <v/>
       </c>
       <c r="AV42" s="12">
@@ -6990,7 +6990,7 @@
         <v/>
       </c>
       <c r="AZ42" s="13">
-        <f>IF(OR(AV42="",AQ42="",(AQ42+AX42)=0),"",(AV42-AQ42-AX42)/(AQ42+AX42))</f>
+        <f>IF(OR(AV42="",AQ42=""),"",IF((AQ42+N(AX42))=0,"",(AV42-AQ42-N(AX42))/(AQ42+N(AX42))))</f>
         <v/>
       </c>
       <c r="BA42" s="12">
@@ -7010,7 +7010,7 @@
         <v/>
       </c>
       <c r="BE42" s="13">
-        <f>IF(OR(BA42="",AV42="",(AV42+BC42)=0),"",(BA42-AV42-BC42)/(AV42+BC42))</f>
+        <f>IF(OR(BA42="",AV42=""),"",IF((AV42+N(BC42))=0,"",(BA42-AV42-N(BC42))/(AV42+N(BC42))))</f>
         <v/>
       </c>
       <c r="BF42" s="12">
@@ -7030,7 +7030,7 @@
         <v/>
       </c>
       <c r="BJ42" s="13">
-        <f>IF(OR(BF42="",BA42="",(BA42+BH42)=0),"",(BF42-BA42-BH42)/(BA42+BH42))</f>
+        <f>IF(OR(BF42="",BA42=""),"",IF((BA42+N(BH42))=0,"",(BF42-BA42-N(BH42))/(BA42+N(BH42))))</f>
         <v/>
       </c>
     </row>
@@ -7045,7 +7045,7 @@
         <v/>
       </c>
       <c r="G43" s="16">
-        <f>IF(OR(C43="",B43="",(B43+E43)=0),"",(C43-B43-E43)/(B43+E43))</f>
+        <f>IF(OR(C43="",B43=""),"",IF((B43+N(E43))=0,"",(C43-B43-N(E43))/(B43+N(E43))))</f>
         <v/>
       </c>
       <c r="H43" s="15" t="n"/>
@@ -7056,7 +7056,7 @@
         <v/>
       </c>
       <c r="L43" s="16">
-        <f>IF(OR(H43="",C43="",(C43+J43)=0),"",(H43-C43-J43)/(C43+J43))</f>
+        <f>IF(OR(H43="",C43=""),"",IF((C43+N(J43))=0,"",(H43-C43-N(J43))/(C43+N(J43))))</f>
         <v/>
       </c>
       <c r="M43" s="15" t="n"/>
@@ -7067,7 +7067,7 @@
         <v/>
       </c>
       <c r="Q43" s="16">
-        <f>IF(OR(M43="",H43="",(H43+O43)=0),"",(M43-H43-O43)/(H43+O43))</f>
+        <f>IF(OR(M43="",H43=""),"",IF((H43+N(O43))=0,"",(M43-H43-N(O43))/(H43+N(O43))))</f>
         <v/>
       </c>
       <c r="R43" s="15" t="n"/>
@@ -7078,7 +7078,7 @@
         <v/>
       </c>
       <c r="V43" s="16">
-        <f>IF(OR(R43="",M43="",(M43+T43)=0),"",(R43-M43-T43)/(M43+T43))</f>
+        <f>IF(OR(R43="",M43=""),"",IF((M43+N(T43))=0,"",(R43-M43-N(T43))/(M43+N(T43))))</f>
         <v/>
       </c>
       <c r="W43" s="15" t="n"/>
@@ -7089,7 +7089,7 @@
         <v/>
       </c>
       <c r="AA43" s="16">
-        <f>IF(OR(W43="",R43="",(R43+Y43)=0),"",(W43-R43-Y43)/(R43+Y43))</f>
+        <f>IF(OR(W43="",R43=""),"",IF((R43+N(Y43))=0,"",(W43-R43-N(Y43))/(R43+N(Y43))))</f>
         <v/>
       </c>
       <c r="AB43" s="15" t="n"/>
@@ -7100,7 +7100,7 @@
         <v/>
       </c>
       <c r="AF43" s="16">
-        <f>IF(OR(AB43="",W43="",(W43+AD43)=0),"",(AB43-W43-AD43)/(W43+AD43))</f>
+        <f>IF(OR(AB43="",W43=""),"",IF((W43+N(AD43))=0,"",(AB43-W43-N(AD43))/(W43+N(AD43))))</f>
         <v/>
       </c>
       <c r="AG43" s="15" t="n"/>
@@ -7111,7 +7111,7 @@
         <v/>
       </c>
       <c r="AK43" s="16">
-        <f>IF(OR(AG43="",AB43="",(AB43+AI43)=0),"",(AG43-AB43-AI43)/(AB43+AI43))</f>
+        <f>IF(OR(AG43="",AB43=""),"",IF((AB43+N(AI43))=0,"",(AG43-AB43-N(AI43))/(AB43+N(AI43))))</f>
         <v/>
       </c>
       <c r="AL43" s="15" t="n"/>
@@ -7122,7 +7122,7 @@
         <v/>
       </c>
       <c r="AP43" s="16">
-        <f>IF(OR(AL43="",AG43="",(AG43+AN43)=0),"",(AL43-AG43-AN43)/(AG43+AN43))</f>
+        <f>IF(OR(AL43="",AG43=""),"",IF((AG43+N(AN43))=0,"",(AL43-AG43-N(AN43))/(AG43+N(AN43))))</f>
         <v/>
       </c>
       <c r="AQ43" s="15" t="n"/>
@@ -7133,7 +7133,7 @@
         <v/>
       </c>
       <c r="AU43" s="16">
-        <f>IF(OR(AQ43="",AL43="",(AL43+AS43)=0),"",(AQ43-AL43-AS43)/(AL43+AS43))</f>
+        <f>IF(OR(AQ43="",AL43=""),"",IF((AL43+N(AS43))=0,"",(AQ43-AL43-N(AS43))/(AL43+N(AS43))))</f>
         <v/>
       </c>
       <c r="AV43" s="15" t="n"/>
@@ -7144,7 +7144,7 @@
         <v/>
       </c>
       <c r="AZ43" s="16">
-        <f>IF(OR(AV43="",AQ43="",(AQ43+AX43)=0),"",(AV43-AQ43-AX43)/(AQ43+AX43))</f>
+        <f>IF(OR(AV43="",AQ43=""),"",IF((AQ43+N(AX43))=0,"",(AV43-AQ43-N(AX43))/(AQ43+N(AX43))))</f>
         <v/>
       </c>
       <c r="BA43" s="15" t="n"/>
@@ -7155,7 +7155,7 @@
         <v/>
       </c>
       <c r="BE43" s="16">
-        <f>IF(OR(BA43="",AV43="",(AV43+BC43)=0),"",(BA43-AV43-BC43)/(AV43+BC43))</f>
+        <f>IF(OR(BA43="",AV43=""),"",IF((AV43+N(BC43))=0,"",(BA43-AV43-N(BC43))/(AV43+N(BC43))))</f>
         <v/>
       </c>
       <c r="BF43" s="15" t="n"/>
@@ -7166,7 +7166,7 @@
         <v/>
       </c>
       <c r="BJ43" s="16">
-        <f>IF(OR(BF43="",BA43="",(BA43+BH43)=0),"",(BF43-BA43-BH43)/(BA43+BH43))</f>
+        <f>IF(OR(BF43="",BA43=""),"",IF((BA43+N(BH43))=0,"",(BF43-BA43-N(BH43))/(BA43+N(BH43))))</f>
         <v/>
       </c>
     </row>
@@ -7181,7 +7181,7 @@
         <v/>
       </c>
       <c r="G44" s="19">
-        <f>IF(OR(C44="",B44="",(B44+E44)=0),"",(C44-B44-E44)/(B44+E44))</f>
+        <f>IF(OR(C44="",B44=""),"",IF((B44+N(E44))=0,"",(C44-B44-N(E44))/(B44+N(E44))))</f>
         <v/>
       </c>
       <c r="H44" s="18" t="n"/>
@@ -7192,7 +7192,7 @@
         <v/>
       </c>
       <c r="L44" s="19">
-        <f>IF(OR(H44="",C44="",(C44+J44)=0),"",(H44-C44-J44)/(C44+J44))</f>
+        <f>IF(OR(H44="",C44=""),"",IF((C44+N(J44))=0,"",(H44-C44-N(J44))/(C44+N(J44))))</f>
         <v/>
       </c>
       <c r="M44" s="18" t="n"/>
@@ -7203,7 +7203,7 @@
         <v/>
       </c>
       <c r="Q44" s="19">
-        <f>IF(OR(M44="",H44="",(H44+O44)=0),"",(M44-H44-O44)/(H44+O44))</f>
+        <f>IF(OR(M44="",H44=""),"",IF((H44+N(O44))=0,"",(M44-H44-N(O44))/(H44+N(O44))))</f>
         <v/>
       </c>
       <c r="R44" s="18" t="n"/>
@@ -7214,7 +7214,7 @@
         <v/>
       </c>
       <c r="V44" s="19">
-        <f>IF(OR(R44="",M44="",(M44+T44)=0),"",(R44-M44-T44)/(M44+T44))</f>
+        <f>IF(OR(R44="",M44=""),"",IF((M44+N(T44))=0,"",(R44-M44-N(T44))/(M44+N(T44))))</f>
         <v/>
       </c>
       <c r="W44" s="18" t="n"/>
@@ -7225,7 +7225,7 @@
         <v/>
       </c>
       <c r="AA44" s="19">
-        <f>IF(OR(W44="",R44="",(R44+Y44)=0),"",(W44-R44-Y44)/(R44+Y44))</f>
+        <f>IF(OR(W44="",R44=""),"",IF((R44+N(Y44))=0,"",(W44-R44-N(Y44))/(R44+N(Y44))))</f>
         <v/>
       </c>
       <c r="AB44" s="18" t="n"/>
@@ -7236,7 +7236,7 @@
         <v/>
       </c>
       <c r="AF44" s="19">
-        <f>IF(OR(AB44="",W44="",(W44+AD44)=0),"",(AB44-W44-AD44)/(W44+AD44))</f>
+        <f>IF(OR(AB44="",W44=""),"",IF((W44+N(AD44))=0,"",(AB44-W44-N(AD44))/(W44+N(AD44))))</f>
         <v/>
       </c>
       <c r="AG44" s="18" t="n"/>
@@ -7247,7 +7247,7 @@
         <v/>
       </c>
       <c r="AK44" s="19">
-        <f>IF(OR(AG44="",AB44="",(AB44+AI44)=0),"",(AG44-AB44-AI44)/(AB44+AI44))</f>
+        <f>IF(OR(AG44="",AB44=""),"",IF((AB44+N(AI44))=0,"",(AG44-AB44-N(AI44))/(AB44+N(AI44))))</f>
         <v/>
       </c>
       <c r="AL44" s="18" t="n"/>
@@ -7258,7 +7258,7 @@
         <v/>
       </c>
       <c r="AP44" s="19">
-        <f>IF(OR(AL44="",AG44="",(AG44+AN44)=0),"",(AL44-AG44-AN44)/(AG44+AN44))</f>
+        <f>IF(OR(AL44="",AG44=""),"",IF((AG44+N(AN44))=0,"",(AL44-AG44-N(AN44))/(AG44+N(AN44))))</f>
         <v/>
       </c>
       <c r="AQ44" s="18" t="n"/>
@@ -7269,7 +7269,7 @@
         <v/>
       </c>
       <c r="AU44" s="19">
-        <f>IF(OR(AQ44="",AL44="",(AL44+AS44)=0),"",(AQ44-AL44-AS44)/(AL44+AS44))</f>
+        <f>IF(OR(AQ44="",AL44=""),"",IF((AL44+N(AS44))=0,"",(AQ44-AL44-N(AS44))/(AL44+N(AS44))))</f>
         <v/>
       </c>
       <c r="AV44" s="18" t="n"/>
@@ -7280,7 +7280,7 @@
         <v/>
       </c>
       <c r="AZ44" s="19">
-        <f>IF(OR(AV44="",AQ44="",(AQ44+AX44)=0),"",(AV44-AQ44-AX44)/(AQ44+AX44))</f>
+        <f>IF(OR(AV44="",AQ44=""),"",IF((AQ44+N(AX44))=0,"",(AV44-AQ44-N(AX44))/(AQ44+N(AX44))))</f>
         <v/>
       </c>
       <c r="BA44" s="18" t="n"/>
@@ -7291,7 +7291,7 @@
         <v/>
       </c>
       <c r="BE44" s="19">
-        <f>IF(OR(BA44="",AV44="",(AV44+BC44)=0),"",(BA44-AV44-BC44)/(AV44+BC44))</f>
+        <f>IF(OR(BA44="",AV44=""),"",IF((AV44+N(BC44))=0,"",(BA44-AV44-N(BC44))/(AV44+N(BC44))))</f>
         <v/>
       </c>
       <c r="BF44" s="18" t="n"/>
@@ -7302,7 +7302,7 @@
         <v/>
       </c>
       <c r="BJ44" s="19">
-        <f>IF(OR(BF44="",BA44="",(BA44+BH44)=0),"",(BF44-BA44-BH44)/(BA44+BH44))</f>
+        <f>IF(OR(BF44="",BA44=""),"",IF((BA44+N(BH44))=0,"",(BF44-BA44-N(BH44))/(BA44+N(BH44))))</f>
         <v/>
       </c>
     </row>
@@ -7317,7 +7317,7 @@
         <v/>
       </c>
       <c r="G45" s="16">
-        <f>IF(OR(C45="",B45="",(B45+E45)=0),"",(C45-B45-E45)/(B45+E45))</f>
+        <f>IF(OR(C45="",B45=""),"",IF((B45+N(E45))=0,"",(C45-B45-N(E45))/(B45+N(E45))))</f>
         <v/>
       </c>
       <c r="H45" s="15" t="n"/>
@@ -7328,7 +7328,7 @@
         <v/>
       </c>
       <c r="L45" s="16">
-        <f>IF(OR(H45="",C45="",(C45+J45)=0),"",(H45-C45-J45)/(C45+J45))</f>
+        <f>IF(OR(H45="",C45=""),"",IF((C45+N(J45))=0,"",(H45-C45-N(J45))/(C45+N(J45))))</f>
         <v/>
       </c>
       <c r="M45" s="15" t="n"/>
@@ -7339,7 +7339,7 @@
         <v/>
       </c>
       <c r="Q45" s="16">
-        <f>IF(OR(M45="",H45="",(H45+O45)=0),"",(M45-H45-O45)/(H45+O45))</f>
+        <f>IF(OR(M45="",H45=""),"",IF((H45+N(O45))=0,"",(M45-H45-N(O45))/(H45+N(O45))))</f>
         <v/>
       </c>
       <c r="R45" s="15" t="n"/>
@@ -7350,7 +7350,7 @@
         <v/>
       </c>
       <c r="V45" s="16">
-        <f>IF(OR(R45="",M45="",(M45+T45)=0),"",(R45-M45-T45)/(M45+T45))</f>
+        <f>IF(OR(R45="",M45=""),"",IF((M45+N(T45))=0,"",(R45-M45-N(T45))/(M45+N(T45))))</f>
         <v/>
       </c>
       <c r="W45" s="15" t="n"/>
@@ -7361,7 +7361,7 @@
         <v/>
       </c>
       <c r="AA45" s="16">
-        <f>IF(OR(W45="",R45="",(R45+Y45)=0),"",(W45-R45-Y45)/(R45+Y45))</f>
+        <f>IF(OR(W45="",R45=""),"",IF((R45+N(Y45))=0,"",(W45-R45-N(Y45))/(R45+N(Y45))))</f>
         <v/>
       </c>
       <c r="AB45" s="15" t="n"/>
@@ -7372,7 +7372,7 @@
         <v/>
       </c>
       <c r="AF45" s="16">
-        <f>IF(OR(AB45="",W45="",(W45+AD45)=0),"",(AB45-W45-AD45)/(W45+AD45))</f>
+        <f>IF(OR(AB45="",W45=""),"",IF((W45+N(AD45))=0,"",(AB45-W45-N(AD45))/(W45+N(AD45))))</f>
         <v/>
       </c>
       <c r="AG45" s="15" t="n"/>
@@ -7383,7 +7383,7 @@
         <v/>
       </c>
       <c r="AK45" s="16">
-        <f>IF(OR(AG45="",AB45="",(AB45+AI45)=0),"",(AG45-AB45-AI45)/(AB45+AI45))</f>
+        <f>IF(OR(AG45="",AB45=""),"",IF((AB45+N(AI45))=0,"",(AG45-AB45-N(AI45))/(AB45+N(AI45))))</f>
         <v/>
       </c>
       <c r="AL45" s="15" t="n"/>
@@ -7394,7 +7394,7 @@
         <v/>
       </c>
       <c r="AP45" s="16">
-        <f>IF(OR(AL45="",AG45="",(AG45+AN45)=0),"",(AL45-AG45-AN45)/(AG45+AN45))</f>
+        <f>IF(OR(AL45="",AG45=""),"",IF((AG45+N(AN45))=0,"",(AL45-AG45-N(AN45))/(AG45+N(AN45))))</f>
         <v/>
       </c>
       <c r="AQ45" s="15" t="n"/>
@@ -7405,7 +7405,7 @@
         <v/>
       </c>
       <c r="AU45" s="16">
-        <f>IF(OR(AQ45="",AL45="",(AL45+AS45)=0),"",(AQ45-AL45-AS45)/(AL45+AS45))</f>
+        <f>IF(OR(AQ45="",AL45=""),"",IF((AL45+N(AS45))=0,"",(AQ45-AL45-N(AS45))/(AL45+N(AS45))))</f>
         <v/>
       </c>
       <c r="AV45" s="15" t="n"/>
@@ -7416,7 +7416,7 @@
         <v/>
       </c>
       <c r="AZ45" s="16">
-        <f>IF(OR(AV45="",AQ45="",(AQ45+AX45)=0),"",(AV45-AQ45-AX45)/(AQ45+AX45))</f>
+        <f>IF(OR(AV45="",AQ45=""),"",IF((AQ45+N(AX45))=0,"",(AV45-AQ45-N(AX45))/(AQ45+N(AX45))))</f>
         <v/>
       </c>
       <c r="BA45" s="15" t="n"/>
@@ -7427,7 +7427,7 @@
         <v/>
       </c>
       <c r="BE45" s="16">
-        <f>IF(OR(BA45="",AV45="",(AV45+BC45)=0),"",(BA45-AV45-BC45)/(AV45+BC45))</f>
+        <f>IF(OR(BA45="",AV45=""),"",IF((AV45+N(BC45))=0,"",(BA45-AV45-N(BC45))/(AV45+N(BC45))))</f>
         <v/>
       </c>
       <c r="BF45" s="15" t="n"/>
@@ -7438,7 +7438,7 @@
         <v/>
       </c>
       <c r="BJ45" s="16">
-        <f>IF(OR(BF45="",BA45="",(BA45+BH45)=0),"",(BF45-BA45-BH45)/(BA45+BH45))</f>
+        <f>IF(OR(BF45="",BA45=""),"",IF((BA45+N(BH45))=0,"",(BF45-BA45-N(BH45))/(BA45+N(BH45))))</f>
         <v/>
       </c>
     </row>
@@ -7453,7 +7453,7 @@
         <v/>
       </c>
       <c r="G46" s="19">
-        <f>IF(OR(C46="",B46="",(B46+E46)=0),"",(C46-B46-E46)/(B46+E46))</f>
+        <f>IF(OR(C46="",B46=""),"",IF((B46+N(E46))=0,"",(C46-B46-N(E46))/(B46+N(E46))))</f>
         <v/>
       </c>
       <c r="H46" s="18" t="n"/>
@@ -7464,7 +7464,7 @@
         <v/>
       </c>
       <c r="L46" s="19">
-        <f>IF(OR(H46="",C46="",(C46+J46)=0),"",(H46-C46-J46)/(C46+J46))</f>
+        <f>IF(OR(H46="",C46=""),"",IF((C46+N(J46))=0,"",(H46-C46-N(J46))/(C46+N(J46))))</f>
         <v/>
       </c>
       <c r="M46" s="18" t="n"/>
@@ -7475,7 +7475,7 @@
         <v/>
       </c>
       <c r="Q46" s="19">
-        <f>IF(OR(M46="",H46="",(H46+O46)=0),"",(M46-H46-O46)/(H46+O46))</f>
+        <f>IF(OR(M46="",H46=""),"",IF((H46+N(O46))=0,"",(M46-H46-N(O46))/(H46+N(O46))))</f>
         <v/>
       </c>
       <c r="R46" s="18" t="n"/>
@@ -7486,7 +7486,7 @@
         <v/>
       </c>
       <c r="V46" s="19">
-        <f>IF(OR(R46="",M46="",(M46+T46)=0),"",(R46-M46-T46)/(M46+T46))</f>
+        <f>IF(OR(R46="",M46=""),"",IF((M46+N(T46))=0,"",(R46-M46-N(T46))/(M46+N(T46))))</f>
         <v/>
       </c>
       <c r="W46" s="18" t="n"/>
@@ -7497,7 +7497,7 @@
         <v/>
       </c>
       <c r="AA46" s="19">
-        <f>IF(OR(W46="",R46="",(R46+Y46)=0),"",(W46-R46-Y46)/(R46+Y46))</f>
+        <f>IF(OR(W46="",R46=""),"",IF((R46+N(Y46))=0,"",(W46-R46-N(Y46))/(R46+N(Y46))))</f>
         <v/>
       </c>
       <c r="AB46" s="18" t="n"/>
@@ -7508,7 +7508,7 @@
         <v/>
       </c>
       <c r="AF46" s="19">
-        <f>IF(OR(AB46="",W46="",(W46+AD46)=0),"",(AB46-W46-AD46)/(W46+AD46))</f>
+        <f>IF(OR(AB46="",W46=""),"",IF((W46+N(AD46))=0,"",(AB46-W46-N(AD46))/(W46+N(AD46))))</f>
         <v/>
       </c>
       <c r="AG46" s="18" t="n"/>
@@ -7519,7 +7519,7 @@
         <v/>
       </c>
       <c r="AK46" s="19">
-        <f>IF(OR(AG46="",AB46="",(AB46+AI46)=0),"",(AG46-AB46-AI46)/(AB46+AI46))</f>
+        <f>IF(OR(AG46="",AB46=""),"",IF((AB46+N(AI46))=0,"",(AG46-AB46-N(AI46))/(AB46+N(AI46))))</f>
         <v/>
       </c>
       <c r="AL46" s="18" t="n"/>
@@ -7530,7 +7530,7 @@
         <v/>
       </c>
       <c r="AP46" s="19">
-        <f>IF(OR(AL46="",AG46="",(AG46+AN46)=0),"",(AL46-AG46-AN46)/(AG46+AN46))</f>
+        <f>IF(OR(AL46="",AG46=""),"",IF((AG46+N(AN46))=0,"",(AL46-AG46-N(AN46))/(AG46+N(AN46))))</f>
         <v/>
       </c>
       <c r="AQ46" s="18" t="n"/>
@@ -7541,7 +7541,7 @@
         <v/>
       </c>
       <c r="AU46" s="19">
-        <f>IF(OR(AQ46="",AL46="",(AL46+AS46)=0),"",(AQ46-AL46-AS46)/(AL46+AS46))</f>
+        <f>IF(OR(AQ46="",AL46=""),"",IF((AL46+N(AS46))=0,"",(AQ46-AL46-N(AS46))/(AL46+N(AS46))))</f>
         <v/>
       </c>
       <c r="AV46" s="18" t="n"/>
@@ -7552,7 +7552,7 @@
         <v/>
       </c>
       <c r="AZ46" s="19">
-        <f>IF(OR(AV46="",AQ46="",(AQ46+AX46)=0),"",(AV46-AQ46-AX46)/(AQ46+AX46))</f>
+        <f>IF(OR(AV46="",AQ46=""),"",IF((AQ46+N(AX46))=0,"",(AV46-AQ46-N(AX46))/(AQ46+N(AX46))))</f>
         <v/>
       </c>
       <c r="BA46" s="18" t="n"/>
@@ -7563,7 +7563,7 @@
         <v/>
       </c>
       <c r="BE46" s="19">
-        <f>IF(OR(BA46="",AV46="",(AV46+BC46)=0),"",(BA46-AV46-BC46)/(AV46+BC46))</f>
+        <f>IF(OR(BA46="",AV46=""),"",IF((AV46+N(BC46))=0,"",(BA46-AV46-N(BC46))/(AV46+N(BC46))))</f>
         <v/>
       </c>
       <c r="BF46" s="18" t="n"/>
@@ -7574,7 +7574,7 @@
         <v/>
       </c>
       <c r="BJ46" s="19">
-        <f>IF(OR(BF46="",BA46="",(BA46+BH46)=0),"",(BF46-BA46-BH46)/(BA46+BH46))</f>
+        <f>IF(OR(BF46="",BA46=""),"",IF((BA46+N(BH46))=0,"",(BF46-BA46-N(BH46))/(BA46+N(BH46))))</f>
         <v/>
       </c>
     </row>
@@ -7589,7 +7589,7 @@
         <v/>
       </c>
       <c r="G47" s="16">
-        <f>IF(OR(C47="",B47="",(B47+E47)=0),"",(C47-B47-E47)/(B47+E47))</f>
+        <f>IF(OR(C47="",B47=""),"",IF((B47+N(E47))=0,"",(C47-B47-N(E47))/(B47+N(E47))))</f>
         <v/>
       </c>
       <c r="H47" s="15" t="n"/>
@@ -7600,7 +7600,7 @@
         <v/>
       </c>
       <c r="L47" s="16">
-        <f>IF(OR(H47="",C47="",(C47+J47)=0),"",(H47-C47-J47)/(C47+J47))</f>
+        <f>IF(OR(H47="",C47=""),"",IF((C47+N(J47))=0,"",(H47-C47-N(J47))/(C47+N(J47))))</f>
         <v/>
       </c>
       <c r="M47" s="15" t="n"/>
@@ -7611,7 +7611,7 @@
         <v/>
       </c>
       <c r="Q47" s="16">
-        <f>IF(OR(M47="",H47="",(H47+O47)=0),"",(M47-H47-O47)/(H47+O47))</f>
+        <f>IF(OR(M47="",H47=""),"",IF((H47+N(O47))=0,"",(M47-H47-N(O47))/(H47+N(O47))))</f>
         <v/>
       </c>
       <c r="R47" s="15" t="n"/>
@@ -7622,7 +7622,7 @@
         <v/>
       </c>
       <c r="V47" s="16">
-        <f>IF(OR(R47="",M47="",(M47+T47)=0),"",(R47-M47-T47)/(M47+T47))</f>
+        <f>IF(OR(R47="",M47=""),"",IF((M47+N(T47))=0,"",(R47-M47-N(T47))/(M47+N(T47))))</f>
         <v/>
       </c>
       <c r="W47" s="15" t="n"/>
@@ -7633,7 +7633,7 @@
         <v/>
       </c>
       <c r="AA47" s="16">
-        <f>IF(OR(W47="",R47="",(R47+Y47)=0),"",(W47-R47-Y47)/(R47+Y47))</f>
+        <f>IF(OR(W47="",R47=""),"",IF((R47+N(Y47))=0,"",(W47-R47-N(Y47))/(R47+N(Y47))))</f>
         <v/>
       </c>
       <c r="AB47" s="15" t="n"/>
@@ -7644,7 +7644,7 @@
         <v/>
       </c>
       <c r="AF47" s="16">
-        <f>IF(OR(AB47="",W47="",(W47+AD47)=0),"",(AB47-W47-AD47)/(W47+AD47))</f>
+        <f>IF(OR(AB47="",W47=""),"",IF((W47+N(AD47))=0,"",(AB47-W47-N(AD47))/(W47+N(AD47))))</f>
         <v/>
       </c>
       <c r="AG47" s="15" t="n"/>
@@ -7655,7 +7655,7 @@
         <v/>
       </c>
       <c r="AK47" s="16">
-        <f>IF(OR(AG47="",AB47="",(AB47+AI47)=0),"",(AG47-AB47-AI47)/(AB47+AI47))</f>
+        <f>IF(OR(AG47="",AB47=""),"",IF((AB47+N(AI47))=0,"",(AG47-AB47-N(AI47))/(AB47+N(AI47))))</f>
         <v/>
       </c>
       <c r="AL47" s="15" t="n"/>
@@ -7666,7 +7666,7 @@
         <v/>
       </c>
       <c r="AP47" s="16">
-        <f>IF(OR(AL47="",AG47="",(AG47+AN47)=0),"",(AL47-AG47-AN47)/(AG47+AN47))</f>
+        <f>IF(OR(AL47="",AG47=""),"",IF((AG47+N(AN47))=0,"",(AL47-AG47-N(AN47))/(AG47+N(AN47))))</f>
         <v/>
       </c>
       <c r="AQ47" s="15" t="n"/>
@@ -7677,7 +7677,7 @@
         <v/>
       </c>
       <c r="AU47" s="16">
-        <f>IF(OR(AQ47="",AL47="",(AL47+AS47)=0),"",(AQ47-AL47-AS47)/(AL47+AS47))</f>
+        <f>IF(OR(AQ47="",AL47=""),"",IF((AL47+N(AS47))=0,"",(AQ47-AL47-N(AS47))/(AL47+N(AS47))))</f>
         <v/>
       </c>
       <c r="AV47" s="15" t="n"/>
@@ -7688,7 +7688,7 @@
         <v/>
       </c>
       <c r="AZ47" s="16">
-        <f>IF(OR(AV47="",AQ47="",(AQ47+AX47)=0),"",(AV47-AQ47-AX47)/(AQ47+AX47))</f>
+        <f>IF(OR(AV47="",AQ47=""),"",IF((AQ47+N(AX47))=0,"",(AV47-AQ47-N(AX47))/(AQ47+N(AX47))))</f>
         <v/>
       </c>
       <c r="BA47" s="15" t="n"/>
@@ -7699,7 +7699,7 @@
         <v/>
       </c>
       <c r="BE47" s="16">
-        <f>IF(OR(BA47="",AV47="",(AV47+BC47)=0),"",(BA47-AV47-BC47)/(AV47+BC47))</f>
+        <f>IF(OR(BA47="",AV47=""),"",IF((AV47+N(BC47))=0,"",(BA47-AV47-N(BC47))/(AV47+N(BC47))))</f>
         <v/>
       </c>
       <c r="BF47" s="15" t="n"/>
@@ -7710,7 +7710,7 @@
         <v/>
       </c>
       <c r="BJ47" s="16">
-        <f>IF(OR(BF47="",BA47="",(BA47+BH47)=0),"",(BF47-BA47-BH47)/(BA47+BH47))</f>
+        <f>IF(OR(BF47="",BA47=""),"",IF((BA47+N(BH47))=0,"",(BF47-BA47-N(BH47))/(BA47+N(BH47))))</f>
         <v/>
       </c>
     </row>
@@ -7725,7 +7725,7 @@
         <v/>
       </c>
       <c r="G48" s="19">
-        <f>IF(OR(C48="",B48="",(B48+E48)=0),"",(C48-B48-E48)/(B48+E48))</f>
+        <f>IF(OR(C48="",B48=""),"",IF((B48+N(E48))=0,"",(C48-B48-N(E48))/(B48+N(E48))))</f>
         <v/>
       </c>
       <c r="H48" s="18" t="n"/>
@@ -7736,7 +7736,7 @@
         <v/>
       </c>
       <c r="L48" s="19">
-        <f>IF(OR(H48="",C48="",(C48+J48)=0),"",(H48-C48-J48)/(C48+J48))</f>
+        <f>IF(OR(H48="",C48=""),"",IF((C48+N(J48))=0,"",(H48-C48-N(J48))/(C48+N(J48))))</f>
         <v/>
       </c>
       <c r="M48" s="18" t="n"/>
@@ -7747,7 +7747,7 @@
         <v/>
       </c>
       <c r="Q48" s="19">
-        <f>IF(OR(M48="",H48="",(H48+O48)=0),"",(M48-H48-O48)/(H48+O48))</f>
+        <f>IF(OR(M48="",H48=""),"",IF((H48+N(O48))=0,"",(M48-H48-N(O48))/(H48+N(O48))))</f>
         <v/>
       </c>
       <c r="R48" s="18" t="n"/>
@@ -7758,7 +7758,7 @@
         <v/>
       </c>
       <c r="V48" s="19">
-        <f>IF(OR(R48="",M48="",(M48+T48)=0),"",(R48-M48-T48)/(M48+T48))</f>
+        <f>IF(OR(R48="",M48=""),"",IF((M48+N(T48))=0,"",(R48-M48-N(T48))/(M48+N(T48))))</f>
         <v/>
       </c>
       <c r="W48" s="18" t="n"/>
@@ -7769,7 +7769,7 @@
         <v/>
       </c>
       <c r="AA48" s="19">
-        <f>IF(OR(W48="",R48="",(R48+Y48)=0),"",(W48-R48-Y48)/(R48+Y48))</f>
+        <f>IF(OR(W48="",R48=""),"",IF((R48+N(Y48))=0,"",(W48-R48-N(Y48))/(R48+N(Y48))))</f>
         <v/>
       </c>
       <c r="AB48" s="18" t="n"/>
@@ -7780,7 +7780,7 @@
         <v/>
       </c>
       <c r="AF48" s="19">
-        <f>IF(OR(AB48="",W48="",(W48+AD48)=0),"",(AB48-W48-AD48)/(W48+AD48))</f>
+        <f>IF(OR(AB48="",W48=""),"",IF((W48+N(AD48))=0,"",(AB48-W48-N(AD48))/(W48+N(AD48))))</f>
         <v/>
       </c>
       <c r="AG48" s="18" t="n"/>
@@ -7791,7 +7791,7 @@
         <v/>
       </c>
       <c r="AK48" s="19">
-        <f>IF(OR(AG48="",AB48="",(AB48+AI48)=0),"",(AG48-AB48-AI48)/(AB48+AI48))</f>
+        <f>IF(OR(AG48="",AB48=""),"",IF((AB48+N(AI48))=0,"",(AG48-AB48-N(AI48))/(AB48+N(AI48))))</f>
         <v/>
       </c>
       <c r="AL48" s="18" t="n"/>
@@ -7802,7 +7802,7 @@
         <v/>
       </c>
       <c r="AP48" s="19">
-        <f>IF(OR(AL48="",AG48="",(AG48+AN48)=0),"",(AL48-AG48-AN48)/(AG48+AN48))</f>
+        <f>IF(OR(AL48="",AG48=""),"",IF((AG48+N(AN48))=0,"",(AL48-AG48-N(AN48))/(AG48+N(AN48))))</f>
         <v/>
       </c>
       <c r="AQ48" s="18" t="n"/>
@@ -7813,7 +7813,7 @@
         <v/>
       </c>
       <c r="AU48" s="19">
-        <f>IF(OR(AQ48="",AL48="",(AL48+AS48)=0),"",(AQ48-AL48-AS48)/(AL48+AS48))</f>
+        <f>IF(OR(AQ48="",AL48=""),"",IF((AL48+N(AS48))=0,"",(AQ48-AL48-N(AS48))/(AL48+N(AS48))))</f>
         <v/>
       </c>
       <c r="AV48" s="18" t="n"/>
@@ -7824,7 +7824,7 @@
         <v/>
       </c>
       <c r="AZ48" s="19">
-        <f>IF(OR(AV48="",AQ48="",(AQ48+AX48)=0),"",(AV48-AQ48-AX48)/(AQ48+AX48))</f>
+        <f>IF(OR(AV48="",AQ48=""),"",IF((AQ48+N(AX48))=0,"",(AV48-AQ48-N(AX48))/(AQ48+N(AX48))))</f>
         <v/>
       </c>
       <c r="BA48" s="18" t="n"/>
@@ -7835,7 +7835,7 @@
         <v/>
       </c>
       <c r="BE48" s="19">
-        <f>IF(OR(BA48="",AV48="",(AV48+BC48)=0),"",(BA48-AV48-BC48)/(AV48+BC48))</f>
+        <f>IF(OR(BA48="",AV48=""),"",IF((AV48+N(BC48))=0,"",(BA48-AV48-N(BC48))/(AV48+N(BC48))))</f>
         <v/>
       </c>
       <c r="BF48" s="18" t="n"/>
@@ -7846,7 +7846,7 @@
         <v/>
       </c>
       <c r="BJ48" s="19">
-        <f>IF(OR(BF48="",BA48="",(BA48+BH48)=0),"",(BF48-BA48-BH48)/(BA48+BH48))</f>
+        <f>IF(OR(BF48="",BA48=""),"",IF((BA48+N(BH48))=0,"",(BF48-BA48-N(BH48))/(BA48+N(BH48))))</f>
         <v/>
       </c>
     </row>
@@ -7877,7 +7877,7 @@
         <v/>
       </c>
       <c r="G49" s="13">
-        <f>IF(OR(C49="",B49="",(B49+E49)=0),"",(C49-B49-E49)/(B49+E49))</f>
+        <f>IF(OR(C49="",B49=""),"",IF((B49+N(E49))=0,"",(C49-B49-N(E49))/(B49+N(E49))))</f>
         <v/>
       </c>
       <c r="H49" s="12">
@@ -7897,7 +7897,7 @@
         <v/>
       </c>
       <c r="L49" s="13">
-        <f>IF(OR(H49="",C49="",(C49+J49)=0),"",(H49-C49-J49)/(C49+J49))</f>
+        <f>IF(OR(H49="",C49=""),"",IF((C49+N(J49))=0,"",(H49-C49-N(J49))/(C49+N(J49))))</f>
         <v/>
       </c>
       <c r="M49" s="12">
@@ -7917,7 +7917,7 @@
         <v/>
       </c>
       <c r="Q49" s="13">
-        <f>IF(OR(M49="",H49="",(H49+O49)=0),"",(M49-H49-O49)/(H49+O49))</f>
+        <f>IF(OR(M49="",H49=""),"",IF((H49+N(O49))=0,"",(M49-H49-N(O49))/(H49+N(O49))))</f>
         <v/>
       </c>
       <c r="R49" s="12">
@@ -7937,7 +7937,7 @@
         <v/>
       </c>
       <c r="V49" s="13">
-        <f>IF(OR(R49="",M49="",(M49+T49)=0),"",(R49-M49-T49)/(M49+T49))</f>
+        <f>IF(OR(R49="",M49=""),"",IF((M49+N(T49))=0,"",(R49-M49-N(T49))/(M49+N(T49))))</f>
         <v/>
       </c>
       <c r="W49" s="12">
@@ -7957,7 +7957,7 @@
         <v/>
       </c>
       <c r="AA49" s="13">
-        <f>IF(OR(W49="",R49="",(R49+Y49)=0),"",(W49-R49-Y49)/(R49+Y49))</f>
+        <f>IF(OR(W49="",R49=""),"",IF((R49+N(Y49))=0,"",(W49-R49-N(Y49))/(R49+N(Y49))))</f>
         <v/>
       </c>
       <c r="AB49" s="12">
@@ -7977,7 +7977,7 @@
         <v/>
       </c>
       <c r="AF49" s="13">
-        <f>IF(OR(AB49="",W49="",(W49+AD49)=0),"",(AB49-W49-AD49)/(W49+AD49))</f>
+        <f>IF(OR(AB49="",W49=""),"",IF((W49+N(AD49))=0,"",(AB49-W49-N(AD49))/(W49+N(AD49))))</f>
         <v/>
       </c>
       <c r="AG49" s="12">
@@ -7997,7 +7997,7 @@
         <v/>
       </c>
       <c r="AK49" s="13">
-        <f>IF(OR(AG49="",AB49="",(AB49+AI49)=0),"",(AG49-AB49-AI49)/(AB49+AI49))</f>
+        <f>IF(OR(AG49="",AB49=""),"",IF((AB49+N(AI49))=0,"",(AG49-AB49-N(AI49))/(AB49+N(AI49))))</f>
         <v/>
       </c>
       <c r="AL49" s="12">
@@ -8017,7 +8017,7 @@
         <v/>
       </c>
       <c r="AP49" s="13">
-        <f>IF(OR(AL49="",AG49="",(AG49+AN49)=0),"",(AL49-AG49-AN49)/(AG49+AN49))</f>
+        <f>IF(OR(AL49="",AG49=""),"",IF((AG49+N(AN49))=0,"",(AL49-AG49-N(AN49))/(AG49+N(AN49))))</f>
         <v/>
       </c>
       <c r="AQ49" s="12">
@@ -8037,7 +8037,7 @@
         <v/>
       </c>
       <c r="AU49" s="13">
-        <f>IF(OR(AQ49="",AL49="",(AL49+AS49)=0),"",(AQ49-AL49-AS49)/(AL49+AS49))</f>
+        <f>IF(OR(AQ49="",AL49=""),"",IF((AL49+N(AS49))=0,"",(AQ49-AL49-N(AS49))/(AL49+N(AS49))))</f>
         <v/>
       </c>
       <c r="AV49" s="12">
@@ -8057,7 +8057,7 @@
         <v/>
       </c>
       <c r="AZ49" s="13">
-        <f>IF(OR(AV49="",AQ49="",(AQ49+AX49)=0),"",(AV49-AQ49-AX49)/(AQ49+AX49))</f>
+        <f>IF(OR(AV49="",AQ49=""),"",IF((AQ49+N(AX49))=0,"",(AV49-AQ49-N(AX49))/(AQ49+N(AX49))))</f>
         <v/>
       </c>
       <c r="BA49" s="12">
@@ -8077,7 +8077,7 @@
         <v/>
       </c>
       <c r="BE49" s="13">
-        <f>IF(OR(BA49="",AV49="",(AV49+BC49)=0),"",(BA49-AV49-BC49)/(AV49+BC49))</f>
+        <f>IF(OR(BA49="",AV49=""),"",IF((AV49+N(BC49))=0,"",(BA49-AV49-N(BC49))/(AV49+N(BC49))))</f>
         <v/>
       </c>
       <c r="BF49" s="12">
@@ -8097,7 +8097,7 @@
         <v/>
       </c>
       <c r="BJ49" s="13">
-        <f>IF(OR(BF49="",BA49="",(BA49+BH49)=0),"",(BF49-BA49-BH49)/(BA49+BH49))</f>
+        <f>IF(OR(BF49="",BA49=""),"",IF((BA49+N(BH49))=0,"",(BF49-BA49-N(BH49))/(BA49+N(BH49))))</f>
         <v/>
       </c>
     </row>
@@ -8112,7 +8112,7 @@
         <v/>
       </c>
       <c r="G50" s="16">
-        <f>IF(OR(C50="",B50="",(B50+E50)=0),"",(C50-B50-E50)/(B50+E50))</f>
+        <f>IF(OR(C50="",B50=""),"",IF((B50+N(E50))=0,"",(C50-B50-N(E50))/(B50+N(E50))))</f>
         <v/>
       </c>
       <c r="H50" s="15" t="n"/>
@@ -8123,7 +8123,7 @@
         <v/>
       </c>
       <c r="L50" s="16">
-        <f>IF(OR(H50="",C50="",(C50+J50)=0),"",(H50-C50-J50)/(C50+J50))</f>
+        <f>IF(OR(H50="",C50=""),"",IF((C50+N(J50))=0,"",(H50-C50-N(J50))/(C50+N(J50))))</f>
         <v/>
       </c>
       <c r="M50" s="15" t="n"/>
@@ -8134,7 +8134,7 @@
         <v/>
       </c>
       <c r="Q50" s="16">
-        <f>IF(OR(M50="",H50="",(H50+O50)=0),"",(M50-H50-O50)/(H50+O50))</f>
+        <f>IF(OR(M50="",H50=""),"",IF((H50+N(O50))=0,"",(M50-H50-N(O50))/(H50+N(O50))))</f>
         <v/>
       </c>
       <c r="R50" s="15" t="n"/>
@@ -8145,7 +8145,7 @@
         <v/>
       </c>
       <c r="V50" s="16">
-        <f>IF(OR(R50="",M50="",(M50+T50)=0),"",(R50-M50-T50)/(M50+T50))</f>
+        <f>IF(OR(R50="",M50=""),"",IF((M50+N(T50))=0,"",(R50-M50-N(T50))/(M50+N(T50))))</f>
         <v/>
       </c>
       <c r="W50" s="15" t="n"/>
@@ -8156,7 +8156,7 @@
         <v/>
       </c>
       <c r="AA50" s="16">
-        <f>IF(OR(W50="",R50="",(R50+Y50)=0),"",(W50-R50-Y50)/(R50+Y50))</f>
+        <f>IF(OR(W50="",R50=""),"",IF((R50+N(Y50))=0,"",(W50-R50-N(Y50))/(R50+N(Y50))))</f>
         <v/>
       </c>
       <c r="AB50" s="15" t="n"/>
@@ -8167,7 +8167,7 @@
         <v/>
       </c>
       <c r="AF50" s="16">
-        <f>IF(OR(AB50="",W50="",(W50+AD50)=0),"",(AB50-W50-AD50)/(W50+AD50))</f>
+        <f>IF(OR(AB50="",W50=""),"",IF((W50+N(AD50))=0,"",(AB50-W50-N(AD50))/(W50+N(AD50))))</f>
         <v/>
       </c>
       <c r="AG50" s="15" t="n"/>
@@ -8178,7 +8178,7 @@
         <v/>
       </c>
       <c r="AK50" s="16">
-        <f>IF(OR(AG50="",AB50="",(AB50+AI50)=0),"",(AG50-AB50-AI50)/(AB50+AI50))</f>
+        <f>IF(OR(AG50="",AB50=""),"",IF((AB50+N(AI50))=0,"",(AG50-AB50-N(AI50))/(AB50+N(AI50))))</f>
         <v/>
       </c>
       <c r="AL50" s="15" t="n"/>
@@ -8189,7 +8189,7 @@
         <v/>
       </c>
       <c r="AP50" s="16">
-        <f>IF(OR(AL50="",AG50="",(AG50+AN50)=0),"",(AL50-AG50-AN50)/(AG50+AN50))</f>
+        <f>IF(OR(AL50="",AG50=""),"",IF((AG50+N(AN50))=0,"",(AL50-AG50-N(AN50))/(AG50+N(AN50))))</f>
         <v/>
       </c>
       <c r="AQ50" s="15" t="n"/>
@@ -8200,7 +8200,7 @@
         <v/>
       </c>
       <c r="AU50" s="16">
-        <f>IF(OR(AQ50="",AL50="",(AL50+AS50)=0),"",(AQ50-AL50-AS50)/(AL50+AS50))</f>
+        <f>IF(OR(AQ50="",AL50=""),"",IF((AL50+N(AS50))=0,"",(AQ50-AL50-N(AS50))/(AL50+N(AS50))))</f>
         <v/>
       </c>
       <c r="AV50" s="15" t="n"/>
@@ -8211,7 +8211,7 @@
         <v/>
       </c>
       <c r="AZ50" s="16">
-        <f>IF(OR(AV50="",AQ50="",(AQ50+AX50)=0),"",(AV50-AQ50-AX50)/(AQ50+AX50))</f>
+        <f>IF(OR(AV50="",AQ50=""),"",IF((AQ50+N(AX50))=0,"",(AV50-AQ50-N(AX50))/(AQ50+N(AX50))))</f>
         <v/>
       </c>
       <c r="BA50" s="15" t="n"/>
@@ -8222,7 +8222,7 @@
         <v/>
       </c>
       <c r="BE50" s="16">
-        <f>IF(OR(BA50="",AV50="",(AV50+BC50)=0),"",(BA50-AV50-BC50)/(AV50+BC50))</f>
+        <f>IF(OR(BA50="",AV50=""),"",IF((AV50+N(BC50))=0,"",(BA50-AV50-N(BC50))/(AV50+N(BC50))))</f>
         <v/>
       </c>
       <c r="BF50" s="15" t="n"/>
@@ -8233,7 +8233,7 @@
         <v/>
       </c>
       <c r="BJ50" s="16">
-        <f>IF(OR(BF50="",BA50="",(BA50+BH50)=0),"",(BF50-BA50-BH50)/(BA50+BH50))</f>
+        <f>IF(OR(BF50="",BA50=""),"",IF((BA50+N(BH50))=0,"",(BF50-BA50-N(BH50))/(BA50+N(BH50))))</f>
         <v/>
       </c>
     </row>
@@ -8248,7 +8248,7 @@
         <v/>
       </c>
       <c r="G51" s="19">
-        <f>IF(OR(C51="",B51="",(B51+E51)=0),"",(C51-B51-E51)/(B51+E51))</f>
+        <f>IF(OR(C51="",B51=""),"",IF((B51+N(E51))=0,"",(C51-B51-N(E51))/(B51+N(E51))))</f>
         <v/>
       </c>
       <c r="H51" s="18" t="n"/>
@@ -8259,7 +8259,7 @@
         <v/>
       </c>
       <c r="L51" s="19">
-        <f>IF(OR(H51="",C51="",(C51+J51)=0),"",(H51-C51-J51)/(C51+J51))</f>
+        <f>IF(OR(H51="",C51=""),"",IF((C51+N(J51))=0,"",(H51-C51-N(J51))/(C51+N(J51))))</f>
         <v/>
       </c>
       <c r="M51" s="18" t="n"/>
@@ -8270,7 +8270,7 @@
         <v/>
       </c>
       <c r="Q51" s="19">
-        <f>IF(OR(M51="",H51="",(H51+O51)=0),"",(M51-H51-O51)/(H51+O51))</f>
+        <f>IF(OR(M51="",H51=""),"",IF((H51+N(O51))=0,"",(M51-H51-N(O51))/(H51+N(O51))))</f>
         <v/>
       </c>
       <c r="R51" s="18" t="n"/>
@@ -8281,7 +8281,7 @@
         <v/>
       </c>
       <c r="V51" s="19">
-        <f>IF(OR(R51="",M51="",(M51+T51)=0),"",(R51-M51-T51)/(M51+T51))</f>
+        <f>IF(OR(R51="",M51=""),"",IF((M51+N(T51))=0,"",(R51-M51-N(T51))/(M51+N(T51))))</f>
         <v/>
       </c>
       <c r="W51" s="18" t="n"/>
@@ -8292,7 +8292,7 @@
         <v/>
       </c>
       <c r="AA51" s="19">
-        <f>IF(OR(W51="",R51="",(R51+Y51)=0),"",(W51-R51-Y51)/(R51+Y51))</f>
+        <f>IF(OR(W51="",R51=""),"",IF((R51+N(Y51))=0,"",(W51-R51-N(Y51))/(R51+N(Y51))))</f>
         <v/>
       </c>
       <c r="AB51" s="18" t="n"/>
@@ -8303,7 +8303,7 @@
         <v/>
       </c>
       <c r="AF51" s="19">
-        <f>IF(OR(AB51="",W51="",(W51+AD51)=0),"",(AB51-W51-AD51)/(W51+AD51))</f>
+        <f>IF(OR(AB51="",W51=""),"",IF((W51+N(AD51))=0,"",(AB51-W51-N(AD51))/(W51+N(AD51))))</f>
         <v/>
       </c>
       <c r="AG51" s="18" t="n"/>
@@ -8314,7 +8314,7 @@
         <v/>
       </c>
       <c r="AK51" s="19">
-        <f>IF(OR(AG51="",AB51="",(AB51+AI51)=0),"",(AG51-AB51-AI51)/(AB51+AI51))</f>
+        <f>IF(OR(AG51="",AB51=""),"",IF((AB51+N(AI51))=0,"",(AG51-AB51-N(AI51))/(AB51+N(AI51))))</f>
         <v/>
       </c>
       <c r="AL51" s="18" t="n"/>
@@ -8325,7 +8325,7 @@
         <v/>
       </c>
       <c r="AP51" s="19">
-        <f>IF(OR(AL51="",AG51="",(AG51+AN51)=0),"",(AL51-AG51-AN51)/(AG51+AN51))</f>
+        <f>IF(OR(AL51="",AG51=""),"",IF((AG51+N(AN51))=0,"",(AL51-AG51-N(AN51))/(AG51+N(AN51))))</f>
         <v/>
       </c>
       <c r="AQ51" s="18" t="n"/>
@@ -8336,7 +8336,7 @@
         <v/>
       </c>
       <c r="AU51" s="19">
-        <f>IF(OR(AQ51="",AL51="",(AL51+AS51)=0),"",(AQ51-AL51-AS51)/(AL51+AS51))</f>
+        <f>IF(OR(AQ51="",AL51=""),"",IF((AL51+N(AS51))=0,"",(AQ51-AL51-N(AS51))/(AL51+N(AS51))))</f>
         <v/>
       </c>
       <c r="AV51" s="18" t="n"/>
@@ -8347,7 +8347,7 @@
         <v/>
       </c>
       <c r="AZ51" s="19">
-        <f>IF(OR(AV51="",AQ51="",(AQ51+AX51)=0),"",(AV51-AQ51-AX51)/(AQ51+AX51))</f>
+        <f>IF(OR(AV51="",AQ51=""),"",IF((AQ51+N(AX51))=0,"",(AV51-AQ51-N(AX51))/(AQ51+N(AX51))))</f>
         <v/>
       </c>
       <c r="BA51" s="18" t="n"/>
@@ -8358,7 +8358,7 @@
         <v/>
       </c>
       <c r="BE51" s="19">
-        <f>IF(OR(BA51="",AV51="",(AV51+BC51)=0),"",(BA51-AV51-BC51)/(AV51+BC51))</f>
+        <f>IF(OR(BA51="",AV51=""),"",IF((AV51+N(BC51))=0,"",(BA51-AV51-N(BC51))/(AV51+N(BC51))))</f>
         <v/>
       </c>
       <c r="BF51" s="18" t="n"/>
@@ -8369,7 +8369,7 @@
         <v/>
       </c>
       <c r="BJ51" s="19">
-        <f>IF(OR(BF51="",BA51="",(BA51+BH51)=0),"",(BF51-BA51-BH51)/(BA51+BH51))</f>
+        <f>IF(OR(BF51="",BA51=""),"",IF((BA51+N(BH51))=0,"",(BF51-BA51-N(BH51))/(BA51+N(BH51))))</f>
         <v/>
       </c>
     </row>
@@ -8384,7 +8384,7 @@
         <v/>
       </c>
       <c r="G52" s="16">
-        <f>IF(OR(C52="",B52="",(B52+E52)=0),"",(C52-B52-E52)/(B52+E52))</f>
+        <f>IF(OR(C52="",B52=""),"",IF((B52+N(E52))=0,"",(C52-B52-N(E52))/(B52+N(E52))))</f>
         <v/>
       </c>
       <c r="H52" s="15" t="n"/>
@@ -8395,7 +8395,7 @@
         <v/>
       </c>
       <c r="L52" s="16">
-        <f>IF(OR(H52="",C52="",(C52+J52)=0),"",(H52-C52-J52)/(C52+J52))</f>
+        <f>IF(OR(H52="",C52=""),"",IF((C52+N(J52))=0,"",(H52-C52-N(J52))/(C52+N(J52))))</f>
         <v/>
       </c>
       <c r="M52" s="15" t="n"/>
@@ -8406,7 +8406,7 @@
         <v/>
       </c>
       <c r="Q52" s="16">
-        <f>IF(OR(M52="",H52="",(H52+O52)=0),"",(M52-H52-O52)/(H52+O52))</f>
+        <f>IF(OR(M52="",H52=""),"",IF((H52+N(O52))=0,"",(M52-H52-N(O52))/(H52+N(O52))))</f>
         <v/>
       </c>
       <c r="R52" s="15" t="n"/>
@@ -8417,7 +8417,7 @@
         <v/>
       </c>
       <c r="V52" s="16">
-        <f>IF(OR(R52="",M52="",(M52+T52)=0),"",(R52-M52-T52)/(M52+T52))</f>
+        <f>IF(OR(R52="",M52=""),"",IF((M52+N(T52))=0,"",(R52-M52-N(T52))/(M52+N(T52))))</f>
         <v/>
       </c>
       <c r="W52" s="15" t="n"/>
@@ -8428,7 +8428,7 @@
         <v/>
       </c>
       <c r="AA52" s="16">
-        <f>IF(OR(W52="",R52="",(R52+Y52)=0),"",(W52-R52-Y52)/(R52+Y52))</f>
+        <f>IF(OR(W52="",R52=""),"",IF((R52+N(Y52))=0,"",(W52-R52-N(Y52))/(R52+N(Y52))))</f>
         <v/>
       </c>
       <c r="AB52" s="15" t="n"/>
@@ -8439,7 +8439,7 @@
         <v/>
       </c>
       <c r="AF52" s="16">
-        <f>IF(OR(AB52="",W52="",(W52+AD52)=0),"",(AB52-W52-AD52)/(W52+AD52))</f>
+        <f>IF(OR(AB52="",W52=""),"",IF((W52+N(AD52))=0,"",(AB52-W52-N(AD52))/(W52+N(AD52))))</f>
         <v/>
       </c>
       <c r="AG52" s="15" t="n"/>
@@ -8450,7 +8450,7 @@
         <v/>
       </c>
       <c r="AK52" s="16">
-        <f>IF(OR(AG52="",AB52="",(AB52+AI52)=0),"",(AG52-AB52-AI52)/(AB52+AI52))</f>
+        <f>IF(OR(AG52="",AB52=""),"",IF((AB52+N(AI52))=0,"",(AG52-AB52-N(AI52))/(AB52+N(AI52))))</f>
         <v/>
       </c>
       <c r="AL52" s="15" t="n"/>
@@ -8461,7 +8461,7 @@
         <v/>
       </c>
       <c r="AP52" s="16">
-        <f>IF(OR(AL52="",AG52="",(AG52+AN52)=0),"",(AL52-AG52-AN52)/(AG52+AN52))</f>
+        <f>IF(OR(AL52="",AG52=""),"",IF((AG52+N(AN52))=0,"",(AL52-AG52-N(AN52))/(AG52+N(AN52))))</f>
         <v/>
       </c>
       <c r="AQ52" s="15" t="n"/>
@@ -8472,7 +8472,7 @@
         <v/>
       </c>
       <c r="AU52" s="16">
-        <f>IF(OR(AQ52="",AL52="",(AL52+AS52)=0),"",(AQ52-AL52-AS52)/(AL52+AS52))</f>
+        <f>IF(OR(AQ52="",AL52=""),"",IF((AL52+N(AS52))=0,"",(AQ52-AL52-N(AS52))/(AL52+N(AS52))))</f>
         <v/>
       </c>
       <c r="AV52" s="15" t="n"/>
@@ -8483,7 +8483,7 @@
         <v/>
       </c>
       <c r="AZ52" s="16">
-        <f>IF(OR(AV52="",AQ52="",(AQ52+AX52)=0),"",(AV52-AQ52-AX52)/(AQ52+AX52))</f>
+        <f>IF(OR(AV52="",AQ52=""),"",IF((AQ52+N(AX52))=0,"",(AV52-AQ52-N(AX52))/(AQ52+N(AX52))))</f>
         <v/>
       </c>
       <c r="BA52" s="15" t="n"/>
@@ -8494,7 +8494,7 @@
         <v/>
       </c>
       <c r="BE52" s="16">
-        <f>IF(OR(BA52="",AV52="",(AV52+BC52)=0),"",(BA52-AV52-BC52)/(AV52+BC52))</f>
+        <f>IF(OR(BA52="",AV52=""),"",IF((AV52+N(BC52))=0,"",(BA52-AV52-N(BC52))/(AV52+N(BC52))))</f>
         <v/>
       </c>
       <c r="BF52" s="15" t="n"/>
@@ -8505,7 +8505,7 @@
         <v/>
       </c>
       <c r="BJ52" s="16">
-        <f>IF(OR(BF52="",BA52="",(BA52+BH52)=0),"",(BF52-BA52-BH52)/(BA52+BH52))</f>
+        <f>IF(OR(BF52="",BA52=""),"",IF((BA52+N(BH52))=0,"",(BF52-BA52-N(BH52))/(BA52+N(BH52))))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Adiciona botao de macro para inserir linhas e melhora os graficos
- Gera tambem um .xlsm com projeto VBA embutido e um botao
  "+ Adicionar linha de ativo" que insere uma linha de ativo ja
  formatada e com as formulas de rentabilidade prontas.
- Graficos: titulos de eixos, rotulos de dados nas barras, marcadores
  na linha e colunas auxiliares que convertem meses vazios em lacuna
  (NA) em vez de cair para zero.

https://claude.ai/code/session_012B6pvzwHHmCv3nAgYhFWdt
</commit_message>
<xml_diff>
--- a/acompanhamento_mensal.xlsx
+++ b/acompanhamento_mensal.xlsx
@@ -417,7 +417,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Evolução do Patrimônio</a:t>
+              <a:t>Evolução do Patrimônio (R$)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -431,7 +431,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Acompanhamento Mensal'!B56</f>
+              <f>'Acompanhamento Mensal'!BL56</f>
             </strRef>
           </tx>
           <spPr>
@@ -440,7 +440,8 @@
             </a:ln>
           </spPr>
           <marker>
-            <symbol val="none"/>
+            <symbol val="circle"/>
+            <size val="6"/>
             <spPr>
               <a:ln>
                 <a:prstDash val="solid"/>
@@ -454,16 +455,17 @@
           </cat>
           <val>
             <numRef>
-              <f>'Acompanhamento Mensal'!$B$57:$B$68</f>
+              <f>'Acompanhamento Mensal'!$BL$57:$BL$68</f>
             </numRef>
           </val>
+          <smooth val="0"/>
         </ser>
         <ser>
           <idx val="1"/>
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Acompanhamento Mensal'!C56</f>
+              <f>'Acompanhamento Mensal'!BM56</f>
             </strRef>
           </tx>
           <spPr>
@@ -472,7 +474,8 @@
             </a:ln>
           </spPr>
           <marker>
-            <symbol val="none"/>
+            <symbol val="circle"/>
+            <size val="6"/>
             <spPr>
               <a:ln>
                 <a:prstDash val="solid"/>
@@ -486,9 +489,10 @@
           </cat>
           <val>
             <numRef>
-              <f>'Acompanhamento Mensal'!$C$57:$C$68</f>
+              <f>'Acompanhamento Mensal'!$BM$57:$BM$68</f>
             </numRef>
           </val>
+          <smooth val="0"/>
         </ser>
         <axId val="10"/>
         <axId val="100"/>
@@ -498,7 +502,23 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Mês</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -509,6 +529,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
         <title>
@@ -520,7 +541,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>R$</a:t>
+                  <a:t>Patrimônio (R$)</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -535,7 +556,7 @@
     <legend>
       <legendPos val="r"/>
     </legend>
-    <plotVisOnly val="1"/>
+    <plotVisOnly val="0"/>
     <dispBlanksAs val="gap"/>
   </chart>
 </chartSpace>
@@ -569,7 +590,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Acompanhamento Mensal'!E56</f>
+              <f>'Acompanhamento Mensal'!BN56</f>
             </strRef>
           </tx>
           <spPr>
@@ -584,11 +605,15 @@
           </cat>
           <val>
             <numRef>
-              <f>'Acompanhamento Mensal'!$E$57:$E$68</f>
+              <f>'Acompanhamento Mensal'!$BN$57:$BN$68</f>
             </numRef>
           </val>
         </ser>
-        <gapWidth val="150"/>
+        <dLbls>
+          <numFmt formatCode="0.00%"/>
+          <showVal val="1"/>
+        </dLbls>
+        <gapWidth val="60"/>
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
@@ -597,7 +622,23 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Mês</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -608,15 +649,31 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Rentabilidade (%)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <numFmt formatCode="0.0%" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
-    <plotVisOnly val="1"/>
+    <plotVisOnly val="0"/>
     <dispBlanksAs val="gap"/>
   </chart>
 </chartSpace>
@@ -631,7 +688,7 @@
       <row>54</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7200000" cy="3600000"/>
+    <ext cx="6840000" cy="3420000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -653,7 +710,7 @@
       <row>75</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7200000" cy="3600000"/>
+    <ext cx="6840000" cy="3420000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -960,7 +1017,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BJ68"/>
+  <dimension ref="A1:BN68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1025,6 +1082,9 @@
     <col width="14" customWidth="1" min="60" max="60"/>
     <col width="13" customWidth="1" min="61" max="61"/>
     <col width="11" customWidth="1" min="62" max="62"/>
+    <col hidden="1" width="13" customWidth="1" min="64" max="64"/>
+    <col hidden="1" width="13" customWidth="1" min="65" max="65"/>
+    <col hidden="1" width="13" customWidth="1" min="66" max="66"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -8547,6 +8607,21 @@
           <t>Rentab. Acum. (%)</t>
         </is>
       </c>
+      <c r="BL56" t="inlineStr">
+        <is>
+          <t>Patrimônio Bruto</t>
+        </is>
+      </c>
+      <c r="BM56" t="inlineStr">
+        <is>
+          <t>Patrimônio Líquido</t>
+        </is>
+      </c>
+      <c r="BN56" t="inlineStr">
+        <is>
+          <t>Rentabilidade Mensal (%)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="28" t="inlineStr">
@@ -8574,6 +8649,18 @@
         <f>IF(E57="","",E57)</f>
         <v/>
       </c>
+      <c r="BL57">
+        <f>IF(B57="",NA(),B57)</f>
+        <v/>
+      </c>
+      <c r="BM57">
+        <f>IF(C57="",NA(),C57)</f>
+        <v/>
+      </c>
+      <c r="BN57">
+        <f>IF(E57="",NA(),E57)</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="32" t="inlineStr">
@@ -8601,6 +8688,18 @@
         <f>IF(E58="",F57,IF(F57="",E58,(1+F57)*(1+E58)-1))</f>
         <v/>
       </c>
+      <c r="BL58">
+        <f>IF(B58="",NA(),B58)</f>
+        <v/>
+      </c>
+      <c r="BM58">
+        <f>IF(C58="",NA(),C58)</f>
+        <v/>
+      </c>
+      <c r="BN58">
+        <f>IF(E58="",NA(),E58)</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="28" t="inlineStr">
@@ -8628,6 +8727,18 @@
         <f>IF(E59="",F58,IF(F58="",E59,(1+F58)*(1+E59)-1))</f>
         <v/>
       </c>
+      <c r="BL59">
+        <f>IF(B59="",NA(),B59)</f>
+        <v/>
+      </c>
+      <c r="BM59">
+        <f>IF(C59="",NA(),C59)</f>
+        <v/>
+      </c>
+      <c r="BN59">
+        <f>IF(E59="",NA(),E59)</f>
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="32" t="inlineStr">
@@ -8655,6 +8766,18 @@
         <f>IF(E60="",F59,IF(F59="",E60,(1+F59)*(1+E60)-1))</f>
         <v/>
       </c>
+      <c r="BL60">
+        <f>IF(B60="",NA(),B60)</f>
+        <v/>
+      </c>
+      <c r="BM60">
+        <f>IF(C60="",NA(),C60)</f>
+        <v/>
+      </c>
+      <c r="BN60">
+        <f>IF(E60="",NA(),E60)</f>
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="28" t="inlineStr">
@@ -8682,6 +8805,18 @@
         <f>IF(E61="",F60,IF(F60="",E61,(1+F60)*(1+E61)-1))</f>
         <v/>
       </c>
+      <c r="BL61">
+        <f>IF(B61="",NA(),B61)</f>
+        <v/>
+      </c>
+      <c r="BM61">
+        <f>IF(C61="",NA(),C61)</f>
+        <v/>
+      </c>
+      <c r="BN61">
+        <f>IF(E61="",NA(),E61)</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="32" t="inlineStr">
@@ -8709,6 +8844,18 @@
         <f>IF(E62="",F61,IF(F61="",E62,(1+F61)*(1+E62)-1))</f>
         <v/>
       </c>
+      <c r="BL62">
+        <f>IF(B62="",NA(),B62)</f>
+        <v/>
+      </c>
+      <c r="BM62">
+        <f>IF(C62="",NA(),C62)</f>
+        <v/>
+      </c>
+      <c r="BN62">
+        <f>IF(E62="",NA(),E62)</f>
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="28" t="inlineStr">
@@ -8736,6 +8883,18 @@
         <f>IF(E63="",F62,IF(F62="",E63,(1+F62)*(1+E63)-1))</f>
         <v/>
       </c>
+      <c r="BL63">
+        <f>IF(B63="",NA(),B63)</f>
+        <v/>
+      </c>
+      <c r="BM63">
+        <f>IF(C63="",NA(),C63)</f>
+        <v/>
+      </c>
+      <c r="BN63">
+        <f>IF(E63="",NA(),E63)</f>
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="32" t="inlineStr">
@@ -8763,6 +8922,18 @@
         <f>IF(E64="",F63,IF(F63="",E64,(1+F63)*(1+E64)-1))</f>
         <v/>
       </c>
+      <c r="BL64">
+        <f>IF(B64="",NA(),B64)</f>
+        <v/>
+      </c>
+      <c r="BM64">
+        <f>IF(C64="",NA(),C64)</f>
+        <v/>
+      </c>
+      <c r="BN64">
+        <f>IF(E64="",NA(),E64)</f>
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="28" t="inlineStr">
@@ -8790,6 +8961,18 @@
         <f>IF(E65="",F64,IF(F64="",E65,(1+F64)*(1+E65)-1))</f>
         <v/>
       </c>
+      <c r="BL65">
+        <f>IF(B65="",NA(),B65)</f>
+        <v/>
+      </c>
+      <c r="BM65">
+        <f>IF(C65="",NA(),C65)</f>
+        <v/>
+      </c>
+      <c r="BN65">
+        <f>IF(E65="",NA(),E65)</f>
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="32" t="inlineStr">
@@ -8817,6 +9000,18 @@
         <f>IF(E66="",F65,IF(F65="",E66,(1+F65)*(1+E66)-1))</f>
         <v/>
       </c>
+      <c r="BL66">
+        <f>IF(B66="",NA(),B66)</f>
+        <v/>
+      </c>
+      <c r="BM66">
+        <f>IF(C66="",NA(),C66)</f>
+        <v/>
+      </c>
+      <c r="BN66">
+        <f>IF(E66="",NA(),E66)</f>
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="28" t="inlineStr">
@@ -8844,6 +9039,18 @@
         <f>IF(E67="",F66,IF(F66="",E67,(1+F66)*(1+E67)-1))</f>
         <v/>
       </c>
+      <c r="BL67">
+        <f>IF(B67="",NA(),B67)</f>
+        <v/>
+      </c>
+      <c r="BM67">
+        <f>IF(C67="",NA(),C67)</f>
+        <v/>
+      </c>
+      <c r="BN67">
+        <f>IF(E67="",NA(),E67)</f>
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="32" t="inlineStr">
@@ -8869,6 +9076,18 @@
       </c>
       <c r="F68" s="35">
         <f>IF(E68="",F67,IF(F67="",E68,(1+F67)*(1+E68)-1))</f>
+        <v/>
+      </c>
+      <c r="BL68">
+        <f>IF(B68="",NA(),B68)</f>
+        <v/>
+      </c>
+      <c r="BM68">
+        <f>IF(C68="",NA(),C68)</f>
+        <v/>
+      </c>
+      <c r="BN68">
+        <f>IF(E68="",NA(),E68)</f>
         <v/>
       </c>
     </row>
@@ -9040,7 +9259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -9079,107 +9298,124 @@
     <row r="7" ht="19" customHeight="1">
       <c r="A7" s="38" t="inlineStr">
         <is>
-          <t>3. Em cada mês preencha apenas 3 colunas por ativo:</t>
+          <t>3. Precisa de mais linhas em uma classe? Selecione uma célula de uma linha de ativo dessa classe e clique no botão azul '+ Adicionar linha de ativo' (no topo da aba). Uma nova linha é inserida já formatada e com as fórmulas prontas.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1">
       <c r="A8" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">     • Valor Bruto      – valor de mercado antes de impostos.</t>
+          <t xml:space="preserve">     • O arquivo .xlsm precisa ter as macros habilitadas: ao abrir, clique em 'Habilitar conteúdo'.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1">
-      <c r="A9" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     • Valor Líquido    – valor já descontado o IR no resgate.</t>
-        </is>
-      </c>
+      <c r="A9" s="37" t="inlineStr"/>
     </row>
     <row r="10" ht="19" customHeight="1">
-      <c r="A10" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                          (em investimentos ISENTOS, repita o valor bruto)</t>
+      <c r="A10" s="38" t="inlineStr">
+        <is>
+          <t>4. Em cada mês preencha apenas 3 colunas por ativo:</t>
         </is>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1">
       <c r="A11" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">     • Movimentação     – aportes com sinal +  e  resgates com sinal −  (deixe vazio se não houve).</t>
+          <t xml:space="preserve">     • Valor Bruto      – valor de mercado antes de impostos.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1">
-      <c r="A12" s="37" t="inlineStr"/>
+      <c r="A12" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     • Valor Líquido    – valor já descontado o IR no resgate.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="19" customHeight="1">
-      <c r="A13" s="38" t="inlineStr">
-        <is>
-          <t>4. As colunas Rentabilidade (R$) e Rentabilidade (%) são calculadas automaticamente:</t>
+      <c r="A13" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                          (em investimentos ISENTOS, repita o valor bruto)</t>
         </is>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1">
       <c r="A14" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Rentab. R$ = Valor Bruto do mês − Valor Bruto do mês anterior − Movimentação.</t>
+          <t xml:space="preserve">     • Movimentação     – aportes com sinal +  e  resgates com sinal −  (deixe vazio se não houve).</t>
         </is>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1">
-      <c r="A15" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     Assim, aportes e resgates NÃO são contados como rendimento.</t>
-        </is>
-      </c>
+      <c r="A15" s="37" t="inlineStr"/>
     </row>
     <row r="16" ht="19" customHeight="1">
-      <c r="A16" s="37" t="inlineStr"/>
+      <c r="A16" s="38" t="inlineStr">
+        <is>
+          <t>5. As colunas Rentabilidade (R$) e Rentabilidade (%) são calculadas automaticamente:</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="19" customHeight="1">
-      <c r="A17" s="38" t="inlineStr">
-        <is>
-          <t>5. A coluna 'Saldo Inicial (Bruto)' é a base do 1º mês. Preencha-a com o valor antes do período acompanhado.</t>
+      <c r="A17" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     Rentab. R$ = Valor Bruto do mês − Valor Bruto do mês anterior − Movimentação.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1">
-      <c r="A18" s="37" t="inlineStr"/>
+      <c r="A18" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     Assim, aportes e resgates NÃO são contados como rendimento.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="19" customHeight="1">
-      <c r="A19" s="38" t="inlineStr">
-        <is>
-          <t>6. As linhas de classe e a linha PATRIMÔNIO TOTAL somam tudo sozinhas — não digite nada nelas.</t>
-        </is>
-      </c>
+      <c r="A19" s="37" t="inlineStr"/>
     </row>
     <row r="20" ht="19" customHeight="1">
-      <c r="A20" s="37" t="inlineStr"/>
+      <c r="A20" s="38" t="inlineStr">
+        <is>
+          <t>6. A coluna 'Saldo Inicial (Bruto)' é a base do 1º mês. Preencha-a com o valor antes do período acompanhado.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="19" customHeight="1">
-      <c r="A21" s="38" t="inlineStr">
-        <is>
-          <t>7. Use os botões [-] / [+] à esquerda das linhas para recolher ou expandir os ativos de cada classe.</t>
-        </is>
-      </c>
+      <c r="A21" s="37" t="inlineStr"/>
     </row>
     <row r="22" ht="19" customHeight="1">
-      <c r="A22" s="37" t="inlineStr"/>
+      <c r="A22" s="38" t="inlineStr">
+        <is>
+          <t>7. As linhas de classe e a linha PATRIMÔNIO TOTAL somam tudo sozinhas — não digite nada nelas.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="19" customHeight="1">
-      <c r="A23" s="38" t="inlineStr">
-        <is>
-          <t>8. O bloco RESUMO e os gráficos no fim da aba se atualizam sozinhos e podem ser usados no envio ao cliente.</t>
-        </is>
-      </c>
+      <c r="A23" s="37" t="inlineStr"/>
     </row>
     <row r="24" ht="19" customHeight="1">
-      <c r="A24" s="37" t="inlineStr"/>
+      <c r="A24" s="38" t="inlineStr">
+        <is>
+          <t>8. Use os botões [-] / [+] à esquerda das linhas para recolher ou expandir os ativos de cada classe.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="19" customHeight="1">
-      <c r="A25" s="37" t="inlineStr">
+      <c r="A25" s="37" t="inlineStr"/>
+    </row>
+    <row r="26" ht="19" customHeight="1">
+      <c r="A26" s="38" t="inlineStr">
+        <is>
+          <t>9. O bloco RESUMO e os gráficos no fim da aba se atualizam sozinhos e podem ser usados no envio ao cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="19" customHeight="1">
+      <c r="A27" s="37" t="inlineStr"/>
+    </row>
+    <row r="28" ht="19" customHeight="1">
+      <c r="A28" s="37" t="inlineStr">
         <is>
           <t>Observação: a diferença entre Valor Bruto e Valor Líquido mostra ao cliente quanto o IR impacta o resgate. Em produtos isentos (LCI, LCA, CRI, CRA, debêntures incentivadas, poupança) os dois valores são iguais.</t>
         </is>

</xml_diff>